<commit_message>
Stage 2 step 2.2: semiannual timeline, phase flags and D16
</commit_message>
<xml_diff>
--- a/model/hydro_pf_model_v1.xlsx
+++ b/model/hydro_pf_model_v1.xlsx
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="182">
   <si>
     <t>Cover</t>
   </si>
@@ -508,16 +508,119 @@
   </si>
   <si>
     <t>D8</t>
+  </si>
+  <si>
+    <t>D16</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>COD</t>
+  </si>
+  <si>
+    <t>Repayment start</t>
+  </si>
+  <si>
+    <t>Debt maturity</t>
+  </si>
+  <si>
+    <t>End of operations</t>
+  </si>
+  <si>
+    <t>Period counter</t>
+  </si>
+  <si>
+    <t>Period start date</t>
+  </si>
+  <si>
+    <t>Period end date</t>
+  </si>
+  <si>
+    <t>Hydrological year</t>
+  </si>
+  <si>
+    <t>Semester</t>
+  </si>
+  <si>
+    <t>Construction flag</t>
+  </si>
+  <si>
+    <t>Operations flag</t>
+  </si>
+  <si>
+    <t>Repayment flag</t>
+  </si>
+  <si>
+    <t>Years from base</t>
+  </si>
+  <si>
+    <t>Check construction Flag</t>
+  </si>
+  <si>
+    <t>Check operation flag</t>
+  </si>
+  <si>
+    <t>Check repayment flag</t>
+  </si>
+  <si>
+    <t>Check overlap</t>
+  </si>
+  <si>
+    <t>Status/Val</t>
+  </si>
+  <si>
+    <t>check</t>
+  </si>
+  <si>
+    <t>Check phase overlap</t>
+  </si>
+  <si>
+    <t>Must be =0</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>1. KEY DATES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.TIME </t>
+  </si>
+  <si>
+    <t>3. CHECKS</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>Financial close date</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>flag</t>
+  </si>
+  <si>
+    <t>Sum of flags</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -589,8 +692,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -605,6 +722,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -637,7 +760,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -688,6 +811,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1152,7 +1287,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T54"/>
+  <dimension ref="A1:T55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.7109375" customWidth="1"/>
@@ -1288,51 +1423,51 @@
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="28" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>178</v>
+      </c>
+      <c r="B11" s="43">
+        <v>46661</v>
+      </c>
+      <c r="C11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="B11" s="33"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="29"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="16">
-        <v>0.92</v>
-      </c>
-      <c r="C12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" t="s">
-        <v>93</v>
-      </c>
-      <c r="E12" t="s">
-        <v>96</v>
-      </c>
-      <c r="F12" t="s">
-        <v>98</v>
-      </c>
+      <c r="B12" s="33"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="29"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="3">
-        <v>65</v>
+        <v>19</v>
+      </c>
+      <c r="B13" s="16">
+        <v>0.92</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
         <v>93</v>
       </c>
-      <c r="E13" s="15" t="s">
-        <v>91</v>
+      <c r="E13" t="s">
+        <v>96</v>
       </c>
       <c r="F13" t="s">
         <v>98</v>
@@ -1340,80 +1475,80 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B14" s="3">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D14" t="s">
         <v>93</v>
       </c>
-      <c r="E14" t="s">
-        <v>92</v>
+      <c r="E14" s="15" t="s">
+        <v>91</v>
       </c>
       <c r="F14" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="B15" s="33"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>144</v>
-      </c>
-      <c r="B16" s="35">
-        <v>10</v>
-      </c>
-      <c r="C16" t="s">
-        <v>145</v>
-      </c>
-      <c r="D16" t="s">
-        <v>93</v>
-      </c>
-      <c r="E16" t="s">
-        <v>146</v>
-      </c>
-      <c r="F16" t="s">
-        <v>147</v>
-      </c>
+      <c r="B16" s="33"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="3">
-        <v>3300</v>
+        <v>144</v>
+      </c>
+      <c r="B17" s="35">
+        <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>26</v>
+        <v>145</v>
       </c>
       <c r="D17" t="s">
         <v>93</v>
       </c>
-      <c r="E17" s="15" t="s">
-        <v>113</v>
+      <c r="E17" t="s">
+        <v>146</v>
       </c>
       <c r="F17" t="s">
-        <v>101</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>103</v>
+        <v>25</v>
       </c>
       <c r="B18" s="3">
-        <v>0</v>
+        <v>3300</v>
       </c>
       <c r="C18" t="s">
         <v>26</v>
@@ -1422,7 +1557,7 @@
         <v>93</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F18" t="s">
         <v>101</v>
@@ -1430,16 +1565,16 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B19" s="3">
-        <v>2024</v>
+        <v>0</v>
       </c>
       <c r="C19" t="s">
-        <v>109</v>
+        <v>26</v>
       </c>
       <c r="D19" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>112</v>
@@ -1450,56 +1585,56 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B20" s="3">
-        <v>0</v>
+        <v>2024</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="D20" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F20" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
+      <c r="A21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" s="3">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="21"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>104</v>
-      </c>
-      <c r="B22" s="16">
-        <v>0.15</v>
-      </c>
-      <c r="C22" t="s">
-        <v>20</v>
-      </c>
-      <c r="D22" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" t="s">
-        <v>92</v>
-      </c>
-      <c r="F22" t="s">
-        <v>101</v>
-      </c>
+      <c r="B22" s="21"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B23" s="16">
-        <v>0.35</v>
+        <v>0.15</v>
       </c>
       <c r="C23" t="s">
         <v>20</v>
@@ -1516,7 +1651,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B24" s="16">
         <v>0.35</v>
@@ -1536,10 +1671,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B25" s="16">
-        <v>0.15</v>
+        <v>0.35</v>
       </c>
       <c r="C25" t="s">
         <v>20</v>
@@ -1556,58 +1691,58 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>107</v>
+      </c>
+      <c r="B26" s="16">
+        <v>0.15</v>
+      </c>
+      <c r="C26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" t="s">
+        <v>93</v>
+      </c>
+      <c r="E26" t="s">
+        <v>92</v>
+      </c>
+      <c r="F26" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>114</v>
       </c>
-      <c r="B26" s="22">
-        <f>SUM(B22:B25)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
+      <c r="B27" s="22">
+        <f>SUM(B23:B26)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>95</v>
-      </c>
-      <c r="B28" s="16">
-        <v>0.03</v>
-      </c>
-      <c r="C28" t="s">
-        <v>24</v>
-      </c>
-      <c r="D28" t="s">
-        <v>93</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="F28" t="s">
-        <v>98</v>
-      </c>
+      <c r="B28" s="33"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="3">
-        <v>0</v>
+        <v>95</v>
+      </c>
+      <c r="B29" s="16">
+        <v>0.03</v>
       </c>
       <c r="C29" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D29" t="s">
         <v>93</v>
       </c>
-      <c r="E29" t="s">
-        <v>92</v>
+      <c r="E29" s="15" t="s">
+        <v>94</v>
       </c>
       <c r="F29" t="s">
         <v>98</v>
@@ -1615,95 +1750,95 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" s="17">
-        <v>0.02</v>
+        <v>32</v>
+      </c>
+      <c r="B30" s="3">
+        <v>0</v>
       </c>
       <c r="C30" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D30" t="s">
         <v>93</v>
       </c>
-      <c r="E30" s="15" t="s">
-        <v>97</v>
+      <c r="E30" t="s">
+        <v>92</v>
       </c>
       <c r="F30" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="28" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="17">
+        <v>0.02</v>
+      </c>
+      <c r="C31" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" t="s">
+        <v>93</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="F31" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="28" t="s">
         <v>142</v>
       </c>
-      <c r="B31" s="33"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="29"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32" s="17">
-        <v>0.35</v>
-      </c>
-      <c r="C32" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" t="s">
-        <v>93</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="F32" t="s">
-        <v>127</v>
-      </c>
+      <c r="B32" s="33"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="29"/>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="B33" s="17">
+        <v>0.35</v>
+      </c>
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="F33" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>128</v>
-      </c>
-      <c r="B34" s="16">
-        <v>0.5</v>
-      </c>
-      <c r="C34" t="s">
-        <v>20</v>
-      </c>
-      <c r="D34" t="s">
-        <v>93</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="F34" t="s">
-        <v>127</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B34" s="3"/>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>129</v>
-      </c>
-      <c r="B35" s="3">
-        <v>50</v>
+        <v>128</v>
+      </c>
+      <c r="B35" s="16">
+        <v>0.5</v>
       </c>
       <c r="C35" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D35" t="s">
         <v>93</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="F35" t="s">
         <v>127</v>
@@ -1711,10 +1846,10 @@
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B36" s="3">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C36" t="s">
         <v>31</v>
@@ -1731,10 +1866,10 @@
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B37" s="3">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C37" t="s">
         <v>31</v>
@@ -1749,51 +1884,51 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="28" t="s">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>131</v>
+      </c>
+      <c r="B38" s="3">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>31</v>
+      </c>
+      <c r="D38" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="F38" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="B38" s="33"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="29"/>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>36</v>
-      </c>
-      <c r="B39" s="3">
-        <v>12</v>
-      </c>
-      <c r="C39" t="s">
-        <v>31</v>
-      </c>
-      <c r="D39" t="s">
-        <v>93</v>
-      </c>
-      <c r="E39" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="F39" t="s">
-        <v>126</v>
-      </c>
+      <c r="B39" s="33"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="29"/>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>37</v>
-      </c>
-      <c r="B40" s="17">
-        <v>0.09</v>
+        <v>36</v>
+      </c>
+      <c r="B40" s="3">
+        <v>12</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="D40" t="s">
         <v>93</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F40" t="s">
         <v>126</v>
@@ -1801,20 +1936,19 @@
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>115</v>
-      </c>
-      <c r="B41" s="24">
-        <f>B40/2</f>
-        <v>4.4999999999999998E-2</v>
+        <v>37</v>
+      </c>
+      <c r="B41" s="17">
+        <v>0.09</v>
       </c>
       <c r="C41" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="D41" t="s">
-        <v>135</v>
-      </c>
-      <c r="E41" t="s">
-        <v>92</v>
+        <v>93</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>117</v>
       </c>
       <c r="F41" t="s">
         <v>126</v>
@@ -1822,16 +1956,17 @@
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>124</v>
-      </c>
-      <c r="B42" s="3">
-        <v>0</v>
+        <v>115</v>
+      </c>
+      <c r="B42" s="24">
+        <f>B41/2</f>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="C42" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>135</v>
       </c>
       <c r="E42" t="s">
         <v>92</v>
@@ -1842,19 +1977,19 @@
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>38</v>
+        <v>124</v>
       </c>
       <c r="B43" s="3">
-        <v>1.35</v>
+        <v>0</v>
       </c>
       <c r="C43" t="s">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="D43" t="s">
         <v>93</v>
       </c>
-      <c r="E43" s="15" t="s">
-        <v>119</v>
+      <c r="E43" t="s">
+        <v>92</v>
       </c>
       <c r="F43" t="s">
         <v>126</v>
@@ -1862,10 +1997,10 @@
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B44" s="3">
-        <v>1.2</v>
+        <v>1.35</v>
       </c>
       <c r="C44" t="s">
         <v>39</v>
@@ -1874,7 +2009,7 @@
         <v>93</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F44" t="s">
         <v>126</v>
@@ -1882,10 +2017,10 @@
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B45" s="3">
-        <v>1.1000000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="C45" t="s">
         <v>39</v>
@@ -1894,7 +2029,7 @@
         <v>93</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F45" t="s">
         <v>126</v>
@@ -1902,61 +2037,61 @@
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>42</v>
-      </c>
-      <c r="B46" s="17">
-        <v>0.7</v>
+        <v>41</v>
+      </c>
+      <c r="B46" s="3">
+        <v>1.1000000000000001</v>
       </c>
       <c r="C46" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D46" t="s">
         <v>93</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F46" t="s">
         <v>126</v>
       </c>
-      <c r="M46" s="12"/>
-      <c r="T46" s="12"/>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>43</v>
-      </c>
-      <c r="B47" s="3">
-        <v>6</v>
+        <v>42</v>
+      </c>
+      <c r="B47" s="17">
+        <v>0.7</v>
       </c>
       <c r="C47" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D47" t="s">
         <v>93</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F47" t="s">
         <v>126</v>
       </c>
+      <c r="M47" s="12"/>
+      <c r="T47" s="12"/>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>44</v>
-      </c>
-      <c r="B48" s="17">
-        <v>1.4999999999999999E-2</v>
+        <v>43</v>
+      </c>
+      <c r="B48" s="3">
+        <v>6</v>
       </c>
       <c r="C48" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D48" t="s">
         <v>93</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F48" t="s">
         <v>126</v>
@@ -1964,10 +2099,10 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B49" s="17">
-        <v>5.0000000000000001E-3</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="C49" t="s">
         <v>20</v>
@@ -1982,37 +2117,57 @@
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E51" s="11"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E54" s="12"/>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>45</v>
+      </c>
+      <c r="B50" s="17">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D50" t="s">
+        <v>93</v>
+      </c>
+      <c r="E50" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="F50" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E52" s="11"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E55" s="12"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E13" r:id="rId1"/>
-    <hyperlink ref="E28" r:id="rId2"/>
-    <hyperlink ref="E30" r:id="rId3"/>
-    <hyperlink ref="E17" r:id="rId4" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
-    <hyperlink ref="E18" r:id="rId5" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
-    <hyperlink ref="E19" r:id="rId6" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
+    <hyperlink ref="E14" r:id="rId1"/>
+    <hyperlink ref="E29" r:id="rId2"/>
+    <hyperlink ref="E31" r:id="rId3"/>
+    <hyperlink ref="E18" r:id="rId4" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
+    <hyperlink ref="E19" r:id="rId5" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
+    <hyperlink ref="E20" r:id="rId6" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
     <hyperlink ref="E9" r:id="rId7" display="IRENA: RENEWABLE ENERGY TECHNOLOGIES: COST ANALYSIS SERIES"/>
-    <hyperlink ref="E20" r:id="rId8" display="IRENA: RENEWABLE ENERGY TECHNOLOGIES: COST ANALYSIS SERIES"/>
-    <hyperlink ref="E39" r:id="rId9"/>
-    <hyperlink ref="E40" r:id="rId10"/>
-    <hyperlink ref="E43" r:id="rId11"/>
-    <hyperlink ref="E44" r:id="rId12"/>
-    <hyperlink ref="E45" r:id="rId13"/>
-    <hyperlink ref="E46" r:id="rId14"/>
-    <hyperlink ref="E47" r:id="rId15"/>
-    <hyperlink ref="E48" r:id="rId16"/>
-    <hyperlink ref="E49" r:id="rId17"/>
+    <hyperlink ref="E21" r:id="rId8" display="IRENA: RENEWABLE ENERGY TECHNOLOGIES: COST ANALYSIS SERIES"/>
+    <hyperlink ref="E40" r:id="rId9"/>
+    <hyperlink ref="E41" r:id="rId10"/>
+    <hyperlink ref="E44" r:id="rId11"/>
+    <hyperlink ref="E45" r:id="rId12"/>
+    <hyperlink ref="E46" r:id="rId13"/>
+    <hyperlink ref="E47" r:id="rId14"/>
+    <hyperlink ref="E48" r:id="rId15"/>
+    <hyperlink ref="E49" r:id="rId16"/>
+    <hyperlink ref="E50" r:id="rId17"/>
     <hyperlink ref="E10" r:id="rId18" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
-    <hyperlink ref="E32" r:id="rId19"/>
-    <hyperlink ref="E34" r:id="rId20" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
-    <hyperlink ref="E35" r:id="rId21"/>
-    <hyperlink ref="E36" r:id="rId22"/>
-    <hyperlink ref="E37" r:id="rId23"/>
+    <hyperlink ref="E33" r:id="rId19"/>
+    <hyperlink ref="E35" r:id="rId20" display="RENEWABLE POWER GENERATION COSTS IN 2024"/>
+    <hyperlink ref="E36" r:id="rId21"/>
+    <hyperlink ref="E37" r:id="rId22"/>
+    <hyperlink ref="E38" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId24"/>
@@ -6727,24 +6882,3265 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:CA31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="5" width="21.28515625" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.140625" customWidth="1"/>
+    <col min="13" max="13" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="10.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="76" max="79" width="9.85546875" style="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:75" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>49</v>
       </c>
     </row>
+    <row r="5" spans="1:75" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="42" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+    </row>
+    <row r="6" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="7" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="6">
+        <f>Inputs!B11</f>
+        <v>46661</v>
+      </c>
+    </row>
+    <row r="8" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" t="s">
+        <v>151</v>
+      </c>
+      <c r="C8" s="6">
+        <f>EDATE(C7, Inputs!B9)</f>
+        <v>47392</v>
+      </c>
+    </row>
+    <row r="9" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="6">
+        <f>EDATE(C8, Inputs!B43*6)</f>
+        <v>47392</v>
+      </c>
+    </row>
+    <row r="10" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" t="s">
+        <v>151</v>
+      </c>
+      <c r="C10" s="6">
+        <f>EDATE(C8,Inputs!B40*12)</f>
+        <v>51775</v>
+      </c>
+    </row>
+    <row r="11" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C11" s="6">
+        <f>EDATE(C8,Inputs!B10*12)</f>
+        <v>58349</v>
+      </c>
+    </row>
+    <row r="14" spans="1:75" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="42" t="s">
+        <v>175</v>
+      </c>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="38"/>
+      <c r="K14" s="38"/>
+      <c r="L14" s="38"/>
+      <c r="M14" s="38"/>
+      <c r="N14" s="38"/>
+      <c r="O14" s="38"/>
+      <c r="P14" s="38"/>
+      <c r="Q14" s="38"/>
+      <c r="R14" s="38"/>
+      <c r="S14" s="38"/>
+      <c r="T14" s="38"/>
+      <c r="U14" s="38"/>
+      <c r="V14" s="38"/>
+      <c r="W14" s="38"/>
+      <c r="X14" s="38"/>
+      <c r="Y14" s="38"/>
+      <c r="Z14" s="38"/>
+      <c r="AA14" s="38"/>
+      <c r="AB14" s="38"/>
+      <c r="AC14" s="38"/>
+      <c r="AD14" s="38"/>
+      <c r="AE14" s="38"/>
+      <c r="AF14" s="38"/>
+      <c r="AG14" s="38"/>
+      <c r="AH14" s="38"/>
+      <c r="AI14" s="38"/>
+      <c r="AJ14" s="38"/>
+      <c r="AK14" s="38"/>
+      <c r="AL14" s="38"/>
+      <c r="AM14" s="38"/>
+      <c r="AN14" s="38"/>
+      <c r="AO14" s="38"/>
+      <c r="AP14" s="38"/>
+      <c r="AQ14" s="38"/>
+      <c r="AR14" s="38"/>
+      <c r="AS14" s="38"/>
+      <c r="AT14" s="38"/>
+      <c r="AU14" s="38"/>
+      <c r="AV14" s="38"/>
+      <c r="AW14" s="38"/>
+      <c r="AX14" s="38"/>
+      <c r="AY14" s="38"/>
+      <c r="AZ14" s="38"/>
+      <c r="BA14" s="38"/>
+      <c r="BB14" s="38"/>
+      <c r="BC14" s="38"/>
+      <c r="BD14" s="38"/>
+      <c r="BE14" s="38"/>
+      <c r="BF14" s="38"/>
+      <c r="BG14" s="38"/>
+      <c r="BH14" s="38"/>
+      <c r="BI14" s="38"/>
+      <c r="BJ14" s="38"/>
+      <c r="BK14" s="38"/>
+      <c r="BL14" s="38"/>
+      <c r="BM14" s="38"/>
+      <c r="BN14" s="38"/>
+      <c r="BO14" s="38"/>
+      <c r="BP14" s="38"/>
+      <c r="BQ14" s="38"/>
+      <c r="BR14" s="38"/>
+      <c r="BS14" s="38"/>
+      <c r="BT14" s="38"/>
+      <c r="BU14" s="38"/>
+      <c r="BV14" s="38"/>
+      <c r="BW14" s="38"/>
+    </row>
+    <row r="15" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" t="s">
+        <v>179</v>
+      </c>
+      <c r="C15" t="s">
+        <v>181</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <f>D15+1</f>
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <f>E15+1</f>
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <f t="shared" ref="G15:BR15" si="0">F15+1</f>
+        <v>4</v>
+      </c>
+      <c r="H15" s="21">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I15" s="21">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="J15" s="21">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="K15" s="21">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="L15" s="21">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="M15" s="21">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="N15" s="21">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="O15" s="21">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="P15" s="21">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="Q15" s="21">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="R15" s="21">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="S15" s="21">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="T15" s="21">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="U15" s="21">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="V15" s="21">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="W15" s="21">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="X15" s="21">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="Y15" s="21">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="Z15" s="21">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="AA15" s="21">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="AB15" s="21">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="AC15" s="21">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="AD15" s="21">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="AE15" s="21">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="AF15" s="21">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="AG15" s="21">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="AH15" s="21">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="AI15" s="21">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="AJ15" s="21">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="AK15" s="21">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="AL15" s="21">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="AM15" s="21">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="AN15" s="21">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="AO15" s="21">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="AP15" s="21">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="AQ15" s="21">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="AR15" s="21">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="AS15" s="21">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="AT15" s="21">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="AU15" s="21">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="AV15" s="21">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="AW15" s="21">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="AX15" s="21">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="AY15" s="21">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="AZ15" s="21">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="BA15" s="21">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="BB15" s="21">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="BC15" s="21">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="BD15" s="21">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="BE15" s="21">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="BF15" s="21">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="BG15" s="21">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+      <c r="BH15" s="21">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+      <c r="BI15" s="21">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+      <c r="BJ15" s="21">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+      <c r="BK15" s="21">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="BL15" s="21">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+      <c r="BM15" s="21">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+      <c r="BN15" s="21">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+      <c r="BO15" s="21">
+        <f>BN15+1</f>
+        <v>64</v>
+      </c>
+      <c r="BP15" s="21">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+      <c r="BQ15" s="21">
+        <f t="shared" si="0"/>
+        <v>66</v>
+      </c>
+      <c r="BR15" s="21">
+        <f t="shared" si="0"/>
+        <v>67</v>
+      </c>
+      <c r="BS15" s="21">
+        <f t="shared" ref="BS15:BU15" si="1">BR15+1</f>
+        <v>68</v>
+      </c>
+      <c r="BT15" s="21">
+        <f t="shared" si="1"/>
+        <v>69</v>
+      </c>
+      <c r="BU15" s="21">
+        <f t="shared" si="1"/>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:75" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16" t="s">
+        <v>151</v>
+      </c>
+      <c r="C16" t="s">
+        <v>135</v>
+      </c>
+      <c r="D16" s="6">
+        <f>C7</f>
+        <v>46661</v>
+      </c>
+      <c r="E16" s="6">
+        <f>D17+1</f>
+        <v>46844</v>
+      </c>
+      <c r="F16" s="6">
+        <f t="shared" ref="F16:BQ16" si="2">E17+1</f>
+        <v>47027</v>
+      </c>
+      <c r="G16" s="6">
+        <f t="shared" si="2"/>
+        <v>47209</v>
+      </c>
+      <c r="H16" s="36">
+        <f t="shared" si="2"/>
+        <v>47392</v>
+      </c>
+      <c r="I16" s="36">
+        <f t="shared" si="2"/>
+        <v>47574</v>
+      </c>
+      <c r="J16" s="36">
+        <f t="shared" si="2"/>
+        <v>47757</v>
+      </c>
+      <c r="K16" s="36">
+        <f t="shared" si="2"/>
+        <v>47939</v>
+      </c>
+      <c r="L16" s="36">
+        <f t="shared" si="2"/>
+        <v>48122</v>
+      </c>
+      <c r="M16" s="36">
+        <f t="shared" si="2"/>
+        <v>48305</v>
+      </c>
+      <c r="N16" s="36">
+        <f t="shared" si="2"/>
+        <v>48488</v>
+      </c>
+      <c r="O16" s="36">
+        <f t="shared" si="2"/>
+        <v>48670</v>
+      </c>
+      <c r="P16" s="36">
+        <f t="shared" si="2"/>
+        <v>48853</v>
+      </c>
+      <c r="Q16" s="36">
+        <f t="shared" si="2"/>
+        <v>49035</v>
+      </c>
+      <c r="R16" s="36">
+        <f t="shared" si="2"/>
+        <v>49218</v>
+      </c>
+      <c r="S16" s="36">
+        <f t="shared" si="2"/>
+        <v>49400</v>
+      </c>
+      <c r="T16" s="36">
+        <f t="shared" si="2"/>
+        <v>49583</v>
+      </c>
+      <c r="U16" s="36">
+        <f t="shared" si="2"/>
+        <v>49766</v>
+      </c>
+      <c r="V16" s="36">
+        <f t="shared" si="2"/>
+        <v>49949</v>
+      </c>
+      <c r="W16" s="36">
+        <f t="shared" si="2"/>
+        <v>50131</v>
+      </c>
+      <c r="X16" s="36">
+        <f t="shared" si="2"/>
+        <v>50314</v>
+      </c>
+      <c r="Y16" s="36">
+        <f t="shared" si="2"/>
+        <v>50496</v>
+      </c>
+      <c r="Z16" s="36">
+        <f t="shared" si="2"/>
+        <v>50679</v>
+      </c>
+      <c r="AA16" s="36">
+        <f t="shared" si="2"/>
+        <v>50861</v>
+      </c>
+      <c r="AB16" s="36">
+        <f t="shared" si="2"/>
+        <v>51044</v>
+      </c>
+      <c r="AC16" s="36">
+        <f t="shared" si="2"/>
+        <v>51227</v>
+      </c>
+      <c r="AD16" s="36">
+        <f t="shared" si="2"/>
+        <v>51410</v>
+      </c>
+      <c r="AE16" s="36">
+        <f t="shared" si="2"/>
+        <v>51592</v>
+      </c>
+      <c r="AF16" s="36">
+        <f t="shared" si="2"/>
+        <v>51775</v>
+      </c>
+      <c r="AG16" s="36">
+        <f t="shared" si="2"/>
+        <v>51957</v>
+      </c>
+      <c r="AH16" s="36">
+        <f t="shared" si="2"/>
+        <v>52140</v>
+      </c>
+      <c r="AI16" s="36">
+        <f t="shared" si="2"/>
+        <v>52322</v>
+      </c>
+      <c r="AJ16" s="36">
+        <f t="shared" si="2"/>
+        <v>52505</v>
+      </c>
+      <c r="AK16" s="36">
+        <f t="shared" si="2"/>
+        <v>52688</v>
+      </c>
+      <c r="AL16" s="36">
+        <f t="shared" si="2"/>
+        <v>52871</v>
+      </c>
+      <c r="AM16" s="36">
+        <f t="shared" si="2"/>
+        <v>53053</v>
+      </c>
+      <c r="AN16" s="36">
+        <f t="shared" si="2"/>
+        <v>53236</v>
+      </c>
+      <c r="AO16" s="36">
+        <f t="shared" si="2"/>
+        <v>53418</v>
+      </c>
+      <c r="AP16" s="36">
+        <f t="shared" si="2"/>
+        <v>53601</v>
+      </c>
+      <c r="AQ16" s="36">
+        <f t="shared" si="2"/>
+        <v>53783</v>
+      </c>
+      <c r="AR16" s="36">
+        <f t="shared" si="2"/>
+        <v>53966</v>
+      </c>
+      <c r="AS16" s="36">
+        <f t="shared" si="2"/>
+        <v>54149</v>
+      </c>
+      <c r="AT16" s="36">
+        <f t="shared" si="2"/>
+        <v>54332</v>
+      </c>
+      <c r="AU16" s="36">
+        <f t="shared" si="2"/>
+        <v>54514</v>
+      </c>
+      <c r="AV16" s="36">
+        <f t="shared" si="2"/>
+        <v>54697</v>
+      </c>
+      <c r="AW16" s="36">
+        <f t="shared" si="2"/>
+        <v>54879</v>
+      </c>
+      <c r="AX16" s="36">
+        <f t="shared" si="2"/>
+        <v>55062</v>
+      </c>
+      <c r="AY16" s="36">
+        <f t="shared" si="2"/>
+        <v>55244</v>
+      </c>
+      <c r="AZ16" s="36">
+        <f t="shared" si="2"/>
+        <v>55427</v>
+      </c>
+      <c r="BA16" s="36">
+        <f t="shared" si="2"/>
+        <v>55610</v>
+      </c>
+      <c r="BB16" s="36">
+        <f t="shared" si="2"/>
+        <v>55793</v>
+      </c>
+      <c r="BC16" s="36">
+        <f t="shared" si="2"/>
+        <v>55975</v>
+      </c>
+      <c r="BD16" s="36">
+        <f t="shared" si="2"/>
+        <v>56158</v>
+      </c>
+      <c r="BE16" s="36">
+        <f t="shared" si="2"/>
+        <v>56340</v>
+      </c>
+      <c r="BF16" s="36">
+        <f t="shared" si="2"/>
+        <v>56523</v>
+      </c>
+      <c r="BG16" s="36">
+        <f t="shared" si="2"/>
+        <v>56705</v>
+      </c>
+      <c r="BH16" s="36">
+        <f t="shared" si="2"/>
+        <v>56888</v>
+      </c>
+      <c r="BI16" s="36">
+        <f t="shared" si="2"/>
+        <v>57071</v>
+      </c>
+      <c r="BJ16" s="36">
+        <f t="shared" si="2"/>
+        <v>57254</v>
+      </c>
+      <c r="BK16" s="36">
+        <f t="shared" si="2"/>
+        <v>57436</v>
+      </c>
+      <c r="BL16" s="36">
+        <f t="shared" si="2"/>
+        <v>57619</v>
+      </c>
+      <c r="BM16" s="36">
+        <f t="shared" si="2"/>
+        <v>57801</v>
+      </c>
+      <c r="BN16" s="36">
+        <f t="shared" si="2"/>
+        <v>57984</v>
+      </c>
+      <c r="BO16" s="36">
+        <f t="shared" si="2"/>
+        <v>58166</v>
+      </c>
+      <c r="BP16" s="36">
+        <f t="shared" si="2"/>
+        <v>58349</v>
+      </c>
+      <c r="BQ16" s="36">
+        <f t="shared" si="2"/>
+        <v>58532</v>
+      </c>
+      <c r="BR16" s="36">
+        <f t="shared" ref="BR16:BU16" si="3">BQ17+1</f>
+        <v>58715</v>
+      </c>
+      <c r="BS16" s="36">
+        <f t="shared" si="3"/>
+        <v>58897</v>
+      </c>
+      <c r="BT16" s="36">
+        <f t="shared" si="3"/>
+        <v>59080</v>
+      </c>
+      <c r="BU16" s="36">
+        <f t="shared" si="3"/>
+        <v>59262</v>
+      </c>
+    </row>
+    <row r="17" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17" t="s">
+        <v>151</v>
+      </c>
+      <c r="C17" t="s">
+        <v>135</v>
+      </c>
+      <c r="D17" s="6">
+        <f>EOMONTH(D16,5)</f>
+        <v>46843</v>
+      </c>
+      <c r="E17" s="6">
+        <f t="shared" ref="E17:BP17" si="4">EOMONTH(E16,5)</f>
+        <v>47026</v>
+      </c>
+      <c r="F17" s="6">
+        <f t="shared" si="4"/>
+        <v>47208</v>
+      </c>
+      <c r="G17" s="6">
+        <f t="shared" si="4"/>
+        <v>47391</v>
+      </c>
+      <c r="H17" s="6">
+        <f t="shared" si="4"/>
+        <v>47573</v>
+      </c>
+      <c r="I17" s="6">
+        <f t="shared" si="4"/>
+        <v>47756</v>
+      </c>
+      <c r="J17" s="6">
+        <f t="shared" si="4"/>
+        <v>47938</v>
+      </c>
+      <c r="K17" s="6">
+        <f t="shared" si="4"/>
+        <v>48121</v>
+      </c>
+      <c r="L17" s="6">
+        <f t="shared" si="4"/>
+        <v>48304</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" si="4"/>
+        <v>48487</v>
+      </c>
+      <c r="N17" s="6">
+        <f t="shared" si="4"/>
+        <v>48669</v>
+      </c>
+      <c r="O17" s="6">
+        <f t="shared" si="4"/>
+        <v>48852</v>
+      </c>
+      <c r="P17" s="6">
+        <f t="shared" si="4"/>
+        <v>49034</v>
+      </c>
+      <c r="Q17" s="6">
+        <f t="shared" si="4"/>
+        <v>49217</v>
+      </c>
+      <c r="R17" s="6">
+        <f t="shared" si="4"/>
+        <v>49399</v>
+      </c>
+      <c r="S17" s="6">
+        <f t="shared" si="4"/>
+        <v>49582</v>
+      </c>
+      <c r="T17" s="6">
+        <f t="shared" si="4"/>
+        <v>49765</v>
+      </c>
+      <c r="U17" s="6">
+        <f t="shared" si="4"/>
+        <v>49948</v>
+      </c>
+      <c r="V17" s="6">
+        <f t="shared" si="4"/>
+        <v>50130</v>
+      </c>
+      <c r="W17" s="6">
+        <f t="shared" si="4"/>
+        <v>50313</v>
+      </c>
+      <c r="X17" s="6">
+        <f t="shared" si="4"/>
+        <v>50495</v>
+      </c>
+      <c r="Y17" s="6">
+        <f t="shared" si="4"/>
+        <v>50678</v>
+      </c>
+      <c r="Z17" s="6">
+        <f t="shared" si="4"/>
+        <v>50860</v>
+      </c>
+      <c r="AA17" s="6">
+        <f t="shared" si="4"/>
+        <v>51043</v>
+      </c>
+      <c r="AB17" s="6">
+        <f t="shared" si="4"/>
+        <v>51226</v>
+      </c>
+      <c r="AC17" s="6">
+        <f t="shared" si="4"/>
+        <v>51409</v>
+      </c>
+      <c r="AD17" s="6">
+        <f t="shared" si="4"/>
+        <v>51591</v>
+      </c>
+      <c r="AE17" s="6">
+        <f t="shared" si="4"/>
+        <v>51774</v>
+      </c>
+      <c r="AF17" s="6">
+        <f t="shared" si="4"/>
+        <v>51956</v>
+      </c>
+      <c r="AG17" s="6">
+        <f t="shared" si="4"/>
+        <v>52139</v>
+      </c>
+      <c r="AH17" s="6">
+        <f t="shared" si="4"/>
+        <v>52321</v>
+      </c>
+      <c r="AI17" s="6">
+        <f t="shared" si="4"/>
+        <v>52504</v>
+      </c>
+      <c r="AJ17" s="6">
+        <f t="shared" si="4"/>
+        <v>52687</v>
+      </c>
+      <c r="AK17" s="6">
+        <f t="shared" si="4"/>
+        <v>52870</v>
+      </c>
+      <c r="AL17" s="6">
+        <f t="shared" si="4"/>
+        <v>53052</v>
+      </c>
+      <c r="AM17" s="6">
+        <f t="shared" si="4"/>
+        <v>53235</v>
+      </c>
+      <c r="AN17" s="6">
+        <f t="shared" si="4"/>
+        <v>53417</v>
+      </c>
+      <c r="AO17" s="6">
+        <f t="shared" si="4"/>
+        <v>53600</v>
+      </c>
+      <c r="AP17" s="6">
+        <f t="shared" si="4"/>
+        <v>53782</v>
+      </c>
+      <c r="AQ17" s="6">
+        <f t="shared" si="4"/>
+        <v>53965</v>
+      </c>
+      <c r="AR17" s="6">
+        <f t="shared" si="4"/>
+        <v>54148</v>
+      </c>
+      <c r="AS17" s="6">
+        <f t="shared" si="4"/>
+        <v>54331</v>
+      </c>
+      <c r="AT17" s="6">
+        <f t="shared" si="4"/>
+        <v>54513</v>
+      </c>
+      <c r="AU17" s="6">
+        <f t="shared" si="4"/>
+        <v>54696</v>
+      </c>
+      <c r="AV17" s="6">
+        <f t="shared" si="4"/>
+        <v>54878</v>
+      </c>
+      <c r="AW17" s="6">
+        <f t="shared" si="4"/>
+        <v>55061</v>
+      </c>
+      <c r="AX17" s="6">
+        <f t="shared" si="4"/>
+        <v>55243</v>
+      </c>
+      <c r="AY17" s="6">
+        <f t="shared" si="4"/>
+        <v>55426</v>
+      </c>
+      <c r="AZ17" s="6">
+        <f t="shared" si="4"/>
+        <v>55609</v>
+      </c>
+      <c r="BA17" s="6">
+        <f t="shared" si="4"/>
+        <v>55792</v>
+      </c>
+      <c r="BB17" s="6">
+        <f t="shared" si="4"/>
+        <v>55974</v>
+      </c>
+      <c r="BC17" s="6">
+        <f t="shared" si="4"/>
+        <v>56157</v>
+      </c>
+      <c r="BD17" s="6">
+        <f t="shared" si="4"/>
+        <v>56339</v>
+      </c>
+      <c r="BE17" s="6">
+        <f t="shared" si="4"/>
+        <v>56522</v>
+      </c>
+      <c r="BF17" s="6">
+        <f t="shared" si="4"/>
+        <v>56704</v>
+      </c>
+      <c r="BG17" s="6">
+        <f t="shared" si="4"/>
+        <v>56887</v>
+      </c>
+      <c r="BH17" s="6">
+        <f t="shared" si="4"/>
+        <v>57070</v>
+      </c>
+      <c r="BI17" s="6">
+        <f t="shared" si="4"/>
+        <v>57253</v>
+      </c>
+      <c r="BJ17" s="6">
+        <f t="shared" si="4"/>
+        <v>57435</v>
+      </c>
+      <c r="BK17" s="6">
+        <f t="shared" si="4"/>
+        <v>57618</v>
+      </c>
+      <c r="BL17" s="6">
+        <f t="shared" si="4"/>
+        <v>57800</v>
+      </c>
+      <c r="BM17" s="6">
+        <f t="shared" si="4"/>
+        <v>57983</v>
+      </c>
+      <c r="BN17" s="6">
+        <f t="shared" si="4"/>
+        <v>58165</v>
+      </c>
+      <c r="BO17" s="6">
+        <f t="shared" si="4"/>
+        <v>58348</v>
+      </c>
+      <c r="BP17" s="6">
+        <f t="shared" si="4"/>
+        <v>58531</v>
+      </c>
+      <c r="BQ17" s="6">
+        <f t="shared" ref="BQ17:BU17" si="5">EOMONTH(BQ16,5)</f>
+        <v>58714</v>
+      </c>
+      <c r="BR17" s="6">
+        <f t="shared" si="5"/>
+        <v>58896</v>
+      </c>
+      <c r="BS17" s="6">
+        <f t="shared" si="5"/>
+        <v>59079</v>
+      </c>
+      <c r="BT17" s="6">
+        <f t="shared" si="5"/>
+        <v>59261</v>
+      </c>
+      <c r="BU17" s="6">
+        <f t="shared" si="5"/>
+        <v>59444</v>
+      </c>
+    </row>
+    <row r="18" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" t="s">
+        <v>135</v>
+      </c>
+      <c r="D18">
+        <f>YEAR(D17)</f>
+        <v>2028</v>
+      </c>
+      <c r="E18">
+        <f>YEAR(E17)</f>
+        <v>2028</v>
+      </c>
+      <c r="F18">
+        <f t="shared" ref="F18:BQ18" si="6">YEAR(F17)</f>
+        <v>2029</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="6"/>
+        <v>2029</v>
+      </c>
+      <c r="H18" s="21">
+        <f t="shared" si="6"/>
+        <v>2030</v>
+      </c>
+      <c r="I18" s="21">
+        <f t="shared" si="6"/>
+        <v>2030</v>
+      </c>
+      <c r="J18" s="21">
+        <f t="shared" si="6"/>
+        <v>2031</v>
+      </c>
+      <c r="K18" s="21">
+        <f t="shared" si="6"/>
+        <v>2031</v>
+      </c>
+      <c r="L18" s="21">
+        <f t="shared" si="6"/>
+        <v>2032</v>
+      </c>
+      <c r="M18" s="21">
+        <f t="shared" si="6"/>
+        <v>2032</v>
+      </c>
+      <c r="N18" s="21">
+        <f t="shared" si="6"/>
+        <v>2033</v>
+      </c>
+      <c r="O18" s="21">
+        <f t="shared" si="6"/>
+        <v>2033</v>
+      </c>
+      <c r="P18" s="21">
+        <f t="shared" si="6"/>
+        <v>2034</v>
+      </c>
+      <c r="Q18" s="21">
+        <f t="shared" si="6"/>
+        <v>2034</v>
+      </c>
+      <c r="R18" s="21">
+        <f t="shared" si="6"/>
+        <v>2035</v>
+      </c>
+      <c r="S18" s="21">
+        <f t="shared" si="6"/>
+        <v>2035</v>
+      </c>
+      <c r="T18" s="21">
+        <f t="shared" si="6"/>
+        <v>2036</v>
+      </c>
+      <c r="U18" s="21">
+        <f t="shared" si="6"/>
+        <v>2036</v>
+      </c>
+      <c r="V18" s="21">
+        <f t="shared" si="6"/>
+        <v>2037</v>
+      </c>
+      <c r="W18" s="21">
+        <f t="shared" si="6"/>
+        <v>2037</v>
+      </c>
+      <c r="X18" s="21">
+        <f t="shared" si="6"/>
+        <v>2038</v>
+      </c>
+      <c r="Y18" s="21">
+        <f t="shared" si="6"/>
+        <v>2038</v>
+      </c>
+      <c r="Z18" s="21">
+        <f t="shared" si="6"/>
+        <v>2039</v>
+      </c>
+      <c r="AA18" s="21">
+        <f t="shared" si="6"/>
+        <v>2039</v>
+      </c>
+      <c r="AB18" s="21">
+        <f t="shared" si="6"/>
+        <v>2040</v>
+      </c>
+      <c r="AC18" s="21">
+        <f t="shared" si="6"/>
+        <v>2040</v>
+      </c>
+      <c r="AD18" s="21">
+        <f t="shared" si="6"/>
+        <v>2041</v>
+      </c>
+      <c r="AE18" s="21">
+        <f t="shared" si="6"/>
+        <v>2041</v>
+      </c>
+      <c r="AF18" s="21">
+        <f t="shared" si="6"/>
+        <v>2042</v>
+      </c>
+      <c r="AG18" s="21">
+        <f t="shared" si="6"/>
+        <v>2042</v>
+      </c>
+      <c r="AH18" s="21">
+        <f t="shared" si="6"/>
+        <v>2043</v>
+      </c>
+      <c r="AI18" s="21">
+        <f t="shared" si="6"/>
+        <v>2043</v>
+      </c>
+      <c r="AJ18" s="21">
+        <f t="shared" si="6"/>
+        <v>2044</v>
+      </c>
+      <c r="AK18" s="21">
+        <f t="shared" si="6"/>
+        <v>2044</v>
+      </c>
+      <c r="AL18" s="21">
+        <f t="shared" si="6"/>
+        <v>2045</v>
+      </c>
+      <c r="AM18" s="21">
+        <f t="shared" si="6"/>
+        <v>2045</v>
+      </c>
+      <c r="AN18" s="21">
+        <f t="shared" si="6"/>
+        <v>2046</v>
+      </c>
+      <c r="AO18" s="21">
+        <f t="shared" si="6"/>
+        <v>2046</v>
+      </c>
+      <c r="AP18" s="21">
+        <f t="shared" si="6"/>
+        <v>2047</v>
+      </c>
+      <c r="AQ18" s="21">
+        <f t="shared" si="6"/>
+        <v>2047</v>
+      </c>
+      <c r="AR18" s="21">
+        <f t="shared" si="6"/>
+        <v>2048</v>
+      </c>
+      <c r="AS18" s="21">
+        <f t="shared" si="6"/>
+        <v>2048</v>
+      </c>
+      <c r="AT18" s="21">
+        <f t="shared" si="6"/>
+        <v>2049</v>
+      </c>
+      <c r="AU18" s="21">
+        <f t="shared" si="6"/>
+        <v>2049</v>
+      </c>
+      <c r="AV18" s="21">
+        <f t="shared" si="6"/>
+        <v>2050</v>
+      </c>
+      <c r="AW18" s="21">
+        <f t="shared" si="6"/>
+        <v>2050</v>
+      </c>
+      <c r="AX18" s="21">
+        <f t="shared" si="6"/>
+        <v>2051</v>
+      </c>
+      <c r="AY18" s="21">
+        <f t="shared" si="6"/>
+        <v>2051</v>
+      </c>
+      <c r="AZ18" s="21">
+        <f t="shared" si="6"/>
+        <v>2052</v>
+      </c>
+      <c r="BA18" s="21">
+        <f t="shared" si="6"/>
+        <v>2052</v>
+      </c>
+      <c r="BB18" s="21">
+        <f t="shared" si="6"/>
+        <v>2053</v>
+      </c>
+      <c r="BC18" s="21">
+        <f t="shared" si="6"/>
+        <v>2053</v>
+      </c>
+      <c r="BD18" s="21">
+        <f t="shared" si="6"/>
+        <v>2054</v>
+      </c>
+      <c r="BE18" s="21">
+        <f t="shared" si="6"/>
+        <v>2054</v>
+      </c>
+      <c r="BF18" s="21">
+        <f t="shared" si="6"/>
+        <v>2055</v>
+      </c>
+      <c r="BG18" s="21">
+        <f t="shared" si="6"/>
+        <v>2055</v>
+      </c>
+      <c r="BH18" s="21">
+        <f t="shared" si="6"/>
+        <v>2056</v>
+      </c>
+      <c r="BI18" s="21">
+        <f t="shared" si="6"/>
+        <v>2056</v>
+      </c>
+      <c r="BJ18" s="21">
+        <f t="shared" si="6"/>
+        <v>2057</v>
+      </c>
+      <c r="BK18" s="21">
+        <f t="shared" si="6"/>
+        <v>2057</v>
+      </c>
+      <c r="BL18" s="21">
+        <f t="shared" si="6"/>
+        <v>2058</v>
+      </c>
+      <c r="BM18" s="21">
+        <f t="shared" si="6"/>
+        <v>2058</v>
+      </c>
+      <c r="BN18" s="21">
+        <f t="shared" si="6"/>
+        <v>2059</v>
+      </c>
+      <c r="BO18" s="21">
+        <f t="shared" si="6"/>
+        <v>2059</v>
+      </c>
+      <c r="BP18" s="21">
+        <f t="shared" si="6"/>
+        <v>2060</v>
+      </c>
+      <c r="BQ18" s="21">
+        <f t="shared" si="6"/>
+        <v>2060</v>
+      </c>
+      <c r="BR18" s="21">
+        <f t="shared" ref="BR18:BU18" si="7">YEAR(BR17)</f>
+        <v>2061</v>
+      </c>
+      <c r="BS18" s="21">
+        <f t="shared" si="7"/>
+        <v>2061</v>
+      </c>
+      <c r="BT18" s="21">
+        <f t="shared" si="7"/>
+        <v>2062</v>
+      </c>
+      <c r="BU18" s="21">
+        <f t="shared" si="7"/>
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="19" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19" s="40" t="str">
+        <f>"1/2"</f>
+        <v>1/2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>135</v>
+      </c>
+      <c r="D19">
+        <f>IF(MONTH(D17)=3,1,2)</f>
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <f>IF(MONTH(E17)=3,1,2)</f>
+        <v>2</v>
+      </c>
+      <c r="F19">
+        <f t="shared" ref="F19:BQ19" si="8">IF(MONTH(F17)=3,1,2)</f>
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="H19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="I19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="J19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="K19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="L19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="M19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="N19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="O19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="P19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="Q19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="R19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="S19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="T19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="U19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="V19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="W19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="X19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="Y19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="Z19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AA19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AB19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AC19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AD19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AE19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AF19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AG19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AH19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AI19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AJ19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AK19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AL19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AM19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AN19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AO19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AP19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AQ19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AR19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AS19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AT19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AU19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AV19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AW19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AX19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="AY19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="AZ19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BA19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BB19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BC19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BD19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BE19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BF19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BG19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BH19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BI19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BJ19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BK19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BL19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BM19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BN19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BO19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BP19" s="21">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="BQ19" s="21">
+        <f t="shared" si="8"/>
+        <v>2</v>
+      </c>
+      <c r="BR19" s="21">
+        <f t="shared" ref="BR19:BU19" si="9">IF(MONTH(BR17)=3,1,2)</f>
+        <v>1</v>
+      </c>
+      <c r="BS19" s="21">
+        <f t="shared" si="9"/>
+        <v>2</v>
+      </c>
+      <c r="BT19" s="21">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="BU19" s="21">
+        <f t="shared" si="9"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>161</v>
+      </c>
+      <c r="B20" s="40" t="s">
+        <v>180</v>
+      </c>
+      <c r="C20">
+        <f>SUM(D20:BU20)</f>
+        <v>4</v>
+      </c>
+      <c r="D20">
+        <f t="shared" ref="D20:AI20" si="10">IF(AND(D16&gt;=$C$7,D16&lt;$C$8),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="H20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="K20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="L20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="M20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="N20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="O20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="P20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="R20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="S20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="T20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="U20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="V20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="W20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="X20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="Y20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="Z20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AA20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AB20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AC20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AD20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AE20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AF20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AG20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AH20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AI20" s="21">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AJ20" s="21">
+        <f t="shared" ref="AJ20:BO20" si="11">IF(AND(AJ16&gt;=$C$7,AJ16&lt;$C$8),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AK20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AL20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AM20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AN20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AO20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AP20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AQ20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AR20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AS20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AT20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AU20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AV20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AW20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AX20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AY20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AZ20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BA20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BB20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BC20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BD20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BE20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BF20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BG20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BH20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BI20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BJ20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BK20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BL20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BM20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BN20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BO20" s="21">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="BP20" s="21">
+        <f t="shared" ref="BP20:BU20" si="12">IF(AND(BP16&gt;=$C$7,BP16&lt;$C$8),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ20" s="21">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="BR20" s="21">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="BS20" s="21">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="BT20" s="21">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="BU20" s="21">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>162</v>
+      </c>
+      <c r="B21" t="s">
+        <v>180</v>
+      </c>
+      <c r="C21">
+        <f>SUM(D21:BU21)</f>
+        <v>60</v>
+      </c>
+      <c r="D21">
+        <f t="shared" ref="D21:AI21" si="13">IF(AND(D16&gt;=$C$8,D16&lt;$C$11),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="H21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="J21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="K21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="L21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="M21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="N21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="O21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="P21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="Q21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="R21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="S21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="T21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="U21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="V21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="W21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="X21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="Y21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="Z21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AA21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AB21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AC21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AD21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AE21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AF21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AG21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AH21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AI21" s="21">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="AJ21" s="21">
+        <f t="shared" ref="AJ21:BO21" si="14">IF(AND(AJ16&gt;=$C$8,AJ16&lt;$C$11),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="AK21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AL21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AM21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AN21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AO21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AP21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AQ21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AR21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AS21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AT21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AU21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AV21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AW21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AX21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AY21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="AZ21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BA21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BB21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BC21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BD21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BE21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BF21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BG21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BH21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BI21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BJ21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BK21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BL21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BM21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BN21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BO21" s="21">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="BP21" s="21">
+        <f t="shared" ref="BP21:BU21" si="15">IF(AND(BP16&gt;=$C$8,BP16&lt;$C$11),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ21" s="21">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="BR21" s="21">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="BS21" s="21">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="BT21" s="21">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="BU21" s="21">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>163</v>
+      </c>
+      <c r="B22" t="s">
+        <v>180</v>
+      </c>
+      <c r="C22">
+        <f>SUM(D22:BU22)</f>
+        <v>24</v>
+      </c>
+      <c r="D22">
+        <f t="shared" ref="D22:AI22" si="16">IF(AND(D16&gt;=$C$9,D16&lt;$C$10),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="H22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="I22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="J22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="K22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="L22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="M22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="N22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="O22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="P22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="Q22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="R22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="S22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="T22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="U22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="V22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="W22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="X22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="Y22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="Z22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AA22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AB22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AC22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AD22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AE22" s="21">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="AF22" s="21">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AG22" s="21">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AH22" s="21">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AI22" s="21">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AJ22" s="21">
+        <f t="shared" ref="AJ22:BO22" si="17">IF(AND(AJ16&gt;=$C$9,AJ16&lt;$C$10),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="AK22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AL22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AM22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AN22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AO22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AP22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AQ22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AR22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AS22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AT22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AU22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AV22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AW22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AX22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AY22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="AZ22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BA22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BB22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BC22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BD22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BE22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BF22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BG22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BH22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BI22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BJ22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BK22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BL22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BM22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BN22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BO22" s="21">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="BP22" s="21">
+        <f t="shared" ref="BP22:BU22" si="18">IF(AND(BP16&gt;=$C$9,BP16&lt;$C$10),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ22" s="21">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="BR22" s="21">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="BS22" s="21">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="BT22" s="21">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="BU22" s="21">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" t="s">
+        <v>135</v>
+      </c>
+      <c r="D23" s="8">
+        <f>(D16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>3.2498288843258041</v>
+      </c>
+      <c r="E23" s="8">
+        <f>(E16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>3.7508555783709787</v>
+      </c>
+      <c r="F23" s="8">
+        <f>(F16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>4.2518822724161529</v>
+      </c>
+      <c r="G23" s="8">
+        <f>(G16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>4.7501711156741955</v>
+      </c>
+      <c r="H23" s="8">
+        <f>(H16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>5.2511978097193701</v>
+      </c>
+      <c r="I23" s="8">
+        <f>(I16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>5.7494866529774127</v>
+      </c>
+      <c r="J23" s="8">
+        <f>(J16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>6.2505133470225873</v>
+      </c>
+      <c r="K23" s="8">
+        <f>(K16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>6.7488021902806299</v>
+      </c>
+      <c r="L23" s="8">
+        <f>(L16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>7.2498288843258045</v>
+      </c>
+      <c r="M23" s="8">
+        <f>(M16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>7.7508555783709792</v>
+      </c>
+      <c r="N23" s="8">
+        <f>(N16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>8.2518822724161538</v>
+      </c>
+      <c r="O23" s="8">
+        <f>(O16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>8.7501711156741955</v>
+      </c>
+      <c r="P23" s="8">
+        <f>(P16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>9.2511978097193701</v>
+      </c>
+      <c r="Q23" s="8">
+        <f>(Q16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>9.7494866529774136</v>
+      </c>
+      <c r="R23" s="8">
+        <f>(R16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>10.250513347022586</v>
+      </c>
+      <c r="S23" s="8">
+        <f>(S16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>10.74880219028063</v>
+      </c>
+      <c r="T23" s="8">
+        <f>(T16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>11.249828884325805</v>
+      </c>
+      <c r="U23" s="8">
+        <f>(U16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>11.750855578370979</v>
+      </c>
+      <c r="V23" s="8">
+        <f>(V16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>12.251882272416154</v>
+      </c>
+      <c r="W23" s="8">
+        <f>(W16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>12.750171115674195</v>
+      </c>
+      <c r="X23" s="8">
+        <f>(X16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>13.25119780971937</v>
+      </c>
+      <c r="Y23" s="8">
+        <f>(Y16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>13.749486652977414</v>
+      </c>
+      <c r="Z23" s="8">
+        <f>(Z16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>14.250513347022586</v>
+      </c>
+      <c r="AA23" s="8">
+        <f>(AA16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>14.74880219028063</v>
+      </c>
+      <c r="AB23" s="8">
+        <f>(AB16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>15.249828884325805</v>
+      </c>
+      <c r="AC23" s="8">
+        <f>(AC16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>15.750855578370979</v>
+      </c>
+      <c r="AD23" s="8">
+        <f>(AD16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>16.251882272416154</v>
+      </c>
+      <c r="AE23" s="8">
+        <f>(AE16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>16.750171115674195</v>
+      </c>
+      <c r="AF23" s="8">
+        <f>(AF16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>17.251197809719372</v>
+      </c>
+      <c r="AG23" s="8">
+        <f>(AG16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>17.749486652977414</v>
+      </c>
+      <c r="AH23" s="8">
+        <f>(AH16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>18.250513347022586</v>
+      </c>
+      <c r="AI23" s="8">
+        <f>(AI16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>18.748802190280628</v>
+      </c>
+      <c r="AJ23" s="8">
+        <f>(AJ16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>19.249828884325805</v>
+      </c>
+      <c r="AK23" s="8">
+        <f>(AK16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>19.750855578370977</v>
+      </c>
+      <c r="AL23" s="8">
+        <f>(AL16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>20.251882272416154</v>
+      </c>
+      <c r="AM23" s="8">
+        <f>(AM16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>20.750171115674195</v>
+      </c>
+      <c r="AN23" s="8">
+        <f>(AN16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>21.251197809719372</v>
+      </c>
+      <c r="AO23" s="8">
+        <f>(AO16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>21.749486652977414</v>
+      </c>
+      <c r="AP23" s="8">
+        <f>(AP16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>22.250513347022586</v>
+      </c>
+      <c r="AQ23" s="8">
+        <f>(AQ16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>22.748802190280628</v>
+      </c>
+      <c r="AR23" s="8">
+        <f>(AR16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>23.249828884325805</v>
+      </c>
+      <c r="AS23" s="8">
+        <f>(AS16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>23.750855578370977</v>
+      </c>
+      <c r="AT23" s="8">
+        <f>(AT16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>24.251882272416154</v>
+      </c>
+      <c r="AU23" s="8">
+        <f>(AU16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>24.750171115674195</v>
+      </c>
+      <c r="AV23" s="8">
+        <f>(AV16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>25.251197809719372</v>
+      </c>
+      <c r="AW23" s="8">
+        <f>(AW16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>25.749486652977414</v>
+      </c>
+      <c r="AX23" s="8">
+        <f>(AX16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>26.250513347022586</v>
+      </c>
+      <c r="AY23" s="8">
+        <f>(AY16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>26.748802190280628</v>
+      </c>
+      <c r="AZ23" s="8">
+        <f>(AZ16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>27.249828884325805</v>
+      </c>
+      <c r="BA23" s="8">
+        <f>(BA16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>27.750855578370977</v>
+      </c>
+      <c r="BB23" s="8">
+        <f>(BB16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>28.251882272416154</v>
+      </c>
+      <c r="BC23" s="8">
+        <f>(BC16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>28.750171115674195</v>
+      </c>
+      <c r="BD23" s="8">
+        <f>(BD16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>29.251197809719372</v>
+      </c>
+      <c r="BE23" s="8">
+        <f>(BE16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>29.749486652977414</v>
+      </c>
+      <c r="BF23" s="8">
+        <f>(BF16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>30.250513347022586</v>
+      </c>
+      <c r="BG23" s="8">
+        <f>(BG16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>30.748802190280628</v>
+      </c>
+      <c r="BH23" s="8">
+        <f>(BH16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>31.249828884325805</v>
+      </c>
+      <c r="BI23" s="8">
+        <f>(BI16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>31.750855578370977</v>
+      </c>
+      <c r="BJ23" s="8">
+        <f>(BJ16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>32.251882272416154</v>
+      </c>
+      <c r="BK23" s="8">
+        <f>(BK16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>32.750171115674199</v>
+      </c>
+      <c r="BL23" s="8">
+        <f>(BL16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>33.251197809719372</v>
+      </c>
+      <c r="BM23" s="8">
+        <f>(BM16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>33.74948665297741</v>
+      </c>
+      <c r="BN23" s="8">
+        <f>(BN16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>34.25051334702259</v>
+      </c>
+      <c r="BO23" s="8">
+        <f>(BO16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>34.748802190280628</v>
+      </c>
+      <c r="BP23" s="8">
+        <f>(BP16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>35.249828884325801</v>
+      </c>
+      <c r="BQ23" s="8">
+        <f>(BQ16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>35.750855578370981</v>
+      </c>
+      <c r="BR23" s="8">
+        <f>(BR16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>36.251882272416154</v>
+      </c>
+      <c r="BS23" s="8">
+        <f>(BS16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>36.750171115674199</v>
+      </c>
+      <c r="BT23" s="8">
+        <f>(BT16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>37.251197809719372</v>
+      </c>
+      <c r="BU23" s="8">
+        <f>(BU16-DATE(Inputs!$B$20,7,1))/365.25</f>
+        <v>37.74948665297741</v>
+      </c>
+    </row>
+    <row r="24" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>171</v>
+      </c>
+      <c r="B24" t="s">
+        <v>170</v>
+      </c>
+      <c r="C24" t="s">
+        <v>135</v>
+      </c>
+      <c r="D24">
+        <f>IF(D20+D21&gt;1,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <f>IF(E20+E21&gt;1,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <f t="shared" ref="F24:BQ24" si="19">IF(F20+F21&gt;1,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="H24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="I24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="J24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="K24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="L24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="N24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="O24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="P24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="Q24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="R24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="S24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="T24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="U24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="V24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="W24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="X24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="Y24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="Z24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AA24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AB24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AC24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AD24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AE24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AF24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AG24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AH24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AI24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AJ24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AK24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AL24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AM24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AN24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AO24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AP24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AQ24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AR24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AS24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AT24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AU24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AV24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AW24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AX24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AY24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AZ24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BA24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BB24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BC24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BD24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BE24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BF24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BG24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BH24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BI24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BJ24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BK24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BL24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BM24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BN24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BO24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BP24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BQ24" s="21">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="BR24" s="21">
+        <f t="shared" ref="BR24:BU24" si="20">IF(BR20+BR21&gt;1,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BS24" s="21">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="BT24" s="21">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="BU24" s="21">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:73" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="42" t="s">
+        <v>176</v>
+      </c>
+      <c r="B26" s="42"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="41"/>
+    </row>
+    <row r="27" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27" t="s">
+        <v>150</v>
+      </c>
+      <c r="C27" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="28" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="B28" t="s">
+        <v>170</v>
+      </c>
+      <c r="C28">
+        <f>SUM(D20:BU20)-Inputs!B9/6</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="E28" s="12"/>
+    </row>
+    <row r="29" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="B29" t="s">
+        <v>170</v>
+      </c>
+      <c r="C29">
+        <f>SUM(D21:BU21)-Inputs!B10*2</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="E29" s="12"/>
+    </row>
+    <row r="30" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="B30" t="s">
+        <v>170</v>
+      </c>
+      <c r="C30">
+        <f>SUM(D22:BU22)-Inputs!B40*2</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="E30" s="12"/>
+    </row>
+    <row r="31" spans="1:73" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="B31" t="s">
+        <v>170</v>
+      </c>
+      <c r="C31">
+        <f>SUM(D24:BU24)</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="E31" s="12"/>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A5:C5"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Stage 2 step 2.8: DSCR, LLCR, project and equity IRR; D22
</commit_message>
<xml_diff>
--- a/model/hydro_pf_model_v1.xlsx
+++ b/model/hydro_pf_model_v1.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22470" windowHeight="4815" firstSheet="4" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22470" windowHeight="4815" firstSheet="5" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="345">
   <si>
     <t>Cover</t>
   </si>
@@ -1094,6 +1094,60 @@
   <si>
     <t>total CFADS − total Debt service + total Initial funding − total Distributions − last column retained cash closing  =</t>
   </si>
+  <si>
+    <t>DSCR (semester)</t>
+  </si>
+  <si>
+    <t>PV of remaining CFADS</t>
+  </si>
+  <si>
+    <t>LLCR</t>
+  </si>
+  <si>
+    <t>Min 12-month DSCR</t>
+  </si>
+  <si>
+    <t>Min LLCR</t>
+  </si>
+  <si>
+    <t>1st semester LLCR - target DSCR =</t>
+  </si>
+  <si>
+    <t>1.A. RATIOS</t>
+  </si>
+  <si>
+    <t>Average DSCR (semester)</t>
+  </si>
+  <si>
+    <t>Project cash flow</t>
+  </si>
+  <si>
+    <t>Equity cash flow</t>
+  </si>
+  <si>
+    <t>Project IRR (semiannual)</t>
+  </si>
+  <si>
+    <t>Project IRR (annual)</t>
+  </si>
+  <si>
+    <t>Equity multiple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit </t>
+  </si>
+  <si>
+    <t>Equity IRR (semiannual)</t>
+  </si>
+  <si>
+    <t>Equity IRR (annual)</t>
+  </si>
+  <si>
+    <t>1. RETURNS: IRR</t>
+  </si>
+  <si>
+    <t>Min DSCR (semester)</t>
+  </si>
 </sst>
 </file>
 
@@ -1262,7 +1316,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1346,6 +1400,7 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1721,46 +1776,3138 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:BU19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75">
+    <row r="1" spans="1:73" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:73">
       <c r="A2" t="s">
         <v>61</v>
       </c>
     </row>
+    <row r="4" spans="1:73" ht="15.75">
+      <c r="A4" s="58" t="s">
+        <v>333</v>
+      </c>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+    </row>
+    <row r="5" spans="1:73">
+      <c r="A5" t="s">
+        <v>273</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="6" spans="1:73">
+      <c r="A6" t="str">
+        <f>Debt!A7</f>
+        <v>Repayment flag</v>
+      </c>
+      <c r="B6" t="str">
+        <f>Debt!B7</f>
+        <v>flag</v>
+      </c>
+      <c r="C6">
+        <f>Debt!C7</f>
+        <v>24</v>
+      </c>
+      <c r="D6">
+        <f>Debt!D7</f>
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <f>Debt!E7</f>
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <f>Debt!F7</f>
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <f>Debt!G7</f>
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <f>Debt!H7</f>
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <f>Debt!I7</f>
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <f>Debt!J7</f>
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <f>Debt!K7</f>
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <f>Debt!L7</f>
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <f>Debt!M7</f>
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <f>Debt!N7</f>
+        <v>1</v>
+      </c>
+      <c r="O6">
+        <f>Debt!O7</f>
+        <v>1</v>
+      </c>
+      <c r="P6">
+        <f>Debt!P7</f>
+        <v>1</v>
+      </c>
+      <c r="Q6">
+        <f>Debt!Q7</f>
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <f>Debt!R7</f>
+        <v>1</v>
+      </c>
+      <c r="S6">
+        <f>Debt!S7</f>
+        <v>1</v>
+      </c>
+      <c r="T6">
+        <f>Debt!T7</f>
+        <v>1</v>
+      </c>
+      <c r="U6">
+        <f>Debt!U7</f>
+        <v>1</v>
+      </c>
+      <c r="V6">
+        <f>Debt!V7</f>
+        <v>1</v>
+      </c>
+      <c r="W6">
+        <f>Debt!W7</f>
+        <v>1</v>
+      </c>
+      <c r="X6">
+        <f>Debt!X7</f>
+        <v>1</v>
+      </c>
+      <c r="Y6">
+        <f>Debt!Y7</f>
+        <v>1</v>
+      </c>
+      <c r="Z6">
+        <f>Debt!Z7</f>
+        <v>1</v>
+      </c>
+      <c r="AA6">
+        <f>Debt!AA7</f>
+        <v>1</v>
+      </c>
+      <c r="AB6">
+        <f>Debt!AB7</f>
+        <v>1</v>
+      </c>
+      <c r="AC6">
+        <f>Debt!AC7</f>
+        <v>1</v>
+      </c>
+      <c r="AD6">
+        <f>Debt!AD7</f>
+        <v>1</v>
+      </c>
+      <c r="AE6">
+        <f>Debt!AE7</f>
+        <v>1</v>
+      </c>
+      <c r="AF6">
+        <f>Debt!AF7</f>
+        <v>0</v>
+      </c>
+      <c r="AG6">
+        <f>Debt!AG7</f>
+        <v>0</v>
+      </c>
+      <c r="AH6">
+        <f>Debt!AH7</f>
+        <v>0</v>
+      </c>
+      <c r="AI6">
+        <f>Debt!AI7</f>
+        <v>0</v>
+      </c>
+      <c r="AJ6">
+        <f>Debt!AJ7</f>
+        <v>0</v>
+      </c>
+      <c r="AK6">
+        <f>Debt!AK7</f>
+        <v>0</v>
+      </c>
+      <c r="AL6">
+        <f>Debt!AL7</f>
+        <v>0</v>
+      </c>
+      <c r="AM6">
+        <f>Debt!AM7</f>
+        <v>0</v>
+      </c>
+      <c r="AN6">
+        <f>Debt!AN7</f>
+        <v>0</v>
+      </c>
+      <c r="AO6">
+        <f>Debt!AO7</f>
+        <v>0</v>
+      </c>
+      <c r="AP6">
+        <f>Debt!AP7</f>
+        <v>0</v>
+      </c>
+      <c r="AQ6">
+        <f>Debt!AQ7</f>
+        <v>0</v>
+      </c>
+      <c r="AR6">
+        <f>Debt!AR7</f>
+        <v>0</v>
+      </c>
+      <c r="AS6">
+        <f>Debt!AS7</f>
+        <v>0</v>
+      </c>
+      <c r="AT6">
+        <f>Debt!AT7</f>
+        <v>0</v>
+      </c>
+      <c r="AU6">
+        <f>Debt!AU7</f>
+        <v>0</v>
+      </c>
+      <c r="AV6">
+        <f>Debt!AV7</f>
+        <v>0</v>
+      </c>
+      <c r="AW6">
+        <f>Debt!AW7</f>
+        <v>0</v>
+      </c>
+      <c r="AX6">
+        <f>Debt!AX7</f>
+        <v>0</v>
+      </c>
+      <c r="AY6">
+        <f>Debt!AY7</f>
+        <v>0</v>
+      </c>
+      <c r="AZ6">
+        <f>Debt!AZ7</f>
+        <v>0</v>
+      </c>
+      <c r="BA6">
+        <f>Debt!BA7</f>
+        <v>0</v>
+      </c>
+      <c r="BB6">
+        <f>Debt!BB7</f>
+        <v>0</v>
+      </c>
+      <c r="BC6">
+        <f>Debt!BC7</f>
+        <v>0</v>
+      </c>
+      <c r="BD6">
+        <f>Debt!BD7</f>
+        <v>0</v>
+      </c>
+      <c r="BE6">
+        <f>Debt!BE7</f>
+        <v>0</v>
+      </c>
+      <c r="BF6">
+        <f>Debt!BF7</f>
+        <v>0</v>
+      </c>
+      <c r="BG6">
+        <f>Debt!BG7</f>
+        <v>0</v>
+      </c>
+      <c r="BH6">
+        <f>Debt!BH7</f>
+        <v>0</v>
+      </c>
+      <c r="BI6">
+        <f>Debt!BI7</f>
+        <v>0</v>
+      </c>
+      <c r="BJ6">
+        <f>Debt!BJ7</f>
+        <v>0</v>
+      </c>
+      <c r="BK6">
+        <f>Debt!BK7</f>
+        <v>0</v>
+      </c>
+      <c r="BL6">
+        <f>Debt!BL7</f>
+        <v>0</v>
+      </c>
+      <c r="BM6">
+        <f>Debt!BM7</f>
+        <v>0</v>
+      </c>
+      <c r="BN6">
+        <f>Debt!BN7</f>
+        <v>0</v>
+      </c>
+      <c r="BO6">
+        <f>Debt!BO7</f>
+        <v>0</v>
+      </c>
+      <c r="BP6">
+        <f>Debt!BP7</f>
+        <v>0</v>
+      </c>
+      <c r="BQ6">
+        <f>Debt!BQ7</f>
+        <v>0</v>
+      </c>
+      <c r="BR6">
+        <f>Debt!BR7</f>
+        <v>0</v>
+      </c>
+      <c r="BS6">
+        <f>Debt!BS7</f>
+        <v>0</v>
+      </c>
+      <c r="BT6">
+        <f>Debt!BT7</f>
+        <v>0</v>
+      </c>
+      <c r="BU6">
+        <f>Debt!BU7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:73">
+      <c r="A7" t="str">
+        <f>Debt!A8</f>
+        <v>CFADS</v>
+      </c>
+      <c r="B7" t="str">
+        <f>Debt!B8</f>
+        <v>USD</v>
+      </c>
+      <c r="C7">
+        <f>Debt!C8</f>
+        <v>32632556.585838038</v>
+      </c>
+      <c r="D7">
+        <f>Debt!D8</f>
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <f>Debt!E8</f>
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <f>Debt!F8</f>
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <f>Debt!G8</f>
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f>Debt!H8</f>
+        <v>1220374.4089345317</v>
+      </c>
+      <c r="I7">
+        <f>Debt!I8</f>
+        <v>367941.26282097551</v>
+      </c>
+      <c r="J7">
+        <f>Debt!J8</f>
+        <v>1209397.0949984677</v>
+      </c>
+      <c r="K7">
+        <f>Debt!K8</f>
+        <v>356855.09485584439</v>
+      </c>
+      <c r="L7">
+        <f>Debt!L8</f>
+        <v>1198200.3865466854</v>
+      </c>
+      <c r="M7">
+        <f>Debt!M8</f>
+        <v>345516.06830213021</v>
+      </c>
+      <c r="N7">
+        <f>Debt!N8</f>
+        <v>1186748.2982463562</v>
+      </c>
+      <c r="O7">
+        <f>Debt!O8</f>
+        <v>333981.70647828188</v>
+      </c>
+      <c r="P7">
+        <f>Debt!P8</f>
+        <v>1175098.9269825253</v>
+      </c>
+      <c r="Q7">
+        <f>Debt!Q8</f>
+        <v>322216.81688222941</v>
+      </c>
+      <c r="R7">
+        <f>Debt!R8</f>
+        <v>1163216.7293477135</v>
+      </c>
+      <c r="S7">
+        <f>Debt!S8</f>
+        <v>310216.79214560974</v>
+      </c>
+      <c r="T7">
+        <f>Debt!T8</f>
+        <v>1151097.0520333601</v>
+      </c>
+      <c r="U7">
+        <f>Debt!U8</f>
+        <v>297943.06514077552</v>
+      </c>
+      <c r="V7">
+        <f>Debt!V8</f>
+        <v>1138700.9433579245</v>
+      </c>
+      <c r="W7">
+        <f>Debt!W8</f>
+        <v>285457.90095756587</v>
+      </c>
+      <c r="X7">
+        <f>Debt!X8</f>
+        <v>1126091.2892581739</v>
+      </c>
+      <c r="Y7">
+        <f>Debt!Y8</f>
+        <v>272723.20609994943</v>
+      </c>
+      <c r="Z7">
+        <f>Debt!Z8</f>
+        <v>1113229.6164067774</v>
+      </c>
+      <c r="AA7">
+        <f>Debt!AA8</f>
+        <v>259733.99340423674</v>
+      </c>
+      <c r="AB7">
+        <f>Debt!AB8</f>
+        <v>1100110.887912899</v>
+      </c>
+      <c r="AC7">
+        <f>Debt!AC8</f>
+        <v>246448.51657114364</v>
+      </c>
+      <c r="AD7">
+        <f>Debt!AD8</f>
+        <v>1086692.9412237522</v>
+      </c>
+      <c r="AE7">
+        <f>Debt!AE8</f>
+        <v>232934.17333635734</v>
+      </c>
+      <c r="AF7">
+        <f>Debt!AF8</f>
+        <v>1073043.8460997068</v>
+      </c>
+      <c r="AG7">
+        <f>Debt!AG8</f>
+        <v>219149.7300746867</v>
+      </c>
+      <c r="AH7">
+        <f>Debt!AH8</f>
+        <v>1059121.9577739565</v>
+      </c>
+      <c r="AI7">
+        <f>Debt!AI8</f>
+        <v>205089.788519767</v>
+      </c>
+      <c r="AJ7">
+        <f>Debt!AJ8</f>
+        <v>1044921.824153874</v>
+      </c>
+      <c r="AK7">
+        <f>Debt!AK8</f>
+        <v>190709.16113469214</v>
+      </c>
+      <c r="AL7">
+        <f>Debt!AL8</f>
+        <v>732272.82580145611</v>
+      </c>
+      <c r="AM7">
+        <f>Debt!AM8</f>
+        <v>176080.80139608099</v>
+      </c>
+      <c r="AN7">
+        <f>Debt!AN8</f>
+        <v>723555.55378948129</v>
+      </c>
+      <c r="AO7">
+        <f>Debt!AO8</f>
+        <v>161160.07670195331</v>
+      </c>
+      <c r="AP7">
+        <f>Debt!AP8</f>
+        <v>718982.63265880744</v>
+      </c>
+      <c r="AQ7">
+        <f>Debt!AQ8</f>
+        <v>145941.14379518793</v>
+      </c>
+      <c r="AR7">
+        <f>Debt!AR8</f>
+        <v>714318.31632683706</v>
+      </c>
+      <c r="AS7">
+        <f>Debt!AS8</f>
+        <v>130375.09023260616</v>
+      </c>
+      <c r="AT7">
+        <f>Debt!AT8</f>
+        <v>709547.61405085807</v>
+      </c>
+      <c r="AU7">
+        <f>Debt!AU8</f>
+        <v>114540.88320348423</v>
+      </c>
+      <c r="AV7">
+        <f>Debt!AV8</f>
+        <v>704694.72778726846</v>
+      </c>
+      <c r="AW7">
+        <f>Debt!AW8</f>
+        <v>98390.210944054183</v>
+      </c>
+      <c r="AX7">
+        <f>Debt!AX8</f>
+        <v>699744.85089028359</v>
+      </c>
+      <c r="AY7">
+        <f>Debt!AY8</f>
+        <v>81916.748524889117</v>
+      </c>
+      <c r="AZ7">
+        <f>Debt!AZ8</f>
+        <v>694696.04488814552</v>
+      </c>
+      <c r="BA7">
+        <f>Debt!BA8</f>
+        <v>65067.551544468035</v>
+      </c>
+      <c r="BB7">
+        <f>Debt!BB8</f>
+        <v>689532.08331884071</v>
+      </c>
+      <c r="BC7">
+        <f>Debt!BC8</f>
+        <v>47928.096628048341</v>
+      </c>
+      <c r="BD7">
+        <f>Debt!BD8</f>
+        <v>684279.16315830906</v>
+      </c>
+      <c r="BE7">
+        <f>Debt!BE8</f>
+        <v>30446.089568821597</v>
+      </c>
+      <c r="BF7">
+        <f>Debt!BF8</f>
+        <v>678921.2572169716</v>
+      </c>
+      <c r="BG7">
+        <f>Debt!BG8</f>
+        <v>12614.684059765772</v>
+      </c>
+      <c r="BH7">
+        <f>Debt!BH8</f>
+        <v>673456.26723065635</v>
+      </c>
+      <c r="BI7">
+        <f>Debt!BI8</f>
+        <v>-5623.4286220169161</v>
+      </c>
+      <c r="BJ7">
+        <f>Debt!BJ8</f>
+        <v>667866.62915503676</v>
+      </c>
+      <c r="BK7">
+        <f>Debt!BK8</f>
+        <v>-24175.725828419672</v>
+      </c>
+      <c r="BL7">
+        <f>Debt!BL8</f>
+        <v>662180.69943936495</v>
+      </c>
+      <c r="BM7">
+        <f>Debt!BM8</f>
+        <v>-43098.812490673736</v>
+      </c>
+      <c r="BN7">
+        <f>Debt!BN8</f>
+        <v>656381.12973820628</v>
+      </c>
+      <c r="BO7">
+        <f>Debt!BO8</f>
+        <v>-62400.099271676852</v>
+      </c>
+      <c r="BP7">
+        <f>Debt!BP8</f>
+        <v>0</v>
+      </c>
+      <c r="BQ7">
+        <f>Debt!BQ8</f>
+        <v>0</v>
+      </c>
+      <c r="BR7">
+        <f>Debt!BR8</f>
+        <v>0</v>
+      </c>
+      <c r="BS7">
+        <f>Debt!BS8</f>
+        <v>0</v>
+      </c>
+      <c r="BT7">
+        <f>Debt!BT8</f>
+        <v>0</v>
+      </c>
+      <c r="BU7">
+        <f>Debt!BU8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:73">
+      <c r="A8" t="str">
+        <f>Debt!A25</f>
+        <v xml:space="preserve">        Debt service</v>
+      </c>
+      <c r="B8" t="str">
+        <f>Debt!B25</f>
+        <v>USD</v>
+      </c>
+      <c r="C8">
+        <f>Debt!C25</f>
+        <v>12963649.757217973</v>
+      </c>
+      <c r="D8">
+        <f>Debt!D25</f>
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <f>Debt!E25</f>
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <f>Debt!F25</f>
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <f>Debt!G25</f>
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <f>Debt!H25</f>
+        <v>903981.04365520866</v>
+      </c>
+      <c r="I8">
+        <f>Debt!I25</f>
+        <v>272549.08357109292</v>
+      </c>
+      <c r="J8">
+        <f>Debt!J25</f>
+        <v>895849.6999988649</v>
+      </c>
+      <c r="K8">
+        <f>Debt!K25</f>
+        <v>264337.10730062547</v>
+      </c>
+      <c r="L8">
+        <f>Debt!L25</f>
+        <v>887555.84188643354</v>
+      </c>
+      <c r="M8">
+        <f>Debt!M25</f>
+        <v>255937.8283719483</v>
+      </c>
+      <c r="N8">
+        <f>Debt!N25</f>
+        <v>879072.81351581938</v>
+      </c>
+      <c r="O8">
+        <f>Debt!O25</f>
+        <v>247393.85665057914</v>
+      </c>
+      <c r="P8">
+        <f>Debt!P25</f>
+        <v>870443.64961668535</v>
+      </c>
+      <c r="Q8">
+        <f>Debt!Q25</f>
+        <v>238679.12361646621</v>
+      </c>
+      <c r="R8">
+        <f>Debt!R25</f>
+        <v>861642.02173904702</v>
+      </c>
+      <c r="S8">
+        <f>Debt!S25</f>
+        <v>229790.21640415533</v>
+      </c>
+      <c r="T8">
+        <f>Debt!T25</f>
+        <v>852664.48298767407</v>
+      </c>
+      <c r="U8">
+        <f>Debt!U25</f>
+        <v>220698.5667709448</v>
+      </c>
+      <c r="V8">
+        <f>Debt!V25</f>
+        <v>843482.18026512919</v>
+      </c>
+      <c r="W8">
+        <f>Debt!W25</f>
+        <v>211450.29700560434</v>
+      </c>
+      <c r="X8">
+        <f>Debt!X25</f>
+        <v>834141.69574679539</v>
+      </c>
+      <c r="Y8">
+        <f>Debt!Y25</f>
+        <v>202017.18970366623</v>
+      </c>
+      <c r="Z8">
+        <f>Debt!Z25</f>
+        <v>824614.53067168687</v>
+      </c>
+      <c r="AA8">
+        <f>Debt!AA25</f>
+        <v>192395.55066980497</v>
+      </c>
+      <c r="AB8">
+        <f>Debt!AB25</f>
+        <v>814896.95400955481</v>
+      </c>
+      <c r="AC8">
+        <f>Debt!AC25</f>
+        <v>182554.45671936564</v>
+      </c>
+      <c r="AD8">
+        <f>Debt!AD25</f>
+        <v>804957.73423981643</v>
+      </c>
+      <c r="AE8">
+        <f>Debt!AE25</f>
+        <v>172543.83210100542</v>
+      </c>
+      <c r="AF8">
+        <f>Debt!AF25</f>
+        <v>0</v>
+      </c>
+      <c r="AG8">
+        <f>Debt!AG25</f>
+        <v>0</v>
+      </c>
+      <c r="AH8">
+        <f>Debt!AH25</f>
+        <v>0</v>
+      </c>
+      <c r="AI8">
+        <f>Debt!AI25</f>
+        <v>0</v>
+      </c>
+      <c r="AJ8">
+        <f>Debt!AJ25</f>
+        <v>0</v>
+      </c>
+      <c r="AK8">
+        <f>Debt!AK25</f>
+        <v>0</v>
+      </c>
+      <c r="AL8">
+        <f>Debt!AL25</f>
+        <v>0</v>
+      </c>
+      <c r="AM8">
+        <f>Debt!AM25</f>
+        <v>0</v>
+      </c>
+      <c r="AN8">
+        <f>Debt!AN25</f>
+        <v>0</v>
+      </c>
+      <c r="AO8">
+        <f>Debt!AO25</f>
+        <v>0</v>
+      </c>
+      <c r="AP8">
+        <f>Debt!AP25</f>
+        <v>0</v>
+      </c>
+      <c r="AQ8">
+        <f>Debt!AQ25</f>
+        <v>0</v>
+      </c>
+      <c r="AR8">
+        <f>Debt!AR25</f>
+        <v>0</v>
+      </c>
+      <c r="AS8">
+        <f>Debt!AS25</f>
+        <v>0</v>
+      </c>
+      <c r="AT8">
+        <f>Debt!AT25</f>
+        <v>0</v>
+      </c>
+      <c r="AU8">
+        <f>Debt!AU25</f>
+        <v>0</v>
+      </c>
+      <c r="AV8">
+        <f>Debt!AV25</f>
+        <v>0</v>
+      </c>
+      <c r="AW8">
+        <f>Debt!AW25</f>
+        <v>0</v>
+      </c>
+      <c r="AX8">
+        <f>Debt!AX25</f>
+        <v>0</v>
+      </c>
+      <c r="AY8">
+        <f>Debt!AY25</f>
+        <v>0</v>
+      </c>
+      <c r="AZ8">
+        <f>Debt!AZ25</f>
+        <v>0</v>
+      </c>
+      <c r="BA8">
+        <f>Debt!BA25</f>
+        <v>0</v>
+      </c>
+      <c r="BB8">
+        <f>Debt!BB25</f>
+        <v>0</v>
+      </c>
+      <c r="BC8">
+        <f>Debt!BC25</f>
+        <v>0</v>
+      </c>
+      <c r="BD8">
+        <f>Debt!BD25</f>
+        <v>0</v>
+      </c>
+      <c r="BE8">
+        <f>Debt!BE25</f>
+        <v>0</v>
+      </c>
+      <c r="BF8">
+        <f>Debt!BF25</f>
+        <v>0</v>
+      </c>
+      <c r="BG8">
+        <f>Debt!BG25</f>
+        <v>0</v>
+      </c>
+      <c r="BH8">
+        <f>Debt!BH25</f>
+        <v>0</v>
+      </c>
+      <c r="BI8">
+        <f>Debt!BI25</f>
+        <v>0</v>
+      </c>
+      <c r="BJ8">
+        <f>Debt!BJ25</f>
+        <v>0</v>
+      </c>
+      <c r="BK8">
+        <f>Debt!BK25</f>
+        <v>0</v>
+      </c>
+      <c r="BL8">
+        <f>Debt!BL25</f>
+        <v>0</v>
+      </c>
+      <c r="BM8">
+        <f>Debt!BM25</f>
+        <v>0</v>
+      </c>
+      <c r="BN8">
+        <f>Debt!BN25</f>
+        <v>0</v>
+      </c>
+      <c r="BO8">
+        <f>Debt!BO25</f>
+        <v>0</v>
+      </c>
+      <c r="BP8">
+        <f>Debt!BP25</f>
+        <v>0</v>
+      </c>
+      <c r="BQ8">
+        <f>Debt!BQ25</f>
+        <v>0</v>
+      </c>
+      <c r="BR8">
+        <f>Debt!BR25</f>
+        <v>0</v>
+      </c>
+      <c r="BS8">
+        <f>Debt!BS25</f>
+        <v>0</v>
+      </c>
+      <c r="BT8">
+        <f>Debt!BT25</f>
+        <v>0</v>
+      </c>
+      <c r="BU8">
+        <f>Debt!BU25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:73">
+      <c r="A9" t="str">
+        <f>Debt!A23</f>
+        <v xml:space="preserve">        Opening balance</v>
+      </c>
+      <c r="B9" t="str">
+        <f>Debt!B23</f>
+        <v>USD</v>
+      </c>
+      <c r="C9">
+        <f>Debt!C23</f>
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <f>Debt!D23</f>
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <f>Debt!E23</f>
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <f>Debt!F23</f>
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <f>Debt!G23</f>
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <f>Debt!H23</f>
+        <v>8064962.5333756506</v>
+      </c>
+      <c r="I9">
+        <f>Debt!I23</f>
+        <v>7523904.8037223462</v>
+      </c>
+      <c r="J9">
+        <f>Debt!J23</f>
+        <v>7589931.4363187589</v>
+      </c>
+      <c r="K9">
+        <f>Debt!K23</f>
+        <v>7035628.6509542381</v>
+      </c>
+      <c r="L9">
+        <f>Debt!L23</f>
+        <v>7087894.8329465538</v>
+      </c>
+      <c r="M9">
+        <f>Debt!M23</f>
+        <v>6519294.2585427156</v>
+      </c>
+      <c r="N9">
+        <f>Debt!N23</f>
+        <v>6556724.6718051899</v>
+      </c>
+      <c r="O9">
+        <f>Debt!O23</f>
+        <v>5972704.4685206041</v>
+      </c>
+      <c r="P9">
+        <f>Debt!P23</f>
+        <v>5994082.3129534516</v>
+      </c>
+      <c r="Q9">
+        <f>Debt!Q23</f>
+        <v>5393372.3674196713</v>
+      </c>
+      <c r="R9">
+        <f>Debt!R23</f>
+        <v>5397395.0003370903</v>
+      </c>
+      <c r="S9">
+        <f>Debt!S23</f>
+        <v>4778635.7536132121</v>
+      </c>
+      <c r="T9">
+        <f>Debt!T23</f>
+        <v>4763884.1461216509</v>
+      </c>
+      <c r="U9">
+        <f>Debt!U23</f>
+        <v>4125594.4497094513</v>
+      </c>
+      <c r="V9">
+        <f>Debt!V23</f>
+        <v>4090547.6331754318</v>
+      </c>
+      <c r="W9">
+        <f>Debt!W23</f>
+        <v>3431140.0964031969</v>
+      </c>
+      <c r="X9">
+        <f>Debt!X23</f>
+        <v>3374091.1037357366</v>
+      </c>
+      <c r="Y9">
+        <f>Debt!Y23</f>
+        <v>2691783.5076570492</v>
+      </c>
+      <c r="Z9">
+        <f>Debt!Z23</f>
+        <v>2610896.5757979504</v>
+      </c>
+      <c r="AA9">
+        <f>Debt!AA23</f>
+        <v>1903772.3910371712</v>
+      </c>
+      <c r="AB9">
+        <f>Debt!AB23</f>
+        <v>1797046.5979640391</v>
+      </c>
+      <c r="AC9">
+        <f>Debt!AC23</f>
+        <v>1063016.7408628659</v>
+      </c>
+      <c r="AD9">
+        <f>Debt!AD23</f>
+        <v>928298.0374823293</v>
+      </c>
+      <c r="AE9">
+        <f>Debt!AE23</f>
+        <v>165113.71492921771</v>
+      </c>
+      <c r="AF9">
+        <f>Debt!AF23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AG9">
+        <f>Debt!AG23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AH9">
+        <f>Debt!AH23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AI9">
+        <f>Debt!AI23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AJ9">
+        <f>Debt!AJ23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AK9">
+        <f>Debt!AK23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AL9">
+        <f>Debt!AL23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AM9">
+        <f>Debt!AM23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AN9">
+        <f>Debt!AN23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AO9">
+        <f>Debt!AO23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AP9">
+        <f>Debt!AP23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AQ9">
+        <f>Debt!AQ23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AR9">
+        <f>Debt!AR23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AS9">
+        <f>Debt!AS23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AT9">
+        <f>Debt!AT23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AU9">
+        <f>Debt!AU23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AV9">
+        <f>Debt!AV23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AW9">
+        <f>Debt!AW23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AX9">
+        <f>Debt!AX23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AY9">
+        <f>Debt!AY23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="AZ9">
+        <f>Debt!AZ23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BA9">
+        <f>Debt!BA23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BB9">
+        <f>Debt!BB23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BC9">
+        <f>Debt!BC23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BD9">
+        <f>Debt!BD23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BE9">
+        <f>Debt!BE23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BF9">
+        <f>Debt!BF23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BG9">
+        <f>Debt!BG23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BH9">
+        <f>Debt!BH23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BI9">
+        <f>Debt!BI23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BJ9">
+        <f>Debt!BJ23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BK9">
+        <f>Debt!BK23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BL9">
+        <f>Debt!BL23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BM9">
+        <f>Debt!BM23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BN9">
+        <f>Debt!BN23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BO9">
+        <f>Debt!BO23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BP9">
+        <f>Debt!BP23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BQ9">
+        <f>Debt!BQ23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BR9">
+        <f>Debt!BR23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BS9">
+        <f>Debt!BS23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BT9">
+        <f>Debt!BT23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+      <c r="BU9">
+        <f>Debt!BU23</f>
+        <v>2.7066562324762344E-8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:73">
+      <c r="A10" t="str">
+        <f>Cashflow!A25</f>
+        <v>12-month DSCR</v>
+      </c>
+      <c r="B10" t="str">
+        <f>Cashflow!B25</f>
+        <v>x</v>
+      </c>
+      <c r="C10">
+        <f>Cashflow!C25</f>
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <f>Cashflow!D25</f>
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <f>Cashflow!E25</f>
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <f>Cashflow!F25</f>
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <f>Cashflow!G25</f>
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <f>Cashflow!H25</f>
+        <v>1.35</v>
+      </c>
+      <c r="I10">
+        <f>Cashflow!I25</f>
+        <v>1.35</v>
+      </c>
+      <c r="J10">
+        <f>Cashflow!J25</f>
+        <v>1.35</v>
+      </c>
+      <c r="K10">
+        <f>Cashflow!K25</f>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="L10">
+        <f>Cashflow!L25</f>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="M10">
+        <f>Cashflow!M25</f>
+        <v>1.35</v>
+      </c>
+      <c r="N10">
+        <f>Cashflow!N25</f>
+        <v>1.35</v>
+      </c>
+      <c r="O10">
+        <f>Cashflow!O25</f>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="P10">
+        <f>Cashflow!P25</f>
+        <v>1.35</v>
+      </c>
+      <c r="Q10">
+        <f>Cashflow!Q25</f>
+        <v>1.35</v>
+      </c>
+      <c r="R10">
+        <f>Cashflow!R25</f>
+        <v>1.3499999999999999</v>
+      </c>
+      <c r="S10">
+        <f>Cashflow!S25</f>
+        <v>1.3499999999999999</v>
+      </c>
+      <c r="T10">
+        <f>Cashflow!T25</f>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="U10">
+        <f>Cashflow!U25</f>
+        <v>1.3499999999999999</v>
+      </c>
+      <c r="V10">
+        <f>Cashflow!V25</f>
+        <v>1.3499999999999999</v>
+      </c>
+      <c r="W10">
+        <f>Cashflow!W25</f>
+        <v>1.3499999999999999</v>
+      </c>
+      <c r="X10">
+        <f>Cashflow!X25</f>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="Y10">
+        <f>Cashflow!Y25</f>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="Z10">
+        <f>Cashflow!Z25</f>
+        <v>1.35</v>
+      </c>
+      <c r="AA10">
+        <f>Cashflow!AA25</f>
+        <v>1.35</v>
+      </c>
+      <c r="AB10">
+        <f>Cashflow!AB25</f>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="AC10">
+        <f>Cashflow!AC25</f>
+        <v>1.35</v>
+      </c>
+      <c r="AD10">
+        <f>Cashflow!AD25</f>
+        <v>1.35</v>
+      </c>
+      <c r="AE10">
+        <f>Cashflow!AE25</f>
+        <v>1.35</v>
+      </c>
+      <c r="AF10">
+        <f>Cashflow!AF25</f>
+        <v>0</v>
+      </c>
+      <c r="AG10">
+        <f>Cashflow!AG25</f>
+        <v>0</v>
+      </c>
+      <c r="AH10">
+        <f>Cashflow!AH25</f>
+        <v>0</v>
+      </c>
+      <c r="AI10">
+        <f>Cashflow!AI25</f>
+        <v>0</v>
+      </c>
+      <c r="AJ10">
+        <f>Cashflow!AJ25</f>
+        <v>0</v>
+      </c>
+      <c r="AK10">
+        <f>Cashflow!AK25</f>
+        <v>0</v>
+      </c>
+      <c r="AL10">
+        <f>Cashflow!AL25</f>
+        <v>0</v>
+      </c>
+      <c r="AM10">
+        <f>Cashflow!AM25</f>
+        <v>0</v>
+      </c>
+      <c r="AN10">
+        <f>Cashflow!AN25</f>
+        <v>0</v>
+      </c>
+      <c r="AO10">
+        <f>Cashflow!AO25</f>
+        <v>0</v>
+      </c>
+      <c r="AP10">
+        <f>Cashflow!AP25</f>
+        <v>0</v>
+      </c>
+      <c r="AQ10">
+        <f>Cashflow!AQ25</f>
+        <v>0</v>
+      </c>
+      <c r="AR10">
+        <f>Cashflow!AR25</f>
+        <v>0</v>
+      </c>
+      <c r="AS10">
+        <f>Cashflow!AS25</f>
+        <v>0</v>
+      </c>
+      <c r="AT10">
+        <f>Cashflow!AT25</f>
+        <v>0</v>
+      </c>
+      <c r="AU10">
+        <f>Cashflow!AU25</f>
+        <v>0</v>
+      </c>
+      <c r="AV10">
+        <f>Cashflow!AV25</f>
+        <v>0</v>
+      </c>
+      <c r="AW10">
+        <f>Cashflow!AW25</f>
+        <v>0</v>
+      </c>
+      <c r="AX10">
+        <f>Cashflow!AX25</f>
+        <v>0</v>
+      </c>
+      <c r="AY10">
+        <f>Cashflow!AY25</f>
+        <v>0</v>
+      </c>
+      <c r="AZ10">
+        <f>Cashflow!AZ25</f>
+        <v>0</v>
+      </c>
+      <c r="BA10">
+        <f>Cashflow!BA25</f>
+        <v>0</v>
+      </c>
+      <c r="BB10">
+        <f>Cashflow!BB25</f>
+        <v>0</v>
+      </c>
+      <c r="BC10">
+        <f>Cashflow!BC25</f>
+        <v>0</v>
+      </c>
+      <c r="BD10">
+        <f>Cashflow!BD25</f>
+        <v>0</v>
+      </c>
+      <c r="BE10">
+        <f>Cashflow!BE25</f>
+        <v>0</v>
+      </c>
+      <c r="BF10">
+        <f>Cashflow!BF25</f>
+        <v>0</v>
+      </c>
+      <c r="BG10">
+        <f>Cashflow!BG25</f>
+        <v>0</v>
+      </c>
+      <c r="BH10">
+        <f>Cashflow!BH25</f>
+        <v>0</v>
+      </c>
+      <c r="BI10">
+        <f>Cashflow!BI25</f>
+        <v>0</v>
+      </c>
+      <c r="BJ10">
+        <f>Cashflow!BJ25</f>
+        <v>0</v>
+      </c>
+      <c r="BK10">
+        <f>Cashflow!BK25</f>
+        <v>0</v>
+      </c>
+      <c r="BL10">
+        <f>Cashflow!BL25</f>
+        <v>0</v>
+      </c>
+      <c r="BM10">
+        <f>Cashflow!BM25</f>
+        <v>0</v>
+      </c>
+      <c r="BN10">
+        <f>Cashflow!BN25</f>
+        <v>0</v>
+      </c>
+      <c r="BO10">
+        <f>Cashflow!BO25</f>
+        <v>0</v>
+      </c>
+      <c r="BP10">
+        <f>Cashflow!BP25</f>
+        <v>0</v>
+      </c>
+      <c r="BQ10">
+        <f>Cashflow!BQ25</f>
+        <v>0</v>
+      </c>
+      <c r="BR10">
+        <f>Cashflow!BR25</f>
+        <v>0</v>
+      </c>
+      <c r="BS10">
+        <f>Cashflow!BS25</f>
+        <v>0</v>
+      </c>
+      <c r="BT10">
+        <f>Cashflow!BT25</f>
+        <v>0</v>
+      </c>
+      <c r="BU10">
+        <f>Cashflow!BU25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:73">
+      <c r="A11" t="s">
+        <v>327</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11">
+        <f>IF(D6=1,D7/D8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <f t="shared" ref="E11:BP11" si="0">IF(E6=1,E7/E8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="0"/>
+        <v>1.3500000000000003</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="V11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="W11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="X11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="Y11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="Z11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="AA11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="AB11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="AC11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="AE11">
+        <f t="shared" si="0"/>
+        <v>1.35</v>
+      </c>
+      <c r="AF11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AG11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AH11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AI11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AJ11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AK11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AL11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AM11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AN11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AO11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AP11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AQ11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AR11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AS11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AT11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AU11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AV11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AW11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AX11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AY11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AZ11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BA11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BB11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BC11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BD11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BE11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BF11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BG11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BH11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BI11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BJ11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BK11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BL11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BM11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BN11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BO11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BP11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="BQ11">
+        <f t="shared" ref="BQ11:BU11" si="1">IF(BQ6=1,BQ7/BQ8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BS11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BT11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="BU11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:73">
+      <c r="A12" t="s">
+        <v>328</v>
+      </c>
+      <c r="B12" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12">
+        <f>(D7*D6+E12)/(1+Inputs!$B$43)</f>
+        <v>9130003.8543221671</v>
+      </c>
+      <c r="E12">
+        <f>(E7*E6+F12)/(1+Inputs!$B$43)</f>
+        <v>9540854.0277666636</v>
+      </c>
+      <c r="F12">
+        <f>(F7*F6+G12)/(1+Inputs!$B$43)</f>
+        <v>9970192.4590161629</v>
+      </c>
+      <c r="G12">
+        <f>(G7*G6+H12)/(1+Inputs!$B$43)</f>
+        <v>10418851.119671889</v>
+      </c>
+      <c r="H12">
+        <f>(H7*H6+I12)/(1+Inputs!$B$43)</f>
+        <v>10887699.420057124</v>
+      </c>
+      <c r="I12">
+        <f>(I7*I6+J12)/(1+Inputs!$B$43)</f>
+        <v>10157271.485025162</v>
+      </c>
+      <c r="J12">
+        <f>(J7*J6+K12)/(1+Inputs!$B$43)</f>
+        <v>10246407.439030318</v>
+      </c>
+      <c r="K12">
+        <f>(K7*K6+L12)/(1+Inputs!$B$43)</f>
+        <v>9498098.6787882131</v>
+      </c>
+      <c r="L12">
+        <f>(L7*L6+M12)/(1+Inputs!$B$43)</f>
+        <v>9568658.0244778376</v>
+      </c>
+      <c r="M12">
+        <f>(M7*M6+N12)/(1+Inputs!$B$43)</f>
+        <v>8801047.2490326557</v>
+      </c>
+      <c r="N12">
+        <f>(N7*N6+O12)/(1+Inputs!$B$43)</f>
+        <v>8851578.3069369942</v>
+      </c>
+      <c r="O12">
+        <f>(O7*O6+P12)/(1+Inputs!$B$43)</f>
+        <v>8063151.0325028021</v>
+      </c>
+      <c r="P12">
+        <f>(P7*P6+Q12)/(1+Inputs!$B$43)</f>
+        <v>8092011.1224871455</v>
+      </c>
+      <c r="Q12">
+        <f>(Q7*Q6+R12)/(1+Inputs!$B$43)</f>
+        <v>7281052.6960165417</v>
+      </c>
+      <c r="R12">
+        <f>(R7*R6+S12)/(1+Inputs!$B$43)</f>
+        <v>7286483.2504550563</v>
+      </c>
+      <c r="S12">
+        <f>(S7*S6+T12)/(1+Inputs!$B$43)</f>
+        <v>6451158.2673778199</v>
+      </c>
+      <c r="T12">
+        <f>(T7*T6+U12)/(1+Inputs!$B$43)</f>
+        <v>6431243.5972642116</v>
+      </c>
+      <c r="U12">
+        <f>(U7*U6+V12)/(1+Inputs!$B$43)</f>
+        <v>5569552.5071077403</v>
+      </c>
+      <c r="V12">
+        <f>(V7*V6+W12)/(1+Inputs!$B$43)</f>
+        <v>5522239.3047868125</v>
+      </c>
+      <c r="W12">
+        <f>(W7*W6+X12)/(1+Inputs!$B$43)</f>
+        <v>4632039.1301442934</v>
+      </c>
+      <c r="X12">
+        <f>(X7*X6+Y12)/(1+Inputs!$B$43)</f>
+        <v>4555022.9900432201</v>
+      </c>
+      <c r="Y12">
+        <f>(Y7*Y6+Z12)/(1+Inputs!$B$43)</f>
+        <v>3633907.735336991</v>
+      </c>
+      <c r="Z12">
+        <f>(Z7*Z6+AA12)/(1+Inputs!$B$43)</f>
+        <v>3524710.3773272061</v>
+      </c>
+      <c r="AA12">
+        <f>(AA7*AA6+AB12)/(1+Inputs!$B$43)</f>
+        <v>2570092.7279001526</v>
+      </c>
+      <c r="AB12">
+        <f>(AB7*AB6+AC12)/(1+Inputs!$B$43)</f>
+        <v>2426012.9072514228</v>
+      </c>
+      <c r="AC12">
+        <f>(AC7*AC6+AD12)/(1+Inputs!$B$43)</f>
+        <v>1435072.6001648374</v>
+      </c>
+      <c r="AD12">
+        <f>(AD7*AD6+AE12)/(1+Inputs!$B$43)</f>
+        <v>1253202.3506011113</v>
+      </c>
+      <c r="AE12">
+        <f>(AE7*AE6+AF12)/(1+Inputs!$B$43)</f>
+        <v>222903.51515440896</v>
+      </c>
+      <c r="AF12">
+        <f>(AF7*AF6+AG12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AG12">
+        <f>(AG7*AG6+AH12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AH12">
+        <f>(AH7*AH6+AI12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AI12">
+        <f>(AI7*AI6+AJ12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ12">
+        <f>(AJ7*AJ6+AK12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AK12">
+        <f>(AK7*AK6+AL12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AL12">
+        <f>(AL7*AL6+AM12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AM12">
+        <f>(AM7*AM6+AN12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AN12">
+        <f>(AN7*AN6+AO12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AO12">
+        <f>(AO7*AO6+AP12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AP12">
+        <f>(AP7*AP6+AQ12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AQ12">
+        <f>(AQ7*AQ6+AR12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AR12">
+        <f>(AR7*AR6+AS12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AS12">
+        <f>(AS7*AS6+AT12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AT12">
+        <f>(AT7*AT6+AU12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AU12">
+        <f>(AU7*AU6+AV12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AV12">
+        <f>(AV7*AV6+AW12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AW12">
+        <f>(AW7*AW6+AX12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AX12">
+        <f>(AX7*AX6+AY12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AY12">
+        <f>(AY7*AY6+AZ12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ12">
+        <f>(AZ7*AZ6+BA12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BA12">
+        <f>(BA7*BA6+BB12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BB12">
+        <f>(BB7*BB6+BC12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BC12">
+        <f>(BC7*BC6+BD12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BD12">
+        <f>(BD7*BD6+BE12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BE12">
+        <f>(BE7*BE6+BF12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BF12">
+        <f>(BF7*BF6+BG12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BG12">
+        <f>(BG7*BG6+BH12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BH12">
+        <f>(BH7*BH6+BI12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BI12">
+        <f>(BI7*BI6+BJ12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BJ12">
+        <f>(BJ7*BJ6+BK12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BK12">
+        <f>(BK7*BK6+BL12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BL12">
+        <f>(BL7*BL6+BM12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BM12">
+        <f>(BM7*BM6+BN12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BN12">
+        <f>(BN7*BN6+BO12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BO12">
+        <f>(BO7*BO6+BP12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BP12">
+        <f>(BP7*BP6+BQ12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BQ12">
+        <f>(BQ7*BQ6+BR12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BR12">
+        <f>(BR7*BR6+BS12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BS12">
+        <f>(BS7*BS6+BT12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BT12">
+        <f>(BT7*BT6+BU12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+      <c r="BU12">
+        <f>(BU7*BU6+BV12)/(1+Inputs!$B$43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:73">
+      <c r="A13" t="s">
+        <v>329</v>
+      </c>
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13">
+        <f>IF(D6=1,D12/D9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <f t="shared" ref="E13:BP13" si="2">IF(E6=1,E12/E9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999994</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999992</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999992</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999988</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999985</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999983</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999981</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999976</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999976</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999972</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999972</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999965</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999963</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999954</v>
+      </c>
+      <c r="V13">
+        <f t="shared" si="2"/>
+        <v>1.349999999999995</v>
+      </c>
+      <c r="W13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999934</v>
+      </c>
+      <c r="X13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999928</v>
+      </c>
+      <c r="Y13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999905</v>
+      </c>
+      <c r="Z13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999897</v>
+      </c>
+      <c r="AA13">
+        <f t="shared" si="2"/>
+        <v>1.349999999999985</v>
+      </c>
+      <c r="AB13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999832</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999703</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999999641</v>
+      </c>
+      <c r="AE13">
+        <f t="shared" si="2"/>
+        <v>1.3499999999997885</v>
+      </c>
+      <c r="AF13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AG13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AJ13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AK13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AL13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AM13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AN13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AO13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AP13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AQ13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AR13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AS13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AT13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AU13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AV13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AW13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AX13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AY13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AZ13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BA13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BB13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BC13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BD13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BE13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BF13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BG13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BH13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BI13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BJ13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BK13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BL13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BM13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BN13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BO13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BP13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="BQ13">
+        <f t="shared" ref="BQ13:BU13" si="3">IF(BQ6=1,BQ12/BQ9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BR13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="BS13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="BT13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="BU13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:73">
+      <c r="A14" t="s">
+        <v>344</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14">
+        <f>_xlfn.AGGREGATE(15,6,D11:BU11/(D6:BU6=1),1)</f>
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:73">
+      <c r="A15" t="s">
+        <v>330</v>
+      </c>
+      <c r="B15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15">
+        <f>_xlfn.AGGREGATE(15,6,D10:BU10/(D6:BU6=1),1)</f>
+        <v>1.3499999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:73">
+      <c r="A16" t="s">
+        <v>331</v>
+      </c>
+      <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="57">
+        <f>_xlfn.AGGREGATE(15,6,D13:BU13/(D6:BU6=1),1)</f>
+        <v>1.3499999999997885</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>334</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17">
+        <f>AVERAGEIF(D6:BU6,1,D11:BU11)</f>
+        <v>1.3500000000000005</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75">
+      <c r="A18" s="58" t="s">
+        <v>239</v>
+      </c>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>332</v>
+      </c>
+      <c r="B19" t="s">
+        <v>165</v>
+      </c>
+      <c r="C19">
+        <f>IF(ABS(H13-Inputs!$B$45)&lt;0.0001,0,1)</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A18:C18"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:BU12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75">
+    <row r="1" spans="1:73" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:73">
       <c r="A2" t="s">
         <v>63</v>
       </c>
     </row>
+    <row r="4" spans="1:73" ht="15.75">
+      <c r="A4" s="58" t="s">
+        <v>343</v>
+      </c>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+    </row>
+    <row r="5" spans="1:73">
+      <c r="A5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" t="s">
+        <v>340</v>
+      </c>
+      <c r="C5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="6" spans="1:73">
+      <c r="A6" t="s">
+        <v>335</v>
+      </c>
+      <c r="B6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C6">
+        <f>SUM(D6:BU6)</f>
+        <v>-3089872.6500542867</v>
+      </c>
+      <c r="D6">
+        <f>Debt!D8 - Construction!D18</f>
+        <v>-5279031.8900696263</v>
+      </c>
+      <c r="E6">
+        <f>Debt!E8 - Construction!E18</f>
+        <v>-12440561.612956891</v>
+      </c>
+      <c r="F6">
+        <f>Debt!F8 - Construction!F18</f>
+        <v>-12564606.796039043</v>
+      </c>
+      <c r="G6">
+        <f>Debt!G8 - Construction!G18</f>
+        <v>-5438228.9368267804</v>
+      </c>
+      <c r="H6">
+        <f>Debt!H8 - Construction!H18</f>
+        <v>1220374.4089345317</v>
+      </c>
+      <c r="I6">
+        <f>Debt!I8 - Construction!I18</f>
+        <v>367941.26282097551</v>
+      </c>
+      <c r="J6">
+        <f>Debt!J8 - Construction!J18</f>
+        <v>1209397.0949984677</v>
+      </c>
+      <c r="K6">
+        <f>Debt!K8 - Construction!K18</f>
+        <v>356855.09485584439</v>
+      </c>
+      <c r="L6">
+        <f>Debt!L8 - Construction!L18</f>
+        <v>1198200.3865466854</v>
+      </c>
+      <c r="M6">
+        <f>Debt!M8 - Construction!M18</f>
+        <v>345516.06830213021</v>
+      </c>
+      <c r="N6">
+        <f>Debt!N8 - Construction!N18</f>
+        <v>1186748.2982463562</v>
+      </c>
+      <c r="O6">
+        <f>Debt!O8 - Construction!O18</f>
+        <v>333981.70647828188</v>
+      </c>
+      <c r="P6">
+        <f>Debt!P8 - Construction!P18</f>
+        <v>1175098.9269825253</v>
+      </c>
+      <c r="Q6">
+        <f>Debt!Q8 - Construction!Q18</f>
+        <v>322216.81688222941</v>
+      </c>
+      <c r="R6">
+        <f>Debt!R8 - Construction!R18</f>
+        <v>1163216.7293477135</v>
+      </c>
+      <c r="S6">
+        <f>Debt!S8 - Construction!S18</f>
+        <v>310216.79214560974</v>
+      </c>
+      <c r="T6">
+        <f>Debt!T8 - Construction!T18</f>
+        <v>1151097.0520333601</v>
+      </c>
+      <c r="U6">
+        <f>Debt!U8 - Construction!U18</f>
+        <v>297943.06514077552</v>
+      </c>
+      <c r="V6">
+        <f>Debt!V8 - Construction!V18</f>
+        <v>1138700.9433579245</v>
+      </c>
+      <c r="W6">
+        <f>Debt!W8 - Construction!W18</f>
+        <v>285457.90095756587</v>
+      </c>
+      <c r="X6">
+        <f>Debt!X8 - Construction!X18</f>
+        <v>1126091.2892581739</v>
+      </c>
+      <c r="Y6">
+        <f>Debt!Y8 - Construction!Y18</f>
+        <v>272723.20609994943</v>
+      </c>
+      <c r="Z6">
+        <f>Debt!Z8 - Construction!Z18</f>
+        <v>1113229.6164067774</v>
+      </c>
+      <c r="AA6">
+        <f>Debt!AA8 - Construction!AA18</f>
+        <v>259733.99340423674</v>
+      </c>
+      <c r="AB6">
+        <f>Debt!AB8 - Construction!AB18</f>
+        <v>1100110.887912899</v>
+      </c>
+      <c r="AC6">
+        <f>Debt!AC8 - Construction!AC18</f>
+        <v>246448.51657114364</v>
+      </c>
+      <c r="AD6">
+        <f>Debt!AD8 - Construction!AD18</f>
+        <v>1086692.9412237522</v>
+      </c>
+      <c r="AE6">
+        <f>Debt!AE8 - Construction!AE18</f>
+        <v>232934.17333635734</v>
+      </c>
+      <c r="AF6">
+        <f>Debt!AF8 - Construction!AF18</f>
+        <v>1073043.8460997068</v>
+      </c>
+      <c r="AG6">
+        <f>Debt!AG8 - Construction!AG18</f>
+        <v>219149.7300746867</v>
+      </c>
+      <c r="AH6">
+        <f>Debt!AH8 - Construction!AH18</f>
+        <v>1059121.9577739565</v>
+      </c>
+      <c r="AI6">
+        <f>Debt!AI8 - Construction!AI18</f>
+        <v>205089.788519767</v>
+      </c>
+      <c r="AJ6">
+        <f>Debt!AJ8 - Construction!AJ18</f>
+        <v>1044921.824153874</v>
+      </c>
+      <c r="AK6">
+        <f>Debt!AK8 - Construction!AK18</f>
+        <v>190709.16113469214</v>
+      </c>
+      <c r="AL6">
+        <f>Debt!AL8 - Construction!AL18</f>
+        <v>732272.82580145611</v>
+      </c>
+      <c r="AM6">
+        <f>Debt!AM8 - Construction!AM18</f>
+        <v>176080.80139608099</v>
+      </c>
+      <c r="AN6">
+        <f>Debt!AN8 - Construction!AN18</f>
+        <v>723555.55378948129</v>
+      </c>
+      <c r="AO6">
+        <f>Debt!AO8 - Construction!AO18</f>
+        <v>161160.07670195331</v>
+      </c>
+      <c r="AP6">
+        <f>Debt!AP8 - Construction!AP18</f>
+        <v>718982.63265880744</v>
+      </c>
+      <c r="AQ6">
+        <f>Debt!AQ8 - Construction!AQ18</f>
+        <v>145941.14379518793</v>
+      </c>
+      <c r="AR6">
+        <f>Debt!AR8 - Construction!AR18</f>
+        <v>714318.31632683706</v>
+      </c>
+      <c r="AS6">
+        <f>Debt!AS8 - Construction!AS18</f>
+        <v>130375.09023260616</v>
+      </c>
+      <c r="AT6">
+        <f>Debt!AT8 - Construction!AT18</f>
+        <v>709547.61405085807</v>
+      </c>
+      <c r="AU6">
+        <f>Debt!AU8 - Construction!AU18</f>
+        <v>114540.88320348423</v>
+      </c>
+      <c r="AV6">
+        <f>Debt!AV8 - Construction!AV18</f>
+        <v>704694.72778726846</v>
+      </c>
+      <c r="AW6">
+        <f>Debt!AW8 - Construction!AW18</f>
+        <v>98390.210944054183</v>
+      </c>
+      <c r="AX6">
+        <f>Debt!AX8 - Construction!AX18</f>
+        <v>699744.85089028359</v>
+      </c>
+      <c r="AY6">
+        <f>Debt!AY8 - Construction!AY18</f>
+        <v>81916.748524889117</v>
+      </c>
+      <c r="AZ6">
+        <f>Debt!AZ8 - Construction!AZ18</f>
+        <v>694696.04488814552</v>
+      </c>
+      <c r="BA6">
+        <f>Debt!BA8 - Construction!BA18</f>
+        <v>65067.551544468035</v>
+      </c>
+      <c r="BB6">
+        <f>Debt!BB8 - Construction!BB18</f>
+        <v>689532.08331884071</v>
+      </c>
+      <c r="BC6">
+        <f>Debt!BC8 - Construction!BC18</f>
+        <v>47928.096628048341</v>
+      </c>
+      <c r="BD6">
+        <f>Debt!BD8 - Construction!BD18</f>
+        <v>684279.16315830906</v>
+      </c>
+      <c r="BE6">
+        <f>Debt!BE8 - Construction!BE18</f>
+        <v>30446.089568821597</v>
+      </c>
+      <c r="BF6">
+        <f>Debt!BF8 - Construction!BF18</f>
+        <v>678921.2572169716</v>
+      </c>
+      <c r="BG6">
+        <f>Debt!BG8 - Construction!BG18</f>
+        <v>12614.684059765772</v>
+      </c>
+      <c r="BH6">
+        <f>Debt!BH8 - Construction!BH18</f>
+        <v>673456.26723065635</v>
+      </c>
+      <c r="BI6">
+        <f>Debt!BI8 - Construction!BI18</f>
+        <v>-5623.4286220169161</v>
+      </c>
+      <c r="BJ6">
+        <f>Debt!BJ8 - Construction!BJ18</f>
+        <v>667866.62915503676</v>
+      </c>
+      <c r="BK6">
+        <f>Debt!BK8 - Construction!BK18</f>
+        <v>-24175.725828419672</v>
+      </c>
+      <c r="BL6">
+        <f>Debt!BL8 - Construction!BL18</f>
+        <v>662180.69943936495</v>
+      </c>
+      <c r="BM6">
+        <f>Debt!BM8 - Construction!BM18</f>
+        <v>-43098.812490673736</v>
+      </c>
+      <c r="BN6">
+        <f>Debt!BN8 - Construction!BN18</f>
+        <v>656381.12973820628</v>
+      </c>
+      <c r="BO6">
+        <f>Debt!BO8 - Construction!BO18</f>
+        <v>-62400.099271676852</v>
+      </c>
+      <c r="BP6">
+        <f>Debt!BP8 - Construction!BP18</f>
+        <v>0</v>
+      </c>
+      <c r="BQ6">
+        <f>Debt!BQ8 - Construction!BQ18</f>
+        <v>0</v>
+      </c>
+      <c r="BR6">
+        <f>Debt!BR8 - Construction!BR18</f>
+        <v>0</v>
+      </c>
+      <c r="BS6">
+        <f>Debt!BS8 - Construction!BS18</f>
+        <v>0</v>
+      </c>
+      <c r="BT6">
+        <f>Debt!BT8 - Construction!BT18</f>
+        <v>0</v>
+      </c>
+      <c r="BU6">
+        <f>Debt!BU8 - Construction!BU18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:73">
+      <c r="A7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C7">
+        <f>SUM(D7:BU7)</f>
+        <v>-8872819.3669456635</v>
+      </c>
+      <c r="D7">
+        <f>Cashflow!D31 - Construction!D44</f>
+        <v>-4253661.5170582291</v>
+      </c>
+      <c r="E7">
+        <f>Cashflow!E31 - Construction!E44</f>
+        <v>-9762387.1338366754</v>
+      </c>
+      <c r="F7">
+        <f>Cashflow!F31 - Construction!F44</f>
+        <v>-9978390.7146649472</v>
+      </c>
+      <c r="G7">
+        <f>Cashflow!G31 - Construction!G44</f>
+        <v>-5135551.893619027</v>
+      </c>
+      <c r="H7">
+        <f>Cashflow!H31 - Construction!H44</f>
+        <v>320459.03710749489</v>
+      </c>
+      <c r="I7">
+        <f>Cashflow!I31 - Construction!I44</f>
+        <v>99498.167385116336</v>
+      </c>
+      <c r="J7">
+        <f>Cashflow!J31 - Construction!J44</f>
+        <v>317694.32405581849</v>
+      </c>
+      <c r="K7">
+        <f>Cashflow!K31 - Construction!K44</f>
+        <v>96717.627019557462</v>
+      </c>
+      <c r="L7">
+        <f>Cashflow!L31 - Construction!L44</f>
+        <v>314886.0588455589</v>
+      </c>
+      <c r="M7">
+        <f>Cashflow!M31 - Construction!M44</f>
+        <v>93850.225790866563</v>
+      </c>
+      <c r="N7">
+        <f>Cashflow!N31 - Construction!N44</f>
+        <v>311990.06668010377</v>
+      </c>
+      <c r="O7">
+        <f>Cashflow!O31 - Construction!O44</f>
+        <v>90945.216344759217</v>
+      </c>
+      <c r="P7">
+        <f>Cashflow!P31 - Construction!P44</f>
+        <v>309056.09130465903</v>
+      </c>
+      <c r="Q7">
+        <f>Cashflow!Q31 - Construction!Q44</f>
+        <v>87982.146871918667</v>
+      </c>
+      <c r="R7">
+        <f>Cashflow!R31 - Construction!R44</f>
+        <v>306063.47698435304</v>
+      </c>
+      <c r="S7">
+        <f>Cashflow!S31 - Construction!S44</f>
+        <v>84972.400558059599</v>
+      </c>
+      <c r="T7">
+        <f>Cashflow!T31 - Construction!T44</f>
+        <v>303023.72040695848</v>
+      </c>
+      <c r="U7">
+        <f>Cashflow!U31 - Construction!U44</f>
+        <v>81868.633252500964</v>
+      </c>
+      <c r="V7">
+        <f>Cashflow!V31 - Construction!V44</f>
+        <v>299889.00535196217</v>
+      </c>
+      <c r="W7">
+        <f>Cashflow!W31 - Construction!W44</f>
+        <v>78724.157602930645</v>
+      </c>
+      <c r="X7">
+        <f>Cashflow!X31 - Construction!X44</f>
+        <v>296713.17604893271</v>
+      </c>
+      <c r="Y7">
+        <f>Cashflow!Y31 - Construction!Y44</f>
+        <v>75516.83591321393</v>
+      </c>
+      <c r="Z7">
+        <f>Cashflow!Z31 - Construction!Z44</f>
+        <v>293473.87406615645</v>
+      </c>
+      <c r="AA7">
+        <f>Cashflow!AA31 - Construction!AA44</f>
+        <v>72258.989709651389</v>
+      </c>
+      <c r="AB7">
+        <f>Cashflow!AB31 - Construction!AB44</f>
+        <v>290183.54378821346</v>
+      </c>
+      <c r="AC7">
+        <f>Cashflow!AC31 - Construction!AC44</f>
+        <v>68899.372160958155</v>
+      </c>
+      <c r="AD7">
+        <f>Cashflow!AD31 - Construction!AD44</f>
+        <v>684214.074103844</v>
+      </c>
+      <c r="AE7">
+        <f>Cashflow!AE31 - Construction!AE44</f>
+        <v>146662.2572858546</v>
+      </c>
+      <c r="AF7">
+        <f>Cashflow!AF31 - Construction!AF44</f>
+        <v>1073043.8460997068</v>
+      </c>
+      <c r="AG7">
+        <f>Cashflow!AG31 - Construction!AG44</f>
+        <v>219149.7300746867</v>
+      </c>
+      <c r="AH7">
+        <f>Cashflow!AH31 - Construction!AH44</f>
+        <v>1059121.9577739565</v>
+      </c>
+      <c r="AI7">
+        <f>Cashflow!AI31 - Construction!AI44</f>
+        <v>205089.788519767</v>
+      </c>
+      <c r="AJ7">
+        <f>Cashflow!AJ31 - Construction!AJ44</f>
+        <v>1044921.824153874</v>
+      </c>
+      <c r="AK7">
+        <f>Cashflow!AK31 - Construction!AK44</f>
+        <v>190709.16113469214</v>
+      </c>
+      <c r="AL7">
+        <f>Cashflow!AL31 - Construction!AL44</f>
+        <v>732272.82580145611</v>
+      </c>
+      <c r="AM7">
+        <f>Cashflow!AM31 - Construction!AM44</f>
+        <v>176080.80139608099</v>
+      </c>
+      <c r="AN7">
+        <f>Cashflow!AN31 - Construction!AN44</f>
+        <v>723555.55378948129</v>
+      </c>
+      <c r="AO7">
+        <f>Cashflow!AO31 - Construction!AO44</f>
+        <v>161160.07670195331</v>
+      </c>
+      <c r="AP7">
+        <f>Cashflow!AP31 - Construction!AP44</f>
+        <v>718982.63265880744</v>
+      </c>
+      <c r="AQ7">
+        <f>Cashflow!AQ31 - Construction!AQ44</f>
+        <v>145941.14379518793</v>
+      </c>
+      <c r="AR7">
+        <f>Cashflow!AR31 - Construction!AR44</f>
+        <v>714318.31632683706</v>
+      </c>
+      <c r="AS7">
+        <f>Cashflow!AS31 - Construction!AS44</f>
+        <v>130375.09023260616</v>
+      </c>
+      <c r="AT7">
+        <f>Cashflow!AT31 - Construction!AT44</f>
+        <v>709547.61405085807</v>
+      </c>
+      <c r="AU7">
+        <f>Cashflow!AU31 - Construction!AU44</f>
+        <v>114540.88320348423</v>
+      </c>
+      <c r="AV7">
+        <f>Cashflow!AV31 - Construction!AV44</f>
+        <v>704694.72778726846</v>
+      </c>
+      <c r="AW7">
+        <f>Cashflow!AW31 - Construction!AW44</f>
+        <v>98390.210944054183</v>
+      </c>
+      <c r="AX7">
+        <f>Cashflow!AX31 - Construction!AX44</f>
+        <v>699744.85089028359</v>
+      </c>
+      <c r="AY7">
+        <f>Cashflow!AY31 - Construction!AY44</f>
+        <v>81916.748524889117</v>
+      </c>
+      <c r="AZ7">
+        <f>Cashflow!AZ31 - Construction!AZ44</f>
+        <v>694696.04488814552</v>
+      </c>
+      <c r="BA7">
+        <f>Cashflow!BA31 - Construction!BA44</f>
+        <v>65067.551544468035</v>
+      </c>
+      <c r="BB7">
+        <f>Cashflow!BB31 - Construction!BB44</f>
+        <v>689532.08331884071</v>
+      </c>
+      <c r="BC7">
+        <f>Cashflow!BC31 - Construction!BC44</f>
+        <v>47928.096628048341</v>
+      </c>
+      <c r="BD7">
+        <f>Cashflow!BD31 - Construction!BD44</f>
+        <v>684279.16315830906</v>
+      </c>
+      <c r="BE7">
+        <f>Cashflow!BE31 - Construction!BE44</f>
+        <v>30446.089568821597</v>
+      </c>
+      <c r="BF7">
+        <f>Cashflow!BF31 - Construction!BF44</f>
+        <v>678921.2572169716</v>
+      </c>
+      <c r="BG7">
+        <f>Cashflow!BG31 - Construction!BG44</f>
+        <v>12614.684059765772</v>
+      </c>
+      <c r="BH7">
+        <f>Cashflow!BH31 - Construction!BH44</f>
+        <v>673456.26723065635</v>
+      </c>
+      <c r="BI7">
+        <f>Cashflow!BI31 - Construction!BI44</f>
+        <v>-5623.4286220169161</v>
+      </c>
+      <c r="BJ7">
+        <f>Cashflow!BJ31 - Construction!BJ44</f>
+        <v>667866.62915503676</v>
+      </c>
+      <c r="BK7">
+        <f>Cashflow!BK31 - Construction!BK44</f>
+        <v>-24175.725828419672</v>
+      </c>
+      <c r="BL7">
+        <f>Cashflow!BL31 - Construction!BL44</f>
+        <v>662180.69943936495</v>
+      </c>
+      <c r="BM7">
+        <f>Cashflow!BM31 - Construction!BM44</f>
+        <v>-43098.812490673736</v>
+      </c>
+      <c r="BN7">
+        <f>Cashflow!BN31 - Construction!BN44</f>
+        <v>656381.12973820628</v>
+      </c>
+      <c r="BO7">
+        <f>Cashflow!BO31 - Construction!BO44</f>
+        <v>-62400.099271676852</v>
+      </c>
+      <c r="BP7">
+        <f>Cashflow!BP31 - Construction!BP44</f>
+        <v>0</v>
+      </c>
+      <c r="BQ7">
+        <f>Cashflow!BQ31 - Construction!BQ44</f>
+        <v>0</v>
+      </c>
+      <c r="BR7">
+        <f>Cashflow!BR31 - Construction!BR44</f>
+        <v>0</v>
+      </c>
+      <c r="BS7">
+        <f>Cashflow!BS31 - Construction!BS44</f>
+        <v>0</v>
+      </c>
+      <c r="BT7">
+        <f>Cashflow!BT31 - Construction!BT44</f>
+        <v>0</v>
+      </c>
+      <c r="BU7">
+        <f>Cashflow!BU31 - Construction!BU44</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:73">
+      <c r="A8" t="s">
+        <v>337</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="46">
+        <f>IRR(D6:BU6)</f>
+        <v>-3.3800721831106495E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:73">
+      <c r="A9" t="s">
+        <v>338</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="46">
+        <f>(1+C8)^2-1</f>
+        <v>-6.7487194782582804E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:73">
+      <c r="A10" t="s">
+        <v>341</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="46">
+        <f>IRR(D7:BU7)</f>
+        <v>-1.016020490163716E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:73">
+      <c r="A11" t="s">
+        <v>342</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="46">
+        <f>(1+C10)^2-1</f>
+        <v>-2.0217180039631022E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:73">
+      <c r="A12" t="s">
+        <v>339</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="8">
+        <f>Cashflow!C31 / Construction!C56</f>
+        <v>0.695406040873774</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7521,11 +10668,11 @@
       </c>
     </row>
     <row r="5" spans="1:75" ht="15.75">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="58" t="s">
         <v>169</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
       <c r="D5" s="43"/>
       <c r="E5" s="43"/>
       <c r="F5" s="43"/>
@@ -7607,12 +10754,12 @@
       </c>
     </row>
     <row r="14" spans="1:75" ht="15.75">
-      <c r="A14" s="57" t="s">
+      <c r="A14" s="58" t="s">
         <v>170</v>
       </c>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
+      <c r="B14" s="58"/>
+      <c r="C14" s="58"/>
+      <c r="D14" s="58"/>
       <c r="E14" s="33"/>
       <c r="F14" s="33"/>
       <c r="G14" s="33"/>
@@ -10890,12 +14037,12 @@
       </c>
     </row>
     <row r="27" spans="1:73" ht="15.75">
-      <c r="A27" s="57" t="s">
+      <c r="A27" s="58" t="s">
         <v>171</v>
       </c>
-      <c r="B27" s="57"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
+      <c r="B27" s="58"/>
+      <c r="C27" s="58"/>
+      <c r="D27" s="58"/>
       <c r="E27" s="41"/>
       <c r="F27" s="41"/>
       <c r="G27" s="41"/>
@@ -11009,11 +14156,11 @@
       </c>
     </row>
     <row r="4" spans="1:74" ht="15.75">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="58" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="1:74">
       <c r="A5" t="s">
@@ -11902,11 +15049,11 @@
       <c r="BV8" s="8"/>
     </row>
     <row r="9" spans="1:74" ht="15.75">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="58" t="s">
         <v>193</v>
       </c>
-      <c r="B9" s="57"/>
-      <c r="C9" s="57"/>
+      <c r="B9" s="58"/>
+      <c r="C9" s="58"/>
     </row>
     <row r="10" spans="1:74">
       <c r="A10" t="s">
@@ -13963,12 +17110,12 @@
       </c>
     </row>
     <row r="19" spans="1:73" ht="15.75">
-      <c r="A19" s="57" t="s">
+      <c r="A19" s="58" t="s">
         <v>194</v>
       </c>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57"/>
-      <c r="D19" s="57"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="58"/>
     </row>
     <row r="20" spans="1:73">
       <c r="A20" t="s">
@@ -14001,11 +17148,11 @@
       </c>
     </row>
     <row r="24" spans="1:73" ht="15.75">
-      <c r="A24" s="57" t="s">
+      <c r="A24" s="58" t="s">
         <v>205</v>
       </c>
-      <c r="B24" s="57"/>
-      <c r="C24" s="57"/>
+      <c r="B24" s="58"/>
+      <c r="C24" s="58"/>
     </row>
     <row r="25" spans="1:73">
       <c r="A25" t="s">
@@ -15790,11 +18937,11 @@
       </c>
     </row>
     <row r="34" spans="1:73" ht="15.75">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="58" t="s">
         <v>206</v>
       </c>
-      <c r="B34" s="57"/>
-      <c r="C34" s="57"/>
+      <c r="B34" s="58"/>
+      <c r="C34" s="58"/>
     </row>
     <row r="35" spans="1:73">
       <c r="A35" t="s">
@@ -15827,11 +18974,11 @@
       </c>
     </row>
     <row r="37" spans="1:73" ht="15.75">
-      <c r="A37" s="57" t="s">
+      <c r="A37" s="58" t="s">
         <v>207</v>
       </c>
-      <c r="B37" s="57"/>
-      <c r="C37" s="57"/>
+      <c r="B37" s="58"/>
+      <c r="C37" s="58"/>
     </row>
     <row r="38" spans="1:73">
       <c r="A38" t="s">
@@ -17874,11 +21021,11 @@
       </c>
     </row>
     <row r="45" spans="1:73" ht="15.75">
-      <c r="A45" s="57" t="s">
+      <c r="A45" s="58" t="s">
         <v>215</v>
       </c>
-      <c r="B45" s="57"/>
-      <c r="C45" s="57"/>
+      <c r="B45" s="58"/>
+      <c r="C45" s="58"/>
     </row>
     <row r="46" spans="1:73">
       <c r="A46" t="s">
@@ -17977,11 +21124,11 @@
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.75">
-      <c r="A54" s="57" t="s">
+      <c r="A54" s="58" t="s">
         <v>216</v>
       </c>
-      <c r="B54" s="57"/>
-      <c r="C54" s="57"/>
+      <c r="B54" s="58"/>
+      <c r="C54" s="58"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
@@ -18044,11 +21191,11 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="15.75">
-      <c r="A61" s="57" t="s">
+      <c r="A61" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="B61" s="57"/>
-      <c r="C61" s="57"/>
+      <c r="B61" s="58"/>
+      <c r="C61" s="58"/>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
@@ -18173,11 +21320,11 @@
       </c>
     </row>
     <row r="4" spans="1:75" ht="15.75">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="58" t="s">
         <v>240</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="1:75">
       <c r="A5" t="s">
@@ -21003,11 +24150,11 @@
       </c>
     </row>
     <row r="18" spans="1:73" ht="15.75">
-      <c r="A18" s="57" t="s">
+      <c r="A18" s="58" t="s">
         <v>239</v>
       </c>
-      <c r="B18" s="57"/>
-      <c r="C18" s="57"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
     </row>
     <row r="19" spans="1:73">
       <c r="A19" t="s">
@@ -21040,11 +24187,11 @@
       </c>
     </row>
     <row r="21" spans="1:73" ht="15.75">
-      <c r="A21" s="57" t="s">
+      <c r="A21" s="58" t="s">
         <v>245</v>
       </c>
-      <c r="B21" s="57"/>
-      <c r="C21" s="57"/>
+      <c r="B21" s="58"/>
+      <c r="C21" s="58"/>
     </row>
     <row r="22" spans="1:73">
       <c r="A22" t="str">
@@ -23092,11 +26239,11 @@
       </c>
     </row>
     <row r="29" spans="1:73" ht="15.75">
-      <c r="A29" s="57" t="s">
+      <c r="A29" s="58" t="s">
         <v>206</v>
       </c>
-      <c r="B29" s="57"/>
-      <c r="C29" s="57"/>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
     </row>
     <row r="30" spans="1:73">
       <c r="A30" t="s">
@@ -23148,11 +26295,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="58" t="s">
         <v>255</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -25251,11 +28398,11 @@
       </c>
     </row>
     <row r="16" spans="1:73" ht="15.75">
-      <c r="A16" s="57" t="s">
+      <c r="A16" s="58" t="s">
         <v>239</v>
       </c>
-      <c r="B16" s="57"/>
-      <c r="C16" s="57"/>
+      <c r="B16" s="58"/>
+      <c r="C16" s="58"/>
     </row>
     <row r="17" spans="1:73" ht="30">
       <c r="A17" s="52" t="s">
@@ -25273,11 +28420,11 @@
       </c>
     </row>
     <row r="18" spans="1:73" ht="15.75">
-      <c r="A18" s="57" t="s">
+      <c r="A18" s="58" t="s">
         <v>257</v>
       </c>
-      <c r="B18" s="57"/>
-      <c r="C18" s="57"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
     </row>
     <row r="19" spans="1:73">
       <c r="A19" t="s">
@@ -29348,11 +32495,11 @@
       </c>
     </row>
     <row r="34" spans="1:73" ht="15.75">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="58" t="s">
         <v>206</v>
       </c>
-      <c r="B34" s="57"/>
-      <c r="C34" s="57"/>
+      <c r="B34" s="58"/>
+      <c r="C34" s="58"/>
     </row>
     <row r="35" spans="1:73">
       <c r="A35" t="s">
@@ -29421,11 +32568,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="58" t="s">
         <v>285</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -31836,11 +34983,11 @@
       </c>
     </row>
     <row r="19" spans="1:73" ht="15.75">
-      <c r="A19" s="57" t="s">
+      <c r="A19" s="58" t="s">
         <v>286</v>
       </c>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
     </row>
     <row r="20" spans="1:73">
       <c r="A20" t="s">
@@ -33321,11 +36468,11 @@
       </c>
     </row>
     <row r="28" spans="1:73" ht="15.75">
-      <c r="A28" s="57" t="s">
+      <c r="A28" s="58" t="s">
         <v>206</v>
       </c>
-      <c r="B28" s="57"/>
-      <c r="C28" s="57"/>
+      <c r="B28" s="58"/>
+      <c r="C28" s="58"/>
     </row>
     <row r="29" spans="1:73">
       <c r="A29" t="s">
@@ -33404,11 +36551,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="58" t="s">
         <v>310</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -37213,11 +40360,11 @@
       </c>
     </row>
     <row r="20" spans="1:73" ht="15.75">
-      <c r="A20" s="57" t="s">
+      <c r="A20" s="58" t="s">
         <v>239</v>
       </c>
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
+      <c r="B20" s="58"/>
+      <c r="C20" s="58"/>
     </row>
     <row r="21" spans="1:73">
       <c r="A21" t="s">
@@ -37244,11 +40391,11 @@
       </c>
     </row>
     <row r="23" spans="1:73" ht="15.75">
-      <c r="A23" s="57" t="s">
+      <c r="A23" s="58" t="s">
         <v>311</v>
       </c>
-      <c r="B23" s="57"/>
-      <c r="C23" s="57"/>
+      <c r="B23" s="58"/>
+      <c r="C23" s="58"/>
     </row>
     <row r="24" spans="1:73">
       <c r="A24" t="s">
@@ -39567,11 +42714,11 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75">
-      <c r="A33" s="57" t="s">
+      <c r="A33" s="58" t="s">
         <v>206</v>
       </c>
-      <c r="B33" s="57"/>
-      <c r="C33" s="57"/>
+      <c r="B33" s="58"/>
+      <c r="C33" s="58"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">

</xml_diff>

<commit_message>
Stage 2 step 2.10: checks sheet, sponsor support during lock-up; D24
</commit_message>
<xml_diff>
--- a/model/hydro_pf_model_v1.xlsx
+++ b/model/hydro_pf_model_v1.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22470" windowHeight="4815" tabRatio="872" firstSheet="4" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22470" windowHeight="4815" tabRatio="872" firstSheet="5" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="384">
   <si>
     <t>Cover</t>
   </si>
@@ -1229,6 +1229,42 @@
   <si>
     <t>Debt reduction, P90 vs P50 sizing</t>
   </si>
+  <si>
+    <t>1. SENSITIVITIES</t>
+  </si>
+  <si>
+    <t>1.A. CHECKS: TIMELINE</t>
+  </si>
+  <si>
+    <t>1.B. CHECKS: CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>1.C. CHECKS: OPERATIONS</t>
+  </si>
+  <si>
+    <t>1.D. CHECKS: TAX</t>
+  </si>
+  <si>
+    <t>1.E. CHECKS: DEBT</t>
+  </si>
+  <si>
+    <t>1.F. CHECKS: CASHFLOW</t>
+  </si>
+  <si>
+    <t>1.G. CHECKS: RATIOS</t>
+  </si>
+  <si>
+    <t>1.H. FINAL CHECKS</t>
+  </si>
+  <si>
+    <t>Total checks</t>
+  </si>
+  <si>
+    <t>Model status</t>
+  </si>
+  <si>
+    <t>1.I. INFO</t>
+  </si>
 </sst>
 </file>
 
@@ -1238,7 +1274,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1343,6 +1379,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1409,7 +1453,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1509,6 +1553,9 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1904,11 +1951,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>333</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -4304,11 +4351,11 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75">
-      <c r="A18" s="68" t="s">
+      <c r="A18" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="B18" s="68"/>
-      <c r="C18" s="68"/>
+      <c r="B18" s="69"/>
+      <c r="C18" s="69"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="59" t="s">
@@ -4356,11 +4403,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>343</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -5027,7 +5074,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -5049,212 +5096,196 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>361</v>
-      </c>
-      <c r="B4" t="s">
-        <v>362</v>
-      </c>
-      <c r="C4" t="s">
-        <v>363</v>
-      </c>
-      <c r="D4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" t="s">
-        <v>364</v>
-      </c>
-      <c r="F4" t="s">
-        <v>365</v>
-      </c>
-      <c r="G4" t="s">
-        <v>366</v>
-      </c>
-      <c r="H4" t="s">
-        <v>367</v>
-      </c>
-      <c r="I4" t="s">
-        <v>368</v>
-      </c>
+    <row r="4" spans="1:9" ht="15.75">
+      <c r="A4" s="69" t="s">
+        <v>372</v>
+      </c>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>350</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>8064962.5333756506</v>
+        <v>361</v>
+      </c>
+      <c r="B5" t="s">
+        <v>362</v>
+      </c>
+      <c r="C5" t="s">
+        <v>363</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>370</v>
-      </c>
-      <c r="F5" s="46">
-        <v>0.21682948118059092</v>
-      </c>
-      <c r="G5">
-        <v>1.3499999999999999</v>
-      </c>
-      <c r="H5" s="46">
-        <v>-6.7487194782582804E-3</v>
-      </c>
-      <c r="I5" s="46">
-        <v>-2.0217180039631022E-2</v>
+        <v>364</v>
+      </c>
+      <c r="F5" t="s">
+        <v>365</v>
+      </c>
+      <c r="G5" t="s">
+        <v>366</v>
+      </c>
+      <c r="H5" t="s">
+        <v>367</v>
+      </c>
+      <c r="I5" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>11959318.570513122</v>
+        <v>8064962.5333756506</v>
       </c>
       <c r="E6" t="s">
         <v>370</v>
       </c>
       <c r="F6" s="46">
-        <v>0.31564297808155756</v>
+        <v>0.21682948118059092</v>
       </c>
       <c r="G6">
         <v>1.3499999999999999</v>
       </c>
       <c r="H6" s="46">
-        <v>2.5415747697412616E-2</v>
+        <v>-6.7487194782582804E-3</v>
       </c>
       <c r="I6" s="46">
-        <v>9.5015933225579552E-3</v>
+        <v>-2.0217180039631022E-2</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7">
-        <v>8064962.5333756506</v>
+        <v>11959318.570513122</v>
       </c>
       <c r="E7" t="s">
         <v>370</v>
       </c>
       <c r="F7" s="46">
-        <v>0.21682948118059092</v>
+        <v>0.31564297808155756</v>
       </c>
       <c r="G7">
-        <v>1.8738120615312523</v>
+        <v>1.3499999999999999</v>
       </c>
       <c r="H7" s="46">
-        <v>2.5100433796284571E-2</v>
+        <v>2.5415747697412616E-2</v>
       </c>
       <c r="I7" s="46">
-        <v>1.4810516926449413E-2</v>
+        <v>9.5015933225579552E-3</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>352</v>
+        <v>369</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8">
-        <v>7178869.6286162753</v>
+        <v>8064962.5333756506</v>
       </c>
       <c r="E8" t="s">
         <v>370</v>
       </c>
       <c r="F8" s="46">
-        <v>0.19383352044709701</v>
+        <v>0.21682948118059092</v>
       </c>
       <c r="G8">
-        <v>1.3499999999999999</v>
+        <v>1.8738120615312523</v>
       </c>
       <c r="H8" s="46">
-        <v>-1.6310029201372811E-2</v>
+        <v>2.5100433796284571E-2</v>
       </c>
       <c r="I8" s="46">
-        <v>-2.9060507776270117E-2</v>
+        <v>1.4810516926449413E-2</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>5245721.090273818</v>
+        <v>7178869.6286162753</v>
       </c>
       <c r="E9" t="s">
         <v>370</v>
       </c>
       <c r="F9" s="46">
-        <v>0.1429636465383648</v>
+        <v>0.19383352044709701</v>
       </c>
       <c r="G9">
         <v>1.3499999999999999</v>
       </c>
       <c r="H9" s="46">
-        <v>-4.2297720327652666E-2</v>
+        <v>-1.6310029201372811E-2</v>
       </c>
       <c r="I9" s="46">
-        <v>-5.3546284652463139E-2</v>
+        <v>-2.9060507776270117E-2</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10">
-        <v>9520357.2663141508</v>
+        <v>5245721.090273818</v>
       </c>
       <c r="E10" t="s">
         <v>370</v>
       </c>
       <c r="F10" s="46">
-        <v>0.25418637293673058</v>
+        <v>0.1429636465383648</v>
       </c>
       <c r="G10">
         <v>1.3499999999999999</v>
       </c>
       <c r="H10" s="46">
-        <v>6.4077776049742408E-3</v>
+        <v>-4.2297720327652666E-2</v>
       </c>
       <c r="I10" s="46">
-        <v>-8.1417850763839672E-3</v>
+        <v>-5.3546284652463139E-2</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -5263,27 +5294,27 @@
         <v>1</v>
       </c>
       <c r="D11">
-        <v>6609567.8004371515</v>
+        <v>9520357.2663141508</v>
       </c>
       <c r="E11" t="s">
         <v>370</v>
       </c>
       <c r="F11" s="46">
-        <v>0.1789481042770813</v>
+        <v>0.25418637293673058</v>
       </c>
       <c r="G11">
         <v>1.3499999999999999</v>
       </c>
       <c r="H11" s="46">
-        <v>-2.2972554827725644E-2</v>
+        <v>6.4077776049742408E-3</v>
       </c>
       <c r="I11" s="46">
-        <v>-3.5268775638916838E-2</v>
+        <v>-8.1417850763839672E-3</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -5292,27 +5323,27 @@
         <v>1</v>
       </c>
       <c r="D12">
-        <v>7091614.8139742455</v>
+        <v>6609567.8004371515</v>
       </c>
       <c r="E12" t="s">
         <v>370</v>
       </c>
       <c r="F12" s="46">
-        <v>0.1673131980841904</v>
+        <v>0.1789481042770813</v>
       </c>
       <c r="G12">
         <v>1.3499999999999999</v>
       </c>
       <c r="H12" s="46">
-        <v>-2.8548419952834303E-2</v>
+        <v>-2.2972554827725644E-2</v>
       </c>
       <c r="I12" s="46">
-        <v>-4.0457803594064146E-2</v>
+        <v>-3.5268775638916838E-2</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -5321,27 +5352,27 @@
         <v>1</v>
       </c>
       <c r="D13">
-        <v>9038310.252777053</v>
+        <v>7091614.8139742455</v>
       </c>
       <c r="E13" t="s">
         <v>370</v>
       </c>
       <c r="F13" s="46">
-        <v>0.28240625401703595</v>
+        <v>0.1673131980841904</v>
       </c>
       <c r="G13">
         <v>1.3499999999999999</v>
       </c>
       <c r="H13" s="46">
-        <v>1.5418626409438474E-2</v>
+        <v>-2.8548419952834303E-2</v>
       </c>
       <c r="I13" s="46">
-        <v>1.6709697098726828E-4</v>
+        <v>-4.0457803594064146E-2</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -5350,27 +5381,27 @@
         <v>1</v>
       </c>
       <c r="D14">
-        <v>7700887.6171713695</v>
+        <v>9038310.252777053</v>
       </c>
       <c r="E14" t="s">
         <v>370</v>
       </c>
       <c r="F14" s="46">
-        <v>0.20683673806828964</v>
+        <v>0.28240625401703595</v>
       </c>
       <c r="G14">
         <v>1.3499999999999999</v>
       </c>
       <c r="H14" s="46">
-        <v>-6.7487194782582804E-3</v>
+        <v>1.5418626409438474E-2</v>
       </c>
       <c r="I14" s="46">
-        <v>-2.0946058887752916E-2</v>
+        <v>1.6709697098726828E-4</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -5379,13 +5410,13 @@
         <v>1</v>
       </c>
       <c r="D15">
-        <v>8456647.5007666796</v>
+        <v>7700887.6171713695</v>
       </c>
       <c r="E15" t="s">
         <v>370</v>
       </c>
       <c r="F15" s="46">
-        <v>0.22761259597296626</v>
+        <v>0.20683673806828964</v>
       </c>
       <c r="G15">
         <v>1.3499999999999999</v>
@@ -5394,12 +5425,12 @@
         <v>-6.7487194782582804E-3</v>
       </c>
       <c r="I15" s="46">
-        <v>-1.9416080386133516E-2</v>
+        <v>-2.0946058887752916E-2</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -5408,58 +5439,649 @@
         <v>1</v>
       </c>
       <c r="D16">
-        <v>9500032.2710536607</v>
+        <v>8456647.5007666796</v>
       </c>
       <c r="E16" t="s">
         <v>370</v>
       </c>
       <c r="F16" s="46">
-        <v>0.25431288201365254</v>
+        <v>0.22761259597296626</v>
       </c>
       <c r="G16">
         <v>1.3499999999999999</v>
       </c>
       <c r="H16" s="46">
+        <v>-6.7487194782582804E-3</v>
+      </c>
+      <c r="I16" s="46">
+        <v>-1.9416080386133516E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>360</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>9500032.2710536607</v>
+      </c>
+      <c r="E17" t="s">
+        <v>370</v>
+      </c>
+      <c r="F17" s="46">
+        <v>0.25431288201365254</v>
+      </c>
+      <c r="G17">
+        <v>1.3499999999999999</v>
+      </c>
+      <c r="H17" s="46">
         <v>2.5676368989479448E-2</v>
       </c>
-      <c r="I16" s="46">
+      <c r="I17" s="46">
         <v>1.4841920742470371E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
         <v>371</v>
       </c>
-      <c r="D18" s="46">
-        <f xml:space="preserve"> 1 - D5/D6</f>
+      <c r="D19" s="46">
+        <f xml:space="preserve"> 1 - D6/D7</f>
         <v>0.32563360647816419</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A4:I4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="1" max="1" width="100.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75">
+    <row r="1" spans="1:4" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
+    <row r="4" spans="1:4" ht="15.75">
+      <c r="A4" s="69" t="s">
+        <v>373</v>
+      </c>
+      <c r="B4" s="69"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="str">
+        <f>Timeline!A29</f>
+        <v>Check construction Flag</v>
+      </c>
+      <c r="B5" t="str">
+        <f>Timeline!B29</f>
+        <v>check</v>
+      </c>
+      <c r="C5">
+        <f>Timeline!C29</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="68" t="str">
+        <f>Timeline!D29</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="str">
+        <f>Timeline!A30</f>
+        <v>Check operation flag</v>
+      </c>
+      <c r="B6" t="str">
+        <f>Timeline!B30</f>
+        <v>check</v>
+      </c>
+      <c r="C6">
+        <f>Timeline!C30</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="68" t="str">
+        <f>Timeline!D30</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="str">
+        <f>Timeline!A31</f>
+        <v>Check repayment flag</v>
+      </c>
+      <c r="B7" t="str">
+        <f>Timeline!B31</f>
+        <v>check</v>
+      </c>
+      <c r="C7">
+        <f>Timeline!C31</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="68" t="str">
+        <f>Timeline!D31</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="str">
+        <f>Timeline!A32</f>
+        <v>Check overlap</v>
+      </c>
+      <c r="B8" t="str">
+        <f>Timeline!B32</f>
+        <v>check</v>
+      </c>
+      <c r="C8">
+        <f>Timeline!C32</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="68" t="str">
+        <f>Timeline!D32</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75">
+      <c r="A9" s="69" t="s">
+        <v>374</v>
+      </c>
+      <c r="B9" s="69"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="str">
+        <f>Construction!A20</f>
+        <v>Disbursement % − 1 =</v>
+      </c>
+      <c r="B10" t="str">
+        <f>Construction!B20</f>
+        <v>check</v>
+      </c>
+      <c r="C10">
+        <f>Construction!C20</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="68" t="str">
+        <f>Construction!D20</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="str">
+        <f>Construction!A21</f>
+        <v>Total nominal CAPEX =</v>
+      </c>
+      <c r="B11" t="str">
+        <f>Construction!B21</f>
+        <v>check</v>
+      </c>
+      <c r="C11">
+        <f>Construction!C21</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="68" t="str">
+        <f>Construction!D21</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="str">
+        <f>Construction!A35</f>
+        <v>Debt drawdown + Equity contribution - Total construction cost</v>
+      </c>
+      <c r="B12" t="str">
+        <f>Construction!B35</f>
+        <v>check</v>
+      </c>
+      <c r="C12">
+        <f>Construction!C35</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="68" t="str">
+        <f>Construction!D35</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="str">
+        <f>Construction!A36</f>
+        <v>Closing balance at COD - Debt commitment</v>
+      </c>
+      <c r="B13" t="str">
+        <f>Construction!B36</f>
+        <v>check</v>
+      </c>
+      <c r="C13">
+        <f>Construction!C36</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="68" t="str">
+        <f>Construction!D36</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="str">
+        <f>Construction!A62</f>
+        <v>Total sources - Total uses</v>
+      </c>
+      <c r="B14" t="str">
+        <f>Construction!B62</f>
+        <v>check</v>
+      </c>
+      <c r="C14">
+        <f>Construction!C62</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="68" t="str">
+        <f>Construction!D62</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75">
+      <c r="A15" s="69" t="s">
+        <v>375</v>
+      </c>
+      <c r="B15" s="69"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="str">
+        <f>Operations!A19</f>
+        <v>Total gross energy − Annual energy × Project life</v>
+      </c>
+      <c r="B16" t="str">
+        <f>Operations!B19</f>
+        <v>check</v>
+      </c>
+      <c r="C16">
+        <f>Operations!C19</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="68" t="str">
+        <f>Operations!D19</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="str">
+        <f>Operations!A20</f>
+        <v>Revenue</v>
+      </c>
+      <c r="B17" t="str">
+        <f>Operations!B20</f>
+        <v>check</v>
+      </c>
+      <c r="C17">
+        <f>Operations!C20</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="68" t="str">
+        <f>Operations!D20</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="str">
+        <f>Operations!A30</f>
+        <v>Total operating costs ≥ 0</v>
+      </c>
+      <c r="B18" t="str">
+        <f>Operations!B30</f>
+        <v>check</v>
+      </c>
+      <c r="C18">
+        <f>Operations!C30</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="68" t="str">
+        <f>Operations!D30</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.75">
+      <c r="A19" s="69" t="s">
+        <v>376</v>
+      </c>
+      <c r="B19" s="69"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="str">
+        <f>Tax!A17</f>
+        <v>Total tax depreciation − (Equipment base + Civil base × Project life / Fiscal life of civil works)</v>
+      </c>
+      <c r="B20" t="str">
+        <f>Tax!B17</f>
+        <v>check</v>
+      </c>
+      <c r="C20">
+        <f>Tax!C17</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="68" t="str">
+        <f>Tax!D17</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="str">
+        <f>Tax!A35</f>
+        <v>Tax paid ≥ 0</v>
+      </c>
+      <c r="B21" t="str">
+        <f>Tax!B35</f>
+        <v>check</v>
+      </c>
+      <c r="C21">
+        <f>Tax!C35</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="68" t="str">
+        <f>Tax!D35</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="str">
+        <f>Tax!A36</f>
+        <v>Corkscrew: Losses generated − Losses used − Expired losses − Last period closing balance =</v>
+      </c>
+      <c r="B22" t="str">
+        <f>Tax!B36</f>
+        <v>check</v>
+      </c>
+      <c r="C22">
+        <f>Tax!C36</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="68" t="str">
+        <f>Tax!D36</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15.75">
+      <c r="A23" s="69" t="s">
+        <v>377</v>
+      </c>
+      <c r="B23" s="69"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="str">
+        <f>Debt!A30</f>
+        <v>Check if Debt size (pasted value) = Debt size (calculated)</v>
+      </c>
+      <c r="B24" t="str">
+        <f>Debt!B30</f>
+        <v>check</v>
+      </c>
+      <c r="C24">
+        <f>Debt!C30</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="68" t="str">
+        <f>Debt!D30</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="str">
+        <f>Debt!A31</f>
+        <v>Check if k (pasted value) = k (calculated)</v>
+      </c>
+      <c r="B25" t="str">
+        <f>Debt!B31</f>
+        <v>check</v>
+      </c>
+      <c r="C25">
+        <f>Debt!C31</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="68" t="str">
+        <f>Debt!D31</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="str">
+        <f>Debt!A32</f>
+        <v>Last semester closing balance</v>
+      </c>
+      <c r="B26" t="str">
+        <f>Debt!B32</f>
+        <v>check</v>
+      </c>
+      <c r="C26">
+        <f>Debt!C32</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="68" t="str">
+        <f>Debt!D32</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15.75">
+      <c r="A27" s="69" t="s">
+        <v>378</v>
+      </c>
+      <c r="B27" s="69"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="str">
+        <f>Cashflow!A21</f>
+        <v>DSRA closing ≥ 0 in every semester</v>
+      </c>
+      <c r="B28" t="str">
+        <f>Cashflow!B21</f>
+        <v>check</v>
+      </c>
+      <c r="C28">
+        <f>Cashflow!C21</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="68">
+        <f>Cashflow!D21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="str">
+        <f>Cashflow!A22</f>
+        <v>DSRA closing in last column =</v>
+      </c>
+      <c r="B29" t="str">
+        <f>Cashflow!B22</f>
+        <v>check</v>
+      </c>
+      <c r="C29">
+        <f>Cashflow!C22</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="68">
+        <f>Cashflow!D22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="str">
+        <f>Cashflow!A34</f>
+        <v>Retained cash closing ≥ 0</v>
+      </c>
+      <c r="B30" t="str">
+        <f>Cashflow!B34</f>
+        <v>check</v>
+      </c>
+      <c r="C30">
+        <f>Cashflow!C34</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="68" t="str">
+        <f>Cashflow!D34</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" t="str">
+        <f>Cashflow!A35</f>
+        <v>total CFADS − total Debt service + total Initial funding − total Distributions − last column retained cash closing  =</v>
+      </c>
+      <c r="B31" t="str">
+        <f>Cashflow!B35</f>
+        <v>check</v>
+      </c>
+      <c r="C31">
+        <f>Cashflow!C35</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="68" t="str">
+        <f>Cashflow!D35</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15.75">
+      <c r="A32" s="69" t="s">
+        <v>379</v>
+      </c>
+      <c r="B32" s="69"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" t="str">
+        <f>Ratios!A19</f>
+        <v>1st semester LLCR - target DSCR =</v>
+      </c>
+      <c r="B33" t="str">
+        <f>Ratios!B19</f>
+        <v>check</v>
+      </c>
+      <c r="C33">
+        <f>Ratios!C19</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="68" t="str">
+        <f>Ratios!D19</f>
+        <v>Must be =0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15.75">
+      <c r="A34" s="69" t="s">
+        <v>380</v>
+      </c>
+      <c r="B34" s="69"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="33"/>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" t="s">
+        <v>381</v>
+      </c>
+      <c r="B35" t="s">
+        <v>165</v>
+      </c>
+      <c r="C35">
+        <f>ROUND(SUM(C5:C33),4)</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="68" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" t="s">
+        <v>382</v>
+      </c>
+      <c r="B36" s="59" t="str">
+        <f>IF(C35=0,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15.75">
+      <c r="A37" s="69" t="s">
+        <v>383</v>
+      </c>
+      <c r="B37" s="69"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="str">
+        <f>Cashflow!A36</f>
+        <v>Lock-up flag</v>
+      </c>
+      <c r="B38" t="str">
+        <f>Cashflow!B36</f>
+        <v>info</v>
+      </c>
+      <c r="C38">
+        <f>Cashflow!C36</f>
+        <v>0</v>
+      </c>
+      <c r="D38" t="str">
+        <f>Cashflow!D36</f>
+        <v>if=0 -&gt; No Lock-up</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="str">
+        <f>Cashflow!A37</f>
+        <v>Default flag</v>
+      </c>
+      <c r="B39" t="str">
+        <f>Cashflow!B37</f>
+        <v>info</v>
+      </c>
+      <c r="C39">
+        <f>Cashflow!C37</f>
+        <v>0</v>
+      </c>
+      <c r="D39" t="str">
+        <f>Cashflow!D37</f>
+        <v>if=0 -&gt; No defaults</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A9:B9"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11208,11 +11830,11 @@
       </c>
     </row>
     <row r="5" spans="1:75" ht="15.75">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="69" t="s">
         <v>169</v>
       </c>
-      <c r="B5" s="68"/>
-      <c r="C5" s="68"/>
+      <c r="B5" s="69"/>
+      <c r="C5" s="69"/>
       <c r="D5" s="43"/>
       <c r="E5" s="43"/>
       <c r="F5" s="43"/>
@@ -11294,12 +11916,12 @@
       </c>
     </row>
     <row r="14" spans="1:75" ht="15.75">
-      <c r="A14" s="68" t="s">
+      <c r="A14" s="69" t="s">
         <v>170</v>
       </c>
-      <c r="B14" s="68"/>
-      <c r="C14" s="68"/>
-      <c r="D14" s="68"/>
+      <c r="B14" s="69"/>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
       <c r="E14" s="33"/>
       <c r="F14" s="33"/>
       <c r="G14" s="33"/>
@@ -14577,12 +15199,12 @@
       </c>
     </row>
     <row r="27" spans="1:73" ht="15.75">
-      <c r="A27" s="68" t="s">
+      <c r="A27" s="69" t="s">
         <v>171</v>
       </c>
-      <c r="B27" s="68"/>
-      <c r="C27" s="68"/>
-      <c r="D27" s="68"/>
+      <c r="B27" s="69"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="69"/>
       <c r="E27" s="41"/>
       <c r="F27" s="41"/>
       <c r="G27" s="41"/>
@@ -14696,11 +15318,11 @@
       </c>
     </row>
     <row r="4" spans="1:74" ht="15.75">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="1:74">
       <c r="A5" t="s">
@@ -15589,11 +16211,11 @@
       <c r="BV8" s="8"/>
     </row>
     <row r="9" spans="1:74" ht="15.75">
-      <c r="A9" s="68" t="s">
+      <c r="A9" s="69" t="s">
         <v>193</v>
       </c>
-      <c r="B9" s="68"/>
-      <c r="C9" s="68"/>
+      <c r="B9" s="69"/>
+      <c r="C9" s="69"/>
     </row>
     <row r="10" spans="1:74">
       <c r="A10" t="s">
@@ -17650,21 +18272,21 @@
       </c>
     </row>
     <row r="19" spans="1:73" ht="15.75">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="69" t="s">
         <v>194</v>
       </c>
-      <c r="B19" s="68"/>
-      <c r="C19" s="68"/>
-      <c r="D19" s="68"/>
+      <c r="B19" s="69"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="69"/>
     </row>
     <row r="20" spans="1:73">
-      <c r="A20" t="s">
+      <c r="A20" s="59" t="s">
         <v>182</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="59" t="s">
         <v>165</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="59">
         <f>SUM(D12:BU12)-1</f>
         <v>0</v>
       </c>
@@ -17673,13 +18295,13 @@
       </c>
     </row>
     <row r="21" spans="1:73">
-      <c r="A21" t="s">
+      <c r="A21" s="59" t="s">
         <v>183</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="59" t="s">
         <v>165</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="59">
         <f>IF(SUM(D14:BU14)&gt;=C10,0,1)</f>
         <v>0</v>
       </c>
@@ -17688,11 +18310,11 @@
       </c>
     </row>
     <row r="24" spans="1:73" ht="15.75">
-      <c r="A24" s="68" t="s">
+      <c r="A24" s="69" t="s">
         <v>205</v>
       </c>
-      <c r="B24" s="68"/>
-      <c r="C24" s="68"/>
+      <c r="B24" s="69"/>
+      <c r="C24" s="69"/>
     </row>
     <row r="25" spans="1:73">
       <c r="A25" t="s">
@@ -19477,11 +20099,11 @@
       </c>
     </row>
     <row r="34" spans="1:73" ht="15.75">
-      <c r="A34" s="68" t="s">
+      <c r="A34" s="69" t="s">
         <v>206</v>
       </c>
-      <c r="B34" s="68"/>
-      <c r="C34" s="68"/>
+      <c r="B34" s="69"/>
+      <c r="C34" s="69"/>
     </row>
     <row r="35" spans="1:73">
       <c r="A35" s="59" t="s">
@@ -19514,11 +20136,11 @@
       </c>
     </row>
     <row r="37" spans="1:73" ht="15.75">
-      <c r="A37" s="68" t="s">
+      <c r="A37" s="69" t="s">
         <v>207</v>
       </c>
-      <c r="B37" s="68"/>
-      <c r="C37" s="68"/>
+      <c r="B37" s="69"/>
+      <c r="C37" s="69"/>
     </row>
     <row r="38" spans="1:73">
       <c r="A38" t="s">
@@ -21561,11 +22183,11 @@
       </c>
     </row>
     <row r="45" spans="1:73" ht="15.75">
-      <c r="A45" s="68" t="s">
+      <c r="A45" s="69" t="s">
         <v>215</v>
       </c>
-      <c r="B45" s="68"/>
-      <c r="C45" s="68"/>
+      <c r="B45" s="69"/>
+      <c r="C45" s="69"/>
     </row>
     <row r="46" spans="1:73">
       <c r="A46" t="s">
@@ -21664,11 +22286,11 @@
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.75">
-      <c r="A54" s="68" t="s">
+      <c r="A54" s="69" t="s">
         <v>216</v>
       </c>
-      <c r="B54" s="68"/>
-      <c r="C54" s="68"/>
+      <c r="B54" s="69"/>
+      <c r="C54" s="69"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
@@ -21731,11 +22353,11 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="15.75">
-      <c r="A61" s="68" t="s">
+      <c r="A61" s="69" t="s">
         <v>222</v>
       </c>
-      <c r="B61" s="68"/>
-      <c r="C61" s="68"/>
+      <c r="B61" s="69"/>
+      <c r="C61" s="69"/>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="59" t="s">
@@ -21860,11 +22482,11 @@
       </c>
     </row>
     <row r="4" spans="1:75" ht="15.75">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>240</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="1:75">
       <c r="A5" t="s">
@@ -24690,11 +25312,11 @@
       </c>
     </row>
     <row r="18" spans="1:73" ht="15.75">
-      <c r="A18" s="68" t="s">
+      <c r="A18" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="B18" s="68"/>
-      <c r="C18" s="68"/>
+      <c r="B18" s="69"/>
+      <c r="C18" s="69"/>
     </row>
     <row r="19" spans="1:73">
       <c r="A19" s="59" t="s">
@@ -24727,11 +25349,11 @@
       </c>
     </row>
     <row r="21" spans="1:73" ht="15.75">
-      <c r="A21" s="68" t="s">
+      <c r="A21" s="69" t="s">
         <v>245</v>
       </c>
-      <c r="B21" s="68"/>
-      <c r="C21" s="68"/>
+      <c r="B21" s="69"/>
+      <c r="C21" s="69"/>
     </row>
     <row r="22" spans="1:73">
       <c r="A22" t="str">
@@ -26779,11 +27401,11 @@
       </c>
     </row>
     <row r="29" spans="1:73" ht="15.75">
-      <c r="A29" s="68" t="s">
+      <c r="A29" s="69" t="s">
         <v>206</v>
       </c>
-      <c r="B29" s="68"/>
-      <c r="C29" s="68"/>
+      <c r="B29" s="69"/>
+      <c r="C29" s="69"/>
     </row>
     <row r="30" spans="1:73">
       <c r="A30" s="59" t="s">
@@ -26835,11 +27457,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>255</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -28938,11 +29560,11 @@
       </c>
     </row>
     <row r="16" spans="1:73" ht="15.75">
-      <c r="A16" s="68" t="s">
+      <c r="A16" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="B16" s="68"/>
-      <c r="C16" s="68"/>
+      <c r="B16" s="69"/>
+      <c r="C16" s="69"/>
     </row>
     <row r="17" spans="1:73" ht="30">
       <c r="A17" s="61" t="s">
@@ -28960,11 +29582,11 @@
       </c>
     </row>
     <row r="18" spans="1:73" ht="15.75">
-      <c r="A18" s="68" t="s">
+      <c r="A18" s="69" t="s">
         <v>257</v>
       </c>
-      <c r="B18" s="68"/>
-      <c r="C18" s="68"/>
+      <c r="B18" s="69"/>
+      <c r="C18" s="69"/>
     </row>
     <row r="19" spans="1:73">
       <c r="A19" t="s">
@@ -33035,11 +33657,11 @@
       </c>
     </row>
     <row r="34" spans="1:73" ht="15.75">
-      <c r="A34" s="68" t="s">
+      <c r="A34" s="69" t="s">
         <v>206</v>
       </c>
-      <c r="B34" s="68"/>
-      <c r="C34" s="68"/>
+      <c r="B34" s="69"/>
+      <c r="C34" s="69"/>
     </row>
     <row r="35" spans="1:73">
       <c r="A35" s="59" t="s">
@@ -33108,11 +33730,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>285</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -35523,11 +36145,11 @@
       </c>
     </row>
     <row r="19" spans="1:73" ht="15.75">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="69" t="s">
         <v>286</v>
       </c>
-      <c r="B19" s="68"/>
-      <c r="C19" s="68"/>
+      <c r="B19" s="69"/>
+      <c r="C19" s="69"/>
     </row>
     <row r="20" spans="1:73">
       <c r="A20" t="s">
@@ -37226,11 +37848,11 @@
       </c>
     </row>
     <row r="29" spans="1:73" ht="15.75">
-      <c r="A29" s="68" t="s">
+      <c r="A29" s="69" t="s">
         <v>206</v>
       </c>
-      <c r="B29" s="68"/>
-      <c r="C29" s="68"/>
+      <c r="B29" s="69"/>
+      <c r="C29" s="69"/>
     </row>
     <row r="30" spans="1:73">
       <c r="A30" s="59" t="s">
@@ -37309,11 +37931,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="69" t="s">
         <v>310</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -41118,11 +41740,11 @@
       </c>
     </row>
     <row r="20" spans="1:73" ht="15.75">
-      <c r="A20" s="68" t="s">
+      <c r="A20" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="B20" s="68"/>
-      <c r="C20" s="68"/>
+      <c r="B20" s="69"/>
+      <c r="C20" s="69"/>
     </row>
     <row r="21" spans="1:73">
       <c r="A21" s="59" t="s">
@@ -41149,11 +41771,11 @@
       </c>
     </row>
     <row r="23" spans="1:73" ht="15.75">
-      <c r="A23" s="68" t="s">
+      <c r="A23" s="69" t="s">
         <v>311</v>
       </c>
-      <c r="B23" s="68"/>
-      <c r="C23" s="68"/>
+      <c r="B23" s="69"/>
+      <c r="C23" s="69"/>
     </row>
     <row r="24" spans="1:73">
       <c r="A24" t="s">
@@ -41451,19 +42073,19 @@
         <v>39</v>
       </c>
       <c r="D25">
-        <f>IF(D7=1, (E8+D8)/(D9+E9),0)</f>
+        <f t="shared" ref="D25:BQ25" si="18">IF(D7=1, (D8+C8)/(C9+D9),0)</f>
         <v>0</v>
       </c>
       <c r="E25">
-        <f>IF(E7=1, (E8+D8)/(D9+E9),0)</f>
+        <f t="shared" ref="E25" si="19">IF(E7=1, (E8+D8)/(D9+E9),0)</f>
         <v>0</v>
       </c>
       <c r="F25">
-        <f t="shared" ref="F25:BQ25" si="18">IF(F7=1, (F8+E8)/(E9+F9),0)</f>
+        <f t="shared" ref="F25" si="20">IF(F7=1, (F8+E8)/(E9+F9),0)</f>
         <v>0</v>
       </c>
       <c r="G25">
-        <f t="shared" si="18"/>
+        <f t="shared" ref="G25" si="21">IF(G7=1, (G8+F8)/(F9+G9),0)</f>
         <v>0</v>
       </c>
       <c r="H25">
@@ -41715,19 +42337,19 @@
         <v>0</v>
       </c>
       <c r="BR25">
-        <f t="shared" ref="BR25:BU25" si="19">IF(BR7=1, (BR8+BQ8)/(BQ9+BR9),0)</f>
+        <f t="shared" ref="BR25:BU25" si="22">IF(BR7=1, (BR8+BQ8)/(BQ9+BR9),0)</f>
         <v>0</v>
       </c>
       <c r="BS25">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="BT25">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="BU25">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
     </row>
@@ -42331,275 +42953,275 @@
         <v>0</v>
       </c>
       <c r="F29">
-        <f t="shared" ref="F29:BQ29" si="20">E32</f>
+        <f t="shared" ref="F29:BQ29" si="23">E32</f>
         <v>0</v>
       </c>
       <c r="G29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="H29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="I29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="J29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="K29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="L29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="M29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="N29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="O29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="P29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="Q29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="R29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="S29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="T29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="U29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="V29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="W29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="X29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="Y29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="Z29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AA29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AB29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AC29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AD29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AE29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AF29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AG29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AH29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AI29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AJ29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AK29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AL29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AM29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AN29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AO29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AP29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AQ29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AR29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AS29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AT29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AU29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AV29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AW29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AX29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AY29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AZ29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BA29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BB29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BC29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BD29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BE29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BF29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BG29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BH29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BI29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BJ29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BK29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BL29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BM29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BN29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BO29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BP29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BQ29">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BR29">
-        <f t="shared" ref="BR29:BU29" si="21">BQ32</f>
+        <f t="shared" ref="BR29:BU29" si="24">BQ32</f>
         <v>0</v>
       </c>
       <c r="BS29">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="BT29">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="BU29">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -42615,279 +43237,279 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <f t="shared" ref="E30:BP30" si="22">E24</f>
+        <f t="shared" ref="E30:BP30" si="25">E24</f>
         <v>0</v>
       </c>
       <c r="F30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="G30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>320459.03710749489</v>
       </c>
       <c r="I30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>99498.167385116336</v>
       </c>
       <c r="J30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>317694.32405581849</v>
       </c>
       <c r="K30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>96717.627019557462</v>
       </c>
       <c r="L30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>314886.0588455589</v>
       </c>
       <c r="M30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>93850.225790866563</v>
       </c>
       <c r="N30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>311990.06668010377</v>
       </c>
       <c r="O30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>90945.216344759217</v>
       </c>
       <c r="P30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>309056.09130465903</v>
       </c>
       <c r="Q30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>87982.146871918667</v>
       </c>
       <c r="R30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>306063.47698435304</v>
       </c>
       <c r="S30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>84972.400558059599</v>
       </c>
       <c r="T30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>303023.72040695848</v>
       </c>
       <c r="U30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>81868.633252500964</v>
       </c>
       <c r="V30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>299889.00535196217</v>
       </c>
       <c r="W30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>78724.157602930645</v>
       </c>
       <c r="X30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>296713.17604893271</v>
       </c>
       <c r="Y30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>75516.83591321393</v>
       </c>
       <c r="Z30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>293473.87406615645</v>
       </c>
       <c r="AA30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>72258.989709651389</v>
       </c>
       <c r="AB30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>290183.54378821346</v>
       </c>
       <c r="AC30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>68899.372160958155</v>
       </c>
       <c r="AD30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>684214.074103844</v>
       </c>
       <c r="AE30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>146662.2572858546</v>
       </c>
       <c r="AF30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>1073043.8460997068</v>
       </c>
       <c r="AG30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>219149.7300746867</v>
       </c>
       <c r="AH30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>1059121.9577739565</v>
       </c>
       <c r="AI30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>205089.788519767</v>
       </c>
       <c r="AJ30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>1044921.824153874</v>
       </c>
       <c r="AK30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>190709.16113469214</v>
       </c>
       <c r="AL30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>732272.82580145611</v>
       </c>
       <c r="AM30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>176080.80139608099</v>
       </c>
       <c r="AN30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>723555.55378948129</v>
       </c>
       <c r="AO30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>161160.07670195331</v>
       </c>
       <c r="AP30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>718982.63265880744</v>
       </c>
       <c r="AQ30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>145941.14379518793</v>
       </c>
       <c r="AR30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>714318.31632683706</v>
       </c>
       <c r="AS30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>130375.09023260616</v>
       </c>
       <c r="AT30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>709547.61405085807</v>
       </c>
       <c r="AU30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>114540.88320348423</v>
       </c>
       <c r="AV30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>704694.72778726846</v>
       </c>
       <c r="AW30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>98390.210944054183</v>
       </c>
       <c r="AX30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>699744.85089028359</v>
       </c>
       <c r="AY30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>81916.748524889117</v>
       </c>
       <c r="AZ30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>694696.04488814552</v>
       </c>
       <c r="BA30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>65067.551544468035</v>
       </c>
       <c r="BB30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>689532.08331884071</v>
       </c>
       <c r="BC30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>47928.096628048341</v>
       </c>
       <c r="BD30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>684279.16315830906</v>
       </c>
       <c r="BE30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>30446.089568821597</v>
       </c>
       <c r="BF30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>678921.2572169716</v>
       </c>
       <c r="BG30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>12614.684059765772</v>
       </c>
       <c r="BH30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>673456.26723065635</v>
       </c>
       <c r="BI30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>-5623.4286220169161</v>
       </c>
       <c r="BJ30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>667866.62915503676</v>
       </c>
       <c r="BK30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>-24175.725828419672</v>
       </c>
       <c r="BL30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>662180.69943936495</v>
       </c>
       <c r="BM30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>-43098.812490673736</v>
       </c>
       <c r="BN30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>656381.12973820628</v>
       </c>
       <c r="BO30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>-62400.099271676852</v>
       </c>
       <c r="BP30">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="BQ30">
-        <f t="shared" ref="BQ30:BU30" si="23">BQ24</f>
+        <f t="shared" ref="BQ30:BU30" si="26">BQ24</f>
         <v>0</v>
       </c>
       <c r="BR30">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="BS30">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="BT30">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="BU30">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
     </row>
@@ -42903,283 +43525,283 @@
         <v>20257171.892233226</v>
       </c>
       <c r="D31">
-        <f>IF(D26=1,0,D29+D30)</f>
+        <f>IF(D26=1,MIN(0,D29+D30),D29+D30)</f>
         <v>0</v>
       </c>
       <c r="E31">
-        <f t="shared" ref="E31:BP31" si="24">IF(E26=1,0,E29+E30)</f>
+        <f t="shared" ref="E31:BP31" si="27">IF(E26=1,MIN(0,E29+E30),E29+E30)</f>
         <v>0</v>
       </c>
       <c r="F31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="G31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="H31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>320459.03710749489</v>
       </c>
       <c r="I31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>99498.167385116336</v>
       </c>
       <c r="J31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>317694.32405581849</v>
       </c>
       <c r="K31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>96717.627019557462</v>
       </c>
       <c r="L31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>314886.0588455589</v>
       </c>
       <c r="M31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>93850.225790866563</v>
       </c>
       <c r="N31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>311990.06668010377</v>
       </c>
       <c r="O31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>90945.216344759217</v>
       </c>
       <c r="P31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>309056.09130465903</v>
       </c>
       <c r="Q31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>87982.146871918667</v>
       </c>
       <c r="R31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>306063.47698435304</v>
       </c>
       <c r="S31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>84972.400558059599</v>
       </c>
       <c r="T31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>303023.72040695848</v>
       </c>
       <c r="U31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>81868.633252500964</v>
       </c>
       <c r="V31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>299889.00535196217</v>
       </c>
       <c r="W31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>78724.157602930645</v>
       </c>
       <c r="X31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>296713.17604893271</v>
       </c>
       <c r="Y31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>75516.83591321393</v>
       </c>
       <c r="Z31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>293473.87406615645</v>
       </c>
       <c r="AA31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>72258.989709651389</v>
       </c>
       <c r="AB31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>290183.54378821346</v>
       </c>
       <c r="AC31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>68899.372160958155</v>
       </c>
       <c r="AD31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>684214.074103844</v>
       </c>
       <c r="AE31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>146662.2572858546</v>
       </c>
       <c r="AF31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>1073043.8460997068</v>
       </c>
       <c r="AG31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>219149.7300746867</v>
       </c>
       <c r="AH31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>1059121.9577739565</v>
       </c>
       <c r="AI31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>205089.788519767</v>
       </c>
       <c r="AJ31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>1044921.824153874</v>
       </c>
       <c r="AK31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>190709.16113469214</v>
       </c>
       <c r="AL31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>732272.82580145611</v>
       </c>
       <c r="AM31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>176080.80139608099</v>
       </c>
       <c r="AN31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>723555.55378948129</v>
       </c>
       <c r="AO31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>161160.07670195331</v>
       </c>
       <c r="AP31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>718982.63265880744</v>
       </c>
       <c r="AQ31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>145941.14379518793</v>
       </c>
       <c r="AR31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>714318.31632683706</v>
       </c>
       <c r="AS31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>130375.09023260616</v>
       </c>
       <c r="AT31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>709547.61405085807</v>
       </c>
       <c r="AU31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>114540.88320348423</v>
       </c>
       <c r="AV31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>704694.72778726846</v>
       </c>
       <c r="AW31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>98390.210944054183</v>
       </c>
       <c r="AX31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>699744.85089028359</v>
       </c>
       <c r="AY31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>81916.748524889117</v>
       </c>
       <c r="AZ31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>694696.04488814552</v>
       </c>
       <c r="BA31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>65067.551544468035</v>
       </c>
       <c r="BB31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>689532.08331884071</v>
       </c>
       <c r="BC31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>47928.096628048341</v>
       </c>
       <c r="BD31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>684279.16315830906</v>
       </c>
       <c r="BE31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>30446.089568821597</v>
       </c>
       <c r="BF31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>678921.2572169716</v>
       </c>
       <c r="BG31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>12614.684059765772</v>
       </c>
       <c r="BH31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>673456.26723065635</v>
       </c>
       <c r="BI31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-5623.4286220169161</v>
       </c>
       <c r="BJ31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>667866.62915503676</v>
       </c>
       <c r="BK31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-24175.725828419672</v>
       </c>
       <c r="BL31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>662180.69943936495</v>
       </c>
       <c r="BM31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-43098.812490673736</v>
       </c>
       <c r="BN31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>656381.12973820628</v>
       </c>
       <c r="BO31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-62400.099271676852</v>
       </c>
       <c r="BP31">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="BQ31">
-        <f t="shared" ref="BQ31:BU31" si="25">IF(BQ26=1,0,BQ29+BQ30)</f>
+        <f t="shared" ref="BQ31:BU31" si="28">IF(BQ26=1,MIN(0,BQ29+BQ30),BQ29+BQ30)</f>
         <v>0</v>
       </c>
       <c r="BR31">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="BS31">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="BT31">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="BU31">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
     </row>
@@ -43195,288 +43817,288 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <f t="shared" ref="E32:BP32" si="26">E29+E30-E31</f>
+        <f t="shared" ref="E32:BP32" si="29">E29+E30-E31</f>
         <v>0</v>
       </c>
       <c r="F32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="G32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="H32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="I32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="J32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="K32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="L32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="M32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="N32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="O32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="P32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="Q32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="R32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="S32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="T32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="U32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="V32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="W32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="X32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="Y32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="Z32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AA32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AB32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AC32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AD32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AE32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AF32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AG32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AH32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AI32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AJ32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AK32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AL32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AM32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AN32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AO32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AP32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AQ32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AR32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AS32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AT32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AU32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AV32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AW32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AX32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AY32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="AZ32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BA32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BB32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BC32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BD32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BE32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BF32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BG32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BH32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BI32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BJ32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BK32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BL32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BN32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BO32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BP32">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BQ32">
-        <f t="shared" ref="BQ32:BU32" si="27">BQ29+BQ30-BQ31</f>
+        <f t="shared" ref="BQ32:BU32" si="30">BQ29+BQ30-BQ31</f>
         <v>0</v>
       </c>
       <c r="BR32">
-        <f t="shared" si="27"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="BS32">
-        <f t="shared" si="27"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="BT32">
-        <f t="shared" si="27"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="BU32">
-        <f t="shared" si="27"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75">
-      <c r="A33" s="68" t="s">
+      <c r="A33" s="69" t="s">
         <v>206</v>
       </c>
-      <c r="B33" s="68"/>
-      <c r="C33" s="68"/>
+      <c r="B33" s="69"/>
+      <c r="C33" s="69"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="59" t="s">

</xml_diff>

<commit_message>
Stage 2 step 2.10: model book, availability sensitivity, label fixes
</commit_message>
<xml_diff>
--- a/model/hydro_pf_model_v1.xlsx
+++ b/model/hydro_pf_model_v1.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22470" windowHeight="4815" tabRatio="872" firstSheet="5" activeTab="12"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22470" windowHeight="4815" tabRatio="872"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="385">
   <si>
     <t>Cover</t>
   </si>
@@ -930,9 +930,6 @@
     <t>Financing costs during construction (IDC + fees)</t>
   </si>
   <si>
-    <t>Interest expense in operations (placeholder, linked in step 2.6)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Label </t>
   </si>
   <si>
@@ -1265,6 +1262,24 @@
   <si>
     <t>1.I. INFO</t>
   </si>
+  <si>
+    <r>
+      <t>Availability factor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = 0,88</t>
+    </r>
+  </si>
+  <si>
+    <t>Interest expense in operations</t>
+  </si>
 </sst>
 </file>
 
@@ -1453,7 +1468,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1557,6 +1572,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1586,11 +1602,11 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="semiannual_energy_1" connectionId="2" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="annual_energy_1" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="annual_energy_1" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="semiannual_energy_1" connectionId="2" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1882,6 +1898,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.75">
@@ -1951,21 +1968,21 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="69" t="s">
-        <v>333</v>
-      </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="A4" s="70" t="s">
+        <v>332</v>
+      </c>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:73">
@@ -3440,7 +3457,7 @@
     </row>
     <row r="11" spans="1:73">
       <c r="A11" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
@@ -3728,7 +3745,7 @@
     </row>
     <row r="12" spans="1:73">
       <c r="A12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B12" t="s">
         <v>184</v>
@@ -4016,7 +4033,7 @@
     </row>
     <row r="13" spans="1:73">
       <c r="A13" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
@@ -4304,7 +4321,7 @@
     </row>
     <row r="14" spans="1:73">
       <c r="A14" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B14" t="s">
         <v>39</v>
@@ -4316,7 +4333,7 @@
     </row>
     <row r="15" spans="1:73">
       <c r="A15" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B15" t="s">
         <v>39</v>
@@ -4328,7 +4345,7 @@
     </row>
     <row r="16" spans="1:73">
       <c r="A16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B16" t="s">
         <v>39</v>
@@ -4340,7 +4357,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B17" t="s">
         <v>39</v>
@@ -4351,15 +4368,15 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75">
-      <c r="A18" s="69" t="s">
+      <c r="A18" s="70" t="s">
         <v>239</v>
       </c>
-      <c r="B18" s="69"/>
-      <c r="C18" s="69"/>
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="59" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B19" s="59" t="s">
         <v>165</v>
@@ -4403,26 +4420,26 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="69" t="s">
-        <v>343</v>
-      </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="A4" s="70" t="s">
+        <v>342</v>
+      </c>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
         <v>145</v>
       </c>
       <c r="B5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" spans="1:73">
       <c r="A6" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B6" t="s">
         <v>184</v>
@@ -4714,7 +4731,7 @@
     </row>
     <row r="7" spans="1:73">
       <c r="A7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B7" t="s">
         <v>184</v>
@@ -5006,7 +5023,7 @@
     </row>
     <row r="8" spans="1:73">
       <c r="A8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B8" t="s">
         <v>39</v>
@@ -5018,7 +5035,7 @@
     </row>
     <row r="9" spans="1:73">
       <c r="A9" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B9" t="s">
         <v>39</v>
@@ -5030,7 +5047,7 @@
     </row>
     <row r="10" spans="1:73">
       <c r="A10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B10" t="s">
         <v>39</v>
@@ -5042,7 +5059,7 @@
     </row>
     <row r="11" spans="1:73">
       <c r="A11" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
@@ -5054,7 +5071,7 @@
     </row>
     <row r="12" spans="1:73">
       <c r="A12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
@@ -5074,7 +5091,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -5097,50 +5114,50 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75">
-      <c r="A4" s="69" t="s">
-        <v>372</v>
-      </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
-      <c r="D4" s="69"/>
-      <c r="E4" s="69"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="69"/>
-      <c r="I4" s="69"/>
+      <c r="A4" s="70" t="s">
+        <v>371</v>
+      </c>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
+      <c r="I4" s="70"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
+        <v>360</v>
+      </c>
+      <c r="B5" t="s">
         <v>361</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>362</v>
-      </c>
-      <c r="C5" t="s">
-        <v>363</v>
       </c>
       <c r="D5" t="s">
         <v>56</v>
       </c>
       <c r="E5" t="s">
+        <v>363</v>
+      </c>
+      <c r="F5" t="s">
         <v>364</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>365</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>366</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>367</v>
-      </c>
-      <c r="I5" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -5152,7 +5169,7 @@
         <v>8064962.5333756506</v>
       </c>
       <c r="E6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F6" s="46">
         <v>0.21682948118059092</v>
@@ -5169,7 +5186,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -5181,7 +5198,7 @@
         <v>11959318.570513122</v>
       </c>
       <c r="E7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F7" s="46">
         <v>0.31564297808155756</v>
@@ -5198,7 +5215,7 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -5210,7 +5227,7 @@
         <v>8064962.5333756506</v>
       </c>
       <c r="E8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F8" s="46">
         <v>0.21682948118059092</v>
@@ -5227,7 +5244,7 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B9">
         <v>3</v>
@@ -5239,7 +5256,7 @@
         <v>7178869.6286162753</v>
       </c>
       <c r="E9" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F9" s="46">
         <v>0.19383352044709701</v>
@@ -5256,7 +5273,7 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B10">
         <v>4</v>
@@ -5268,7 +5285,7 @@
         <v>5245721.090273818</v>
       </c>
       <c r="E10" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F10" s="46">
         <v>0.1429636465383648</v>
@@ -5285,7 +5302,7 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -5297,7 +5314,7 @@
         <v>9520357.2663141508</v>
       </c>
       <c r="E11" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F11" s="46">
         <v>0.25418637293673058</v>
@@ -5314,7 +5331,7 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -5326,7 +5343,7 @@
         <v>6609567.8004371515</v>
       </c>
       <c r="E12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F12" s="46">
         <v>0.1789481042770813</v>
@@ -5343,7 +5360,7 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -5355,7 +5372,7 @@
         <v>7091614.8139742455</v>
       </c>
       <c r="E13" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F13" s="46">
         <v>0.1673131980841904</v>
@@ -5372,7 +5389,7 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -5384,7 +5401,7 @@
         <v>9038310.252777053</v>
       </c>
       <c r="E14" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F14" s="46">
         <v>0.28240625401703595</v>
@@ -5401,7 +5418,7 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -5413,7 +5430,7 @@
         <v>7700887.6171713695</v>
       </c>
       <c r="E15" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F15" s="46">
         <v>0.20683673806828964</v>
@@ -5430,7 +5447,7 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -5442,7 +5459,7 @@
         <v>8456647.5007666796</v>
       </c>
       <c r="E16" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F16" s="46">
         <v>0.22761259597296626</v>
@@ -5459,7 +5476,7 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -5471,7 +5488,7 @@
         <v>9500032.2710536607</v>
       </c>
       <c r="E17" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F17" s="46">
         <v>0.25431288201365254</v>
@@ -5486,11 +5503,40 @@
         <v>1.4841920742470371E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
-      <c r="A19" t="s">
-        <v>371</v>
-      </c>
-      <c r="D19" s="46">
+    <row r="18" spans="1:9">
+      <c r="A18" s="69" t="s">
+        <v>383</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>7432182.2147067385</v>
+      </c>
+      <c r="E18" t="s">
+        <v>369</v>
+      </c>
+      <c r="F18" s="46">
+        <v>0.20042440908592229</v>
+      </c>
+      <c r="G18">
+        <v>1.35</v>
+      </c>
+      <c r="H18" s="46">
+        <v>-1.3511357092961584E-2</v>
+      </c>
+      <c r="I18" s="46">
+        <v>-2.6496306700358296E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>370</v>
+      </c>
+      <c r="D20" s="46">
         <f xml:space="preserve"> 1 - D6/D7</f>
         <v>0.32563360647816419</v>
       </c>
@@ -5500,6 +5546,7 @@
     <mergeCell ref="A4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5523,10 +5570,10 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75">
-      <c r="A4" s="69" t="s">
-        <v>373</v>
-      </c>
-      <c r="B4" s="69"/>
+      <c r="A4" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="B4" s="70"/>
       <c r="C4" s="33"/>
       <c r="D4" s="33"/>
     </row>
@@ -5603,10 +5650,10 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75">
-      <c r="A9" s="69" t="s">
-        <v>374</v>
-      </c>
-      <c r="B9" s="69"/>
+      <c r="A9" s="70" t="s">
+        <v>373</v>
+      </c>
+      <c r="B9" s="70"/>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
     </row>
@@ -5701,10 +5748,10 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75">
-      <c r="A15" s="69" t="s">
-        <v>375</v>
-      </c>
-      <c r="B15" s="69"/>
+      <c r="A15" s="70" t="s">
+        <v>374</v>
+      </c>
+      <c r="B15" s="70"/>
       <c r="C15" s="33"/>
       <c r="D15" s="33"/>
     </row>
@@ -5763,10 +5810,10 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75">
-      <c r="A19" s="69" t="s">
-        <v>376</v>
-      </c>
-      <c r="B19" s="69"/>
+      <c r="A19" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="B19" s="70"/>
       <c r="C19" s="33"/>
       <c r="D19" s="33"/>
     </row>
@@ -5825,10 +5872,10 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="15.75">
-      <c r="A23" s="69" t="s">
-        <v>377</v>
-      </c>
-      <c r="B23" s="69"/>
+      <c r="A23" s="70" t="s">
+        <v>376</v>
+      </c>
+      <c r="B23" s="70"/>
       <c r="C23" s="33"/>
       <c r="D23" s="33"/>
     </row>
@@ -5887,10 +5934,10 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75">
-      <c r="A27" s="69" t="s">
-        <v>378</v>
-      </c>
-      <c r="B27" s="69"/>
+      <c r="A27" s="70" t="s">
+        <v>377</v>
+      </c>
+      <c r="B27" s="70"/>
       <c r="C27" s="33"/>
       <c r="D27" s="33"/>
     </row>
@@ -5967,10 +6014,10 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75">
-      <c r="A32" s="69" t="s">
-        <v>379</v>
-      </c>
-      <c r="B32" s="69"/>
+      <c r="A32" s="70" t="s">
+        <v>378</v>
+      </c>
+      <c r="B32" s="70"/>
       <c r="C32" s="33"/>
       <c r="D32" s="33"/>
     </row>
@@ -5993,16 +6040,16 @@
       </c>
     </row>
     <row r="34" spans="1:4" ht="15.75">
-      <c r="A34" s="69" t="s">
-        <v>380</v>
-      </c>
-      <c r="B34" s="69"/>
+      <c r="A34" s="70" t="s">
+        <v>379</v>
+      </c>
+      <c r="B34" s="70"/>
       <c r="C34" s="33"/>
       <c r="D34" s="33"/>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B35" t="s">
         <v>165</v>
@@ -6017,7 +6064,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B36" s="59" t="str">
         <f>IF(C35=0,"OK","ERROR")</f>
@@ -6025,10 +6072,10 @@
       </c>
     </row>
     <row r="37" spans="1:4" ht="15.75">
-      <c r="A37" s="69" t="s">
-        <v>383</v>
-      </c>
-      <c r="B37" s="69"/>
+      <c r="A37" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B37" s="70"/>
       <c r="C37" s="29"/>
       <c r="D37" s="29"/>
     </row>
@@ -6146,7 +6193,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D6" t="s">
         <v>131</v>
@@ -6154,13 +6201,13 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
+        <v>344</v>
+      </c>
+      <c r="B7" s="63">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
         <v>345</v>
-      </c>
-      <c r="B7" s="63">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>346</v>
       </c>
       <c r="D7" t="s">
         <v>131</v>
@@ -6303,9 +6350,8 @@
       <c r="C15" t="s">
         <v>22</v>
       </c>
-      <c r="D15">
-        <f>D13 / (Inputs!B39 * 2)</f>
-        <v>0</v>
+      <c r="D15" t="s">
+        <v>93</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>91</v>
@@ -7487,7 +7533,7 @@
         <v>75</v>
       </c>
       <c r="K19" s="57" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="L19">
         <f>_xlfn.PERCENTILE.INC($C$5:$C$73,0.1)*$L$10</f>
@@ -11830,11 +11876,11 @@
       </c>
     </row>
     <row r="5" spans="1:75" ht="15.75">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="70" t="s">
         <v>169</v>
       </c>
-      <c r="B5" s="69"/>
-      <c r="C5" s="69"/>
+      <c r="B5" s="70"/>
+      <c r="C5" s="70"/>
       <c r="D5" s="43"/>
       <c r="E5" s="43"/>
       <c r="F5" s="43"/>
@@ -11916,12 +11962,12 @@
       </c>
     </row>
     <row r="14" spans="1:75" ht="15.75">
-      <c r="A14" s="69" t="s">
+      <c r="A14" s="70" t="s">
         <v>170</v>
       </c>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69"/>
-      <c r="D14" s="69"/>
+      <c r="B14" s="70"/>
+      <c r="C14" s="70"/>
+      <c r="D14" s="70"/>
       <c r="E14" s="33"/>
       <c r="F14" s="33"/>
       <c r="G14" s="33"/>
@@ -15199,12 +15245,12 @@
       </c>
     </row>
     <row r="27" spans="1:73" ht="15.75">
-      <c r="A27" s="69" t="s">
+      <c r="A27" s="70" t="s">
         <v>171</v>
       </c>
-      <c r="B27" s="69"/>
-      <c r="C27" s="69"/>
-      <c r="D27" s="69"/>
+      <c r="B27" s="70"/>
+      <c r="C27" s="70"/>
+      <c r="D27" s="70"/>
       <c r="E27" s="41"/>
       <c r="F27" s="41"/>
       <c r="G27" s="41"/>
@@ -15318,11 +15364,11 @@
       </c>
     </row>
     <row r="4" spans="1:74" ht="15.75">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="70" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:74">
       <c r="A5" t="s">
@@ -16211,11 +16257,11 @@
       <c r="BV8" s="8"/>
     </row>
     <row r="9" spans="1:74" ht="15.75">
-      <c r="A9" s="69" t="s">
+      <c r="A9" s="70" t="s">
         <v>193</v>
       </c>
-      <c r="B9" s="69"/>
-      <c r="C9" s="69"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="70"/>
     </row>
     <row r="10" spans="1:74">
       <c r="A10" t="s">
@@ -18272,12 +18318,12 @@
       </c>
     </row>
     <row r="19" spans="1:73" ht="15.75">
-      <c r="A19" s="69" t="s">
+      <c r="A19" s="70" t="s">
         <v>194</v>
       </c>
-      <c r="B19" s="69"/>
-      <c r="C19" s="69"/>
-      <c r="D19" s="69"/>
+      <c r="B19" s="70"/>
+      <c r="C19" s="70"/>
+      <c r="D19" s="70"/>
     </row>
     <row r="20" spans="1:73">
       <c r="A20" s="59" t="s">
@@ -18310,15 +18356,15 @@
       </c>
     </row>
     <row r="24" spans="1:73" ht="15.75">
-      <c r="A24" s="69" t="s">
+      <c r="A24" s="70" t="s">
         <v>205</v>
       </c>
-      <c r="B24" s="69"/>
-      <c r="C24" s="69"/>
+      <c r="B24" s="70"/>
+      <c r="C24" s="70"/>
     </row>
     <row r="25" spans="1:73">
       <c r="A25" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B25" t="s">
         <v>184</v>
@@ -20099,11 +20145,11 @@
       </c>
     </row>
     <row r="34" spans="1:73" ht="15.75">
-      <c r="A34" s="69" t="s">
+      <c r="A34" s="70" t="s">
         <v>206</v>
       </c>
-      <c r="B34" s="69"/>
-      <c r="C34" s="69"/>
+      <c r="B34" s="70"/>
+      <c r="C34" s="70"/>
     </row>
     <row r="35" spans="1:73">
       <c r="A35" s="59" t="s">
@@ -20136,11 +20182,11 @@
       </c>
     </row>
     <row r="37" spans="1:73" ht="15.75">
-      <c r="A37" s="69" t="s">
+      <c r="A37" s="70" t="s">
         <v>207</v>
       </c>
-      <c r="B37" s="69"/>
-      <c r="C37" s="69"/>
+      <c r="B37" s="70"/>
+      <c r="C37" s="70"/>
     </row>
     <row r="38" spans="1:73">
       <c r="A38" t="s">
@@ -21600,7 +21646,7 @@
     </row>
     <row r="43" spans="1:73">
       <c r="A43" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B43" t="s">
         <v>184</v>
@@ -22183,11 +22229,11 @@
       </c>
     </row>
     <row r="45" spans="1:73" ht="15.75">
-      <c r="A45" s="69" t="s">
+      <c r="A45" s="70" t="s">
         <v>215</v>
       </c>
-      <c r="B45" s="69"/>
-      <c r="C45" s="69"/>
+      <c r="B45" s="70"/>
+      <c r="C45" s="70"/>
     </row>
     <row r="46" spans="1:73">
       <c r="A46" t="s">
@@ -22286,11 +22332,11 @@
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.75">
-      <c r="A54" s="69" t="s">
+      <c r="A54" s="70" t="s">
         <v>216</v>
       </c>
-      <c r="B54" s="69"/>
-      <c r="C54" s="69"/>
+      <c r="B54" s="70"/>
+      <c r="C54" s="70"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
@@ -22353,11 +22399,11 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="15.75">
-      <c r="A61" s="69" t="s">
+      <c r="A61" s="70" t="s">
         <v>222</v>
       </c>
-      <c r="B61" s="69"/>
-      <c r="C61" s="69"/>
+      <c r="B61" s="70"/>
+      <c r="C61" s="70"/>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="59" t="s">
@@ -22482,11 +22528,11 @@
       </c>
     </row>
     <row r="4" spans="1:75" ht="15.75">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="70" t="s">
         <v>240</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:75">
       <c r="A5" t="s">
@@ -25312,11 +25358,11 @@
       </c>
     </row>
     <row r="18" spans="1:73" ht="15.75">
-      <c r="A18" s="69" t="s">
+      <c r="A18" s="70" t="s">
         <v>239</v>
       </c>
-      <c r="B18" s="69"/>
-      <c r="C18" s="69"/>
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
     </row>
     <row r="19" spans="1:73">
       <c r="A19" s="59" t="s">
@@ -25349,11 +25395,11 @@
       </c>
     </row>
     <row r="21" spans="1:73" ht="15.75">
-      <c r="A21" s="69" t="s">
+      <c r="A21" s="70" t="s">
         <v>245</v>
       </c>
-      <c r="B21" s="69"/>
-      <c r="C21" s="69"/>
+      <c r="B21" s="70"/>
+      <c r="C21" s="70"/>
     </row>
     <row r="22" spans="1:73">
       <c r="A22" t="str">
@@ -27401,11 +27447,11 @@
       </c>
     </row>
     <row r="29" spans="1:73" ht="15.75">
-      <c r="A29" s="69" t="s">
+      <c r="A29" s="70" t="s">
         <v>206</v>
       </c>
-      <c r="B29" s="69"/>
-      <c r="C29" s="69"/>
+      <c r="B29" s="70"/>
+      <c r="C29" s="70"/>
     </row>
     <row r="30" spans="1:73">
       <c r="A30" s="59" t="s">
@@ -27457,11 +27503,11 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="70" t="s">
         <v>255</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
@@ -29560,11 +29606,11 @@
       </c>
     </row>
     <row r="16" spans="1:73" ht="15.75">
-      <c r="A16" s="69" t="s">
+      <c r="A16" s="70" t="s">
         <v>239</v>
       </c>
-      <c r="B16" s="69"/>
-      <c r="C16" s="69"/>
+      <c r="B16" s="70"/>
+      <c r="C16" s="70"/>
     </row>
     <row r="17" spans="1:73" ht="30">
       <c r="A17" s="61" t="s">
@@ -29582,11 +29628,11 @@
       </c>
     </row>
     <row r="18" spans="1:73" ht="15.75">
-      <c r="A18" s="69" t="s">
+      <c r="A18" s="70" t="s">
         <v>257</v>
       </c>
-      <c r="B18" s="69"/>
-      <c r="C18" s="69"/>
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
     </row>
     <row r="19" spans="1:73">
       <c r="A19" t="s">
@@ -29882,7 +29928,7 @@
     </row>
     <row r="20" spans="1:73">
       <c r="A20" t="s">
-        <v>272</v>
+        <v>384</v>
       </c>
       <c r="B20" s="27" t="s">
         <v>184</v>
@@ -33657,11 +33703,11 @@
       </c>
     </row>
     <row r="34" spans="1:73" ht="15.75">
-      <c r="A34" s="69" t="s">
+      <c r="A34" s="70" t="s">
         <v>206</v>
       </c>
-      <c r="B34" s="69"/>
-      <c r="C34" s="69"/>
+      <c r="B34" s="70"/>
+      <c r="C34" s="70"/>
     </row>
     <row r="35" spans="1:73">
       <c r="A35" s="59" t="s">
@@ -33730,21 +33776,21 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="69" t="s">
-        <v>285</v>
-      </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="A4" s="70" t="s">
+        <v>284</v>
+      </c>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:73">
@@ -34631,7 +34677,7 @@
     </row>
     <row r="9" spans="1:73">
       <c r="A9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B9" t="s">
         <v>173</v>
@@ -34922,7 +34968,7 @@
     </row>
     <row r="10" spans="1:73">
       <c r="A10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B10" t="s">
         <v>184</v>
@@ -35214,7 +35260,7 @@
     </row>
     <row r="11" spans="1:73">
       <c r="A11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
@@ -35502,7 +35548,7 @@
     </row>
     <row r="12" spans="1:73">
       <c r="A12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B12" t="s">
         <v>184</v>
@@ -35794,7 +35840,7 @@
     </row>
     <row r="13" spans="1:73">
       <c r="A13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B13" t="s">
         <v>184</v>
@@ -35806,7 +35852,7 @@
     </row>
     <row r="14" spans="1:73">
       <c r="A14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B14" t="s">
         <v>184</v>
@@ -35818,7 +35864,7 @@
     </row>
     <row r="15" spans="1:73">
       <c r="A15" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B15" t="s">
         <v>184</v>
@@ -35830,7 +35876,7 @@
     </row>
     <row r="16" spans="1:73">
       <c r="A16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B16" t="s">
         <v>131</v>
@@ -35842,7 +35888,7 @@
     </row>
     <row r="17" spans="1:73">
       <c r="A17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B17" t="s">
         <v>39</v>
@@ -35854,7 +35900,7 @@
     </row>
     <row r="18" spans="1:73">
       <c r="A18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B18" t="s">
         <v>184</v>
@@ -36145,15 +36191,15 @@
       </c>
     </row>
     <row r="19" spans="1:73" ht="15.75">
-      <c r="A19" s="69" t="s">
-        <v>286</v>
-      </c>
-      <c r="B19" s="69"/>
-      <c r="C19" s="69"/>
+      <c r="A19" s="70" t="s">
+        <v>285</v>
+      </c>
+      <c r="B19" s="70"/>
+      <c r="C19" s="70"/>
     </row>
     <row r="20" spans="1:73">
       <c r="A20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B20" t="s">
         <v>184</v>
@@ -36164,7 +36210,7 @@
     </row>
     <row r="21" spans="1:73">
       <c r="A21" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B21" t="s">
         <v>39</v>
@@ -36175,7 +36221,7 @@
     </row>
     <row r="22" spans="1:73">
       <c r="A22" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="23" spans="1:73">
@@ -36467,7 +36513,7 @@
     </row>
     <row r="24" spans="1:73">
       <c r="A24" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B24" t="s">
         <v>184</v>
@@ -36759,7 +36805,7 @@
     </row>
     <row r="25" spans="1:73">
       <c r="A25" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B25" t="s">
         <v>184</v>
@@ -37051,7 +37097,7 @@
     </row>
     <row r="26" spans="1:73">
       <c r="A26" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B26" t="s">
         <v>184</v>
@@ -37631,7 +37677,7 @@
     </row>
     <row r="28" spans="1:73">
       <c r="A28" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C28">
         <v>12963649.757217973</v>
@@ -37848,15 +37894,15 @@
       </c>
     </row>
     <row r="29" spans="1:73" ht="15.75">
-      <c r="A29" s="69" t="s">
+      <c r="A29" s="70" t="s">
         <v>206</v>
       </c>
-      <c r="B29" s="69"/>
-      <c r="C29" s="69"/>
+      <c r="B29" s="70"/>
+      <c r="C29" s="70"/>
     </row>
     <row r="30" spans="1:73">
       <c r="A30" s="59" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B30" s="59" t="s">
         <v>165</v>
@@ -37871,7 +37917,7 @@
     </row>
     <row r="31" spans="1:73">
       <c r="A31" s="59" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B31" s="59" t="s">
         <v>165</v>
@@ -37886,7 +37932,7 @@
     </row>
     <row r="32" spans="1:73">
       <c r="A32" s="59" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B32" s="59" t="s">
         <v>165</v>
@@ -37931,21 +37977,21 @@
       </c>
     </row>
     <row r="4" spans="1:73" ht="15.75">
-      <c r="A4" s="69" t="s">
-        <v>310</v>
-      </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="A4" s="70" t="s">
+        <v>309</v>
+      </c>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:73">
       <c r="A5" t="s">
         <v>145</v>
       </c>
       <c r="B5" t="s">
+        <v>296</v>
+      </c>
+      <c r="C5" t="s">
         <v>297</v>
-      </c>
-      <c r="C5" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="6" spans="1:73">
@@ -39126,7 +39172,7 @@
     </row>
     <row r="10" spans="1:73">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B10" t="s">
         <v>184</v>
@@ -39414,7 +39460,7 @@
     </row>
     <row r="11" spans="1:73">
       <c r="A11" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B11" t="s">
         <v>174</v>
@@ -39702,7 +39748,7 @@
     </row>
     <row r="12" spans="1:73">
       <c r="A12" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B12" t="s">
         <v>184</v>
@@ -39990,7 +40036,7 @@
     </row>
     <row r="13" spans="1:73">
       <c r="A13" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B13" t="s">
         <v>131</v>
@@ -40285,7 +40331,7 @@
     </row>
     <row r="15" spans="1:73">
       <c r="A15" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B15" t="s">
         <v>184</v>
@@ -40577,7 +40623,7 @@
     </row>
     <row r="16" spans="1:73">
       <c r="A16" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B16" t="s">
         <v>184</v>
@@ -40869,7 +40915,7 @@
     </row>
     <row r="17" spans="1:73">
       <c r="A17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B17" t="s">
         <v>184</v>
@@ -41161,7 +41207,7 @@
     </row>
     <row r="18" spans="1:73">
       <c r="A18" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B18" t="s">
         <v>184</v>
@@ -41740,15 +41786,15 @@
       </c>
     </row>
     <row r="20" spans="1:73" ht="15.75">
-      <c r="A20" s="69" t="s">
+      <c r="A20" s="70" t="s">
         <v>239</v>
       </c>
-      <c r="B20" s="69"/>
-      <c r="C20" s="69"/>
+      <c r="B20" s="70"/>
+      <c r="C20" s="70"/>
     </row>
     <row r="21" spans="1:73">
       <c r="A21" s="59" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B21" s="59" t="s">
         <v>165</v>
@@ -41760,7 +41806,7 @@
     </row>
     <row r="22" spans="1:73">
       <c r="A22" s="59" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B22" s="59" t="s">
         <v>165</v>
@@ -41771,15 +41817,15 @@
       </c>
     </row>
     <row r="23" spans="1:73" ht="15.75">
-      <c r="A23" s="69" t="s">
-        <v>311</v>
-      </c>
-      <c r="B23" s="69"/>
-      <c r="C23" s="69"/>
+      <c r="A23" s="70" t="s">
+        <v>310</v>
+      </c>
+      <c r="B23" s="70"/>
+      <c r="C23" s="70"/>
     </row>
     <row r="24" spans="1:73">
       <c r="A24" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B24" t="s">
         <v>184</v>
@@ -42067,7 +42113,7 @@
     </row>
     <row r="25" spans="1:73">
       <c r="A25" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B25" t="s">
         <v>39</v>
@@ -42355,7 +42401,7 @@
     </row>
     <row r="26" spans="1:73">
       <c r="A26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B26" t="s">
         <v>174</v>
@@ -42643,7 +42689,7 @@
     </row>
     <row r="27" spans="1:73" ht="15.75">
       <c r="A27" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B27" t="s">
         <v>174</v>
@@ -42932,7 +42978,7 @@
     </row>
     <row r="28" spans="1:73">
       <c r="A28" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B28" t="s">
         <v>131</v>
@@ -42940,7 +42986,7 @@
     </row>
     <row r="29" spans="1:73">
       <c r="A29" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B29" t="s">
         <v>184</v>
@@ -43227,7 +43273,7 @@
     </row>
     <row r="30" spans="1:73">
       <c r="A30" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B30" t="s">
         <v>184</v>
@@ -43515,7 +43561,7 @@
     </row>
     <row r="31" spans="1:73">
       <c r="A31" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B31" t="s">
         <v>184</v>
@@ -43807,7 +43853,7 @@
     </row>
     <row r="32" spans="1:73">
       <c r="A32" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B32" t="s">
         <v>184</v>
@@ -44094,15 +44140,15 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75">
-      <c r="A33" s="69" t="s">
+      <c r="A33" s="70" t="s">
         <v>206</v>
       </c>
-      <c r="B33" s="69"/>
-      <c r="C33" s="69"/>
+      <c r="B33" s="70"/>
+      <c r="C33" s="70"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="59" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B34" s="59" t="s">
         <v>165</v>
@@ -44117,7 +44163,7 @@
     </row>
     <row r="35" spans="1:4" ht="30">
       <c r="A35" s="61" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B35" s="62" t="s">
         <v>165</v>
@@ -44132,32 +44178,32 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="59" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B36" s="59" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C36" s="59">
         <f>SUM(D26:BU26)</f>
         <v>0</v>
       </c>
       <c r="D36" s="37" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="59" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B37" s="59" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C37" s="59">
         <f>SUM(D27:BU27)</f>
         <v>0</v>
       </c>
       <c r="D37" s="37" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>